<commit_message>
📊 Steam 차트 업데이트: 2026-04-27
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="일별 스냅샷" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="오늘의 차트" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="롱런 게임 분석" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2주+ 롱런 분석" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="4주+ 롱런 분석" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -457,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -465,13 +466,12 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,35 +502,30 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>2주 플레이어</t>
+          <t>긍정리뷰(%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>긍정리뷰(%)</t>
+          <t>총 리뷰수</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>총 리뷰수</t>
+          <t>긍정리뷰수</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>긍정리뷰수</t>
+          <t>가격(₩)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>가격(₩)</t>
+          <t>할인율(%)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>할인율(%)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>정가(₩)</t>
         </is>
@@ -557,24 +552,21 @@
         <v>1013936</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>86.7</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>86.7</v>
+        <v>8815087</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>8815087</v>
+        <v>7642084</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>7642084</v>
+        <v/>
       </c>
       <c r="J2" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -599,24 +591,21 @@
         <v>124262</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>67.09999999999999</v>
+        <v>994979</v>
       </c>
       <c r="H3" t="n">
-        <v>994979</v>
+        <v>668053</v>
       </c>
       <c r="I3" t="n">
-        <v>668053</v>
+        <v/>
       </c>
       <c r="J3" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
         <v/>
       </c>
     </row>
@@ -641,24 +630,21 @@
         <v>314682</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>59.4</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>59.4</v>
+        <v>2557944</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2557944</v>
+        <v>1520457</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>1520457</v>
+        <v/>
       </c>
       <c r="J4" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -683,24 +669,21 @@
         <v>18028</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>94.09999999999999</v>
+        <v>380709</v>
       </c>
       <c r="H5" t="n">
-        <v>380709</v>
+        <v>358266</v>
       </c>
       <c r="I5" t="n">
-        <v>358266</v>
+        <v>32000</v>
       </c>
       <c r="J5" t="n">
-        <v>32000</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
         <v>32000</v>
       </c>
     </row>
@@ -725,24 +708,21 @@
         <v>43819</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>89.90000000000001</v>
+        <v>1161472</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1161472</v>
+        <v>1044264</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1044264</v>
+        <v/>
       </c>
       <c r="J6" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -767,24 +747,21 @@
         <v>67419</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>58.8</v>
       </c>
       <c r="G7" t="n">
-        <v>58.8</v>
+        <v>714114</v>
       </c>
       <c r="H7" t="n">
-        <v>714114</v>
+        <v>419594</v>
       </c>
       <c r="I7" t="n">
-        <v>419594</v>
+        <v/>
       </c>
       <c r="J7" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
         <v/>
       </c>
     </row>
@@ -809,24 +786,21 @@
         <v>5583</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>68.59999999999999</v>
+        <v>286878</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>286878</v>
+        <v>196798</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>196798</v>
+        <v/>
       </c>
       <c r="J8" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -851,24 +825,21 @@
         <v>15004</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="G9" t="n">
-        <v>96.7</v>
+        <v>1150098</v>
       </c>
       <c r="H9" t="n">
-        <v>1150098</v>
+        <v>1111720</v>
       </c>
       <c r="I9" t="n">
-        <v>1111720</v>
+        <v>64800</v>
       </c>
       <c r="J9" t="n">
-        <v>64800</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
         <v>64800</v>
       </c>
     </row>
@@ -893,24 +864,21 @@
         <v>67851</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>87.40000000000001</v>
+        <v>1990556</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1990556</v>
+        <v>1739980</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>1739980</v>
+        <v/>
       </c>
       <c r="J10" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -935,24 +903,21 @@
         <v>25122</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="G11" t="n">
-        <v>97.5</v>
+        <v>963983</v>
       </c>
       <c r="H11" t="n">
-        <v>963983</v>
+        <v>940221</v>
       </c>
       <c r="I11" t="n">
-        <v>940221</v>
+        <v>11000</v>
       </c>
       <c r="J11" t="n">
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
         <v>11000</v>
       </c>
     </row>
@@ -977,24 +942,21 @@
         <v>10408</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>91.2</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>91.2</v>
+        <v>555368</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>555368</v>
+        <v>506516</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>506516</v>
+        <v/>
       </c>
       <c r="J12" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -1019,24 +981,21 @@
         <v>17355</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="G13" t="n">
-        <v>71</v>
+        <v>202021</v>
       </c>
       <c r="H13" t="n">
-        <v>202021</v>
+        <v>143481</v>
       </c>
       <c r="I13" t="n">
-        <v>143481</v>
+        <v/>
       </c>
       <c r="J13" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
         <v/>
       </c>
     </row>
@@ -1061,24 +1020,21 @@
         <v>50478</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>64</v>
+        <v>757086</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>757086</v>
+        <v>484469</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>484469</v>
+        <v/>
       </c>
       <c r="J14" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -1103,24 +1059,21 @@
         <v>12494</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>58.3</v>
       </c>
       <c r="G15" t="n">
-        <v>58.3</v>
+        <v>218415</v>
       </c>
       <c r="H15" t="n">
-        <v>218415</v>
+        <v>127273</v>
       </c>
       <c r="I15" t="n">
-        <v>127273</v>
+        <v>84800</v>
       </c>
       <c r="J15" t="n">
-        <v>84800</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
         <v>84800</v>
       </c>
     </row>
@@ -1145,24 +1098,21 @@
         <v>53399</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>76.2</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>76.2</v>
+        <v>1017635</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>1017635</v>
+        <v>775883</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>775883</v>
+        <v>44800</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>44800</v>
+        <v>0</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="2" t="n">
         <v>44800</v>
       </c>
     </row>
@@ -1187,24 +1137,21 @@
         <v>36195</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>87.09999999999999</v>
+        <v>626503</v>
       </c>
       <c r="H17" t="n">
-        <v>626503</v>
+        <v>545393</v>
       </c>
       <c r="I17" t="n">
-        <v>545393</v>
+        <v/>
       </c>
       <c r="J17" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
         <v/>
       </c>
     </row>
@@ -1229,24 +1176,21 @@
         <v>29529</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>92.90000000000001</v>
+        <v>1056677</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>1056677</v>
+        <v>981540</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>981540</v>
+        <v>64800</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>64800</v>
+        <v>0</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="2" t="n">
         <v>64800</v>
       </c>
     </row>
@@ -1271,24 +1215,21 @@
         <v>24580</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="G19" t="n">
-        <v>97.5</v>
+        <v>1409473</v>
       </c>
       <c r="H19" t="n">
-        <v>1409473</v>
+        <v>1373979</v>
       </c>
       <c r="I19" t="n">
-        <v>1373979</v>
+        <v>11000</v>
       </c>
       <c r="J19" t="n">
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
         <v>11000</v>
       </c>
     </row>
@@ -1313,24 +1254,21 @@
         <v>16727</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>70.09999999999999</v>
+        <v>169021</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>169021</v>
+        <v>118511</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>118511</v>
+        <v/>
       </c>
       <c r="J20" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -1355,24 +1293,21 @@
         <v>91184</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="G21" t="n">
-        <v>98</v>
+        <v>894458</v>
       </c>
       <c r="H21" t="n">
-        <v>894458</v>
+        <v>876898</v>
       </c>
       <c r="I21" t="n">
-        <v>876898</v>
+        <v>5600</v>
       </c>
       <c r="J21" t="n">
-        <v>5600</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
         <v>5600</v>
       </c>
     </row>
@@ -1397,24 +1332,21 @@
         <v>54771</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>96.8</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>96.8</v>
+        <v>760662</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>760662</v>
+        <v>736688</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>736688</v>
+        <v>66000</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>66000</v>
+        <v>0</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="2" t="n">
         <v>66000</v>
       </c>
     </row>
@@ -1439,24 +1371,21 @@
         <v>14169</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>81.5</v>
       </c>
       <c r="G23" t="n">
-        <v>81.5</v>
+        <v>386456</v>
       </c>
       <c r="H23" t="n">
-        <v>386456</v>
+        <v>314809</v>
       </c>
       <c r="I23" t="n">
-        <v>314809</v>
+        <v/>
       </c>
       <c r="J23" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="n">
         <v/>
       </c>
     </row>
@@ -1481,24 +1410,21 @@
         <v>18400</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0</v>
+        <v>96.8</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>96.8</v>
+        <v>1159707</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>1159707</v>
+        <v>1122546</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1122546</v>
+        <v>5250</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>5250</v>
+        <v>50</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="L24" s="2" t="n">
         <v>10500</v>
       </c>
     </row>
@@ -1523,24 +1449,21 @@
         <v>24619</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="G25" t="n">
-        <v>79.59999999999999</v>
+        <v>625616</v>
       </c>
       <c r="H25" t="n">
-        <v>625616</v>
+        <v>497891</v>
       </c>
       <c r="I25" t="n">
-        <v>497891</v>
+        <v/>
       </c>
       <c r="J25" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
         <v/>
       </c>
     </row>
@@ -1565,24 +1488,21 @@
         <v>51847</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>83.90000000000001</v>
+        <v>1398584</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>1398584</v>
+        <v>1172854</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>1172854</v>
+        <v/>
       </c>
       <c r="J26" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -1607,24 +1527,21 @@
         <v>143870</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>87.2</v>
       </c>
       <c r="G27" t="n">
-        <v>87.2</v>
+        <v>1227784</v>
       </c>
       <c r="H27" t="n">
-        <v>1227784</v>
+        <v>1071135</v>
       </c>
       <c r="I27" t="n">
-        <v>1071135</v>
+        <v>42000</v>
       </c>
       <c r="J27" t="n">
-        <v>42000</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="n">
         <v>42000</v>
       </c>
     </row>
@@ -1649,24 +1566,21 @@
         <v>8518</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>77</v>
+        <v>146552</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>146552</v>
+        <v>112887</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>112887</v>
+        <v/>
       </c>
       <c r="J28" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -1691,24 +1605,21 @@
         <v>22170</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>83.8</v>
       </c>
       <c r="G29" t="n">
-        <v>83.8</v>
+        <v>730170</v>
       </c>
       <c r="H29" t="n">
-        <v>730170</v>
+        <v>612177</v>
       </c>
       <c r="I29" t="n">
-        <v>612177</v>
+        <v>16500</v>
       </c>
       <c r="J29" t="n">
-        <v>16500</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" t="n">
         <v>16500</v>
       </c>
     </row>
@@ -1733,24 +1644,21 @@
         <v>50662</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>98.40000000000001</v>
+        <v>886195</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>886195</v>
+        <v>872384</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>872384</v>
+        <v>16000</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>16000</v>
+        <v>0</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" s="2" t="n">
         <v>16000</v>
       </c>
     </row>
@@ -1775,24 +1683,21 @@
         <v>2892</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>95.5</v>
       </c>
       <c r="G31" t="n">
-        <v>95.5</v>
+        <v>627791</v>
       </c>
       <c r="H31" t="n">
-        <v>627791</v>
+        <v>599805</v>
       </c>
       <c r="I31" t="n">
-        <v>599805</v>
+        <v>20500</v>
       </c>
       <c r="J31" t="n">
-        <v>20500</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="n">
         <v>20500</v>
       </c>
     </row>
@@ -1817,24 +1722,21 @@
         <v>256</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>64.09999999999999</v>
+        <v>3082</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>3082</v>
+        <v>1977</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>1977</v>
+        <v/>
       </c>
       <c r="J32" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -1859,24 +1761,21 @@
         <v>4694</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>89.3</v>
       </c>
       <c r="G33" t="n">
-        <v>89.3</v>
+        <v>235091</v>
       </c>
       <c r="H33" t="n">
-        <v>235091</v>
+        <v>209822</v>
       </c>
       <c r="I33" t="n">
-        <v>209822</v>
+        <v/>
       </c>
       <c r="J33" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" t="n">
         <v/>
       </c>
     </row>
@@ -1901,24 +1800,21 @@
         <v>27254</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>89.59999999999999</v>
+        <v>663082</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>663082</v>
+        <v>594327</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>594327</v>
+        <v>10700</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>10700</v>
+        <v>0</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" s="2" t="n">
         <v>10700</v>
       </c>
     </row>
@@ -1943,24 +1839,21 @@
         <v>270</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="G35" t="n">
-        <v>66.40000000000001</v>
+        <v>82197</v>
       </c>
       <c r="H35" t="n">
-        <v>82197</v>
+        <v>54554</v>
       </c>
       <c r="I35" t="n">
-        <v>54554</v>
+        <v/>
       </c>
       <c r="J35" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" t="n">
         <v/>
       </c>
     </row>
@@ -1985,24 +1878,21 @@
         <v>0</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0</v>
+        <v>82.5</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>82.5</v>
+        <v>175272</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>175272</v>
+        <v>144570</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>144570</v>
+        <v/>
       </c>
       <c r="J36" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -2027,24 +1917,21 @@
         <v>5831</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="G37" t="n">
-        <v>79.59999999999999</v>
+        <v>110623</v>
       </c>
       <c r="H37" t="n">
-        <v>110623</v>
+        <v>88027</v>
       </c>
       <c r="I37" t="n">
-        <v>88027</v>
+        <v>37500</v>
       </c>
       <c r="J37" t="n">
-        <v>37500</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" t="n">
         <v>37500</v>
       </c>
     </row>
@@ -2069,24 +1956,21 @@
         <v>2</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0</v>
+        <v>89.3</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>89.3</v>
+        <v>13686</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>13686</v>
+        <v>12215</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>12215</v>
+        <v/>
       </c>
       <c r="J38" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L38" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -2111,24 +1995,21 @@
         <v>22265</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>84.40000000000001</v>
+        <v>844921</v>
       </c>
       <c r="H39" t="n">
-        <v>844921</v>
+        <v>713071</v>
       </c>
       <c r="I39" t="n">
-        <v>713071</v>
+        <v>23100</v>
       </c>
       <c r="J39" t="n">
-        <v>23100</v>
+        <v>65</v>
       </c>
       <c r="K39" t="n">
-        <v>65</v>
-      </c>
-      <c r="L39" t="n">
         <v>66000</v>
       </c>
     </row>
@@ -2153,24 +2034,21 @@
         <v>44886</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>79.09999999999999</v>
+        <v>797216</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>797216</v>
+        <v>630223</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>630223</v>
+        <v>8600</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>8600</v>
+        <v>60</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="L40" s="2" t="n">
         <v>21500</v>
       </c>
     </row>
@@ -2195,24 +2073,21 @@
         <v>5716</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>90.2</v>
       </c>
       <c r="G41" t="n">
-        <v>90.2</v>
+        <v>321395</v>
       </c>
       <c r="H41" t="n">
-        <v>321395</v>
+        <v>289966</v>
       </c>
       <c r="I41" t="n">
-        <v>289966</v>
+        <v>79800</v>
       </c>
       <c r="J41" t="n">
-        <v>79800</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
-      </c>
-      <c r="L41" t="n">
         <v>79800</v>
       </c>
     </row>
@@ -2237,24 +2112,21 @@
         <v>34699</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>75.59999999999999</v>
+        <v>240355</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>240355</v>
+        <v>181623</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>181623</v>
+        <v/>
       </c>
       <c r="J42" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L42" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -2279,24 +2151,21 @@
         <v>15893</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="G43" t="n">
-        <v>96.09999999999999</v>
+        <v>835349</v>
       </c>
       <c r="H43" t="n">
-        <v>835349</v>
+        <v>802993</v>
       </c>
       <c r="I43" t="n">
-        <v>802993</v>
+        <v>6960</v>
       </c>
       <c r="J43" t="n">
-        <v>6960</v>
+        <v>80</v>
       </c>
       <c r="K43" t="n">
-        <v>80</v>
-      </c>
-      <c r="L43" t="n">
         <v>34800</v>
       </c>
     </row>
@@ -2321,24 +2190,21 @@
         <v>3832</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>700785</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>700785</v>
+        <v>643681</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>643681</v>
+        <v>5500</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>5500</v>
+        <v>0</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" s="2" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -2363,24 +2229,21 @@
         <v>664</v>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>81.3</v>
       </c>
       <c r="G45" t="n">
-        <v>81.3</v>
+        <v>473743</v>
       </c>
       <c r="H45" t="n">
-        <v>473743</v>
+        <v>385154</v>
       </c>
       <c r="I45" t="n">
-        <v>385154</v>
+        <v/>
       </c>
       <c r="J45" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" t="n">
         <v/>
       </c>
     </row>
@@ -2405,24 +2268,21 @@
         <v>8551</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>92.40000000000001</v>
+        <v>295218</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>295218</v>
+        <v>272900</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>272900</v>
+        <v>9460</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>9460</v>
+        <v>78</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="L46" s="2" t="n">
         <v>43000</v>
       </c>
     </row>
@@ -2447,24 +2307,21 @@
         <v>17281</v>
       </c>
       <c r="F47" t="n">
-        <v>0</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="G47" t="n">
-        <v>97.40000000000001</v>
+        <v>867404</v>
       </c>
       <c r="H47" t="n">
-        <v>867404</v>
+        <v>844480</v>
       </c>
       <c r="I47" t="n">
-        <v>844480</v>
+        <v>24800</v>
       </c>
       <c r="J47" t="n">
-        <v>24800</v>
+        <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
-      </c>
-      <c r="L47" t="n">
         <v>24800</v>
       </c>
     </row>
@@ -2489,24 +2346,21 @@
         <v>14439</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0</v>
+        <v>94.3</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>94.3</v>
+        <v>499828</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>499828</v>
+        <v>471451</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>471451</v>
+        <v>11000</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>11000</v>
+        <v>50</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="L48" s="2" t="n">
         <v>22000</v>
       </c>
     </row>
@@ -2531,24 +2385,21 @@
         <v>9978</v>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
+        <v>95.8</v>
       </c>
       <c r="G49" t="n">
-        <v>95.8</v>
+        <v>768779</v>
       </c>
       <c r="H49" t="n">
-        <v>768779</v>
+        <v>736611</v>
       </c>
       <c r="I49" t="n">
-        <v>736611</v>
+        <v>21500</v>
       </c>
       <c r="J49" t="n">
-        <v>21500</v>
+        <v>0</v>
       </c>
       <c r="K49" t="n">
-        <v>0</v>
-      </c>
-      <c r="L49" t="n">
         <v>21500</v>
       </c>
     </row>
@@ -2573,24 +2424,21 @@
         <v>1028</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>85</v>
+        <v>346404</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>346404</v>
+        <v>294373</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>294373</v>
+        <v/>
       </c>
       <c r="J50" s="2" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L50" s="2" t="n">
         <v/>
       </c>
     </row>
@@ -2615,24 +2463,21 @@
         <v>66954</v>
       </c>
       <c r="F51" t="n">
-        <v>0</v>
+        <v>69.5</v>
       </c>
       <c r="G51" t="n">
-        <v>69.5</v>
+        <v>324927</v>
       </c>
       <c r="H51" t="n">
-        <v>324927</v>
+        <v>225960</v>
       </c>
       <c r="I51" t="n">
-        <v>225960</v>
+        <v/>
       </c>
       <c r="J51" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" t="n">
         <v/>
       </c>
     </row>
@@ -2647,17 +2492,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2685,25 +2529,20 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>2주 플레이어</t>
+          <t>긍정리뷰(%)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>긍정리뷰(%)</t>
+          <t>총 리뷰수</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>총 리뷰수</t>
+          <t>가격(₩)</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
-        <is>
-          <t>가격(₩)</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>할인율(%)</t>
         </is>
@@ -2722,18 +2561,15 @@
         <v>1013936</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>86.7</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>86.7</v>
+        <v>8815087</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>8815087</v>
+        <v/>
       </c>
       <c r="G4" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H4" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2750,18 +2586,15 @@
         <v>124262</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>67.09999999999999</v>
+        <v>994979</v>
       </c>
       <c r="F5" t="n">
-        <v>994979</v>
+        <v/>
       </c>
       <c r="G5" t="n">
-        <v/>
-      </c>
-      <c r="H5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2778,18 +2611,15 @@
         <v>314682</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0</v>
+        <v>59.4</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>59.4</v>
+        <v>2557944</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>2557944</v>
+        <v/>
       </c>
       <c r="G6" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H6" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2806,18 +2636,15 @@
         <v>18028</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>94.09999999999999</v>
+        <v>380709</v>
       </c>
       <c r="F7" t="n">
-        <v>380709</v>
+        <v>32000</v>
       </c>
       <c r="G7" t="n">
-        <v>32000</v>
-      </c>
-      <c r="H7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2834,18 +2661,15 @@
         <v>43819</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>89.90000000000001</v>
+        <v>1161472</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>1161472</v>
+        <v/>
       </c>
       <c r="G8" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H8" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2862,18 +2686,15 @@
         <v>67419</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>58.8</v>
       </c>
       <c r="E9" t="n">
-        <v>58.8</v>
+        <v>714114</v>
       </c>
       <c r="F9" t="n">
-        <v>714114</v>
+        <v/>
       </c>
       <c r="G9" t="n">
-        <v/>
-      </c>
-      <c r="H9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2890,18 +2711,15 @@
         <v>5583</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>68.59999999999999</v>
+        <v>286878</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>286878</v>
+        <v/>
       </c>
       <c r="G10" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H10" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2918,18 +2736,15 @@
         <v>15004</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="E11" t="n">
-        <v>96.7</v>
+        <v>1150098</v>
       </c>
       <c r="F11" t="n">
-        <v>1150098</v>
+        <v>64800</v>
       </c>
       <c r="G11" t="n">
-        <v>64800</v>
-      </c>
-      <c r="H11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2946,18 +2761,15 @@
         <v>67851</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>87.40000000000001</v>
+        <v>1990556</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>1990556</v>
+        <v/>
       </c>
       <c r="G12" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H12" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2974,18 +2786,15 @@
         <v>25122</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="E13" t="n">
-        <v>97.5</v>
+        <v>963983</v>
       </c>
       <c r="F13" t="n">
-        <v>963983</v>
+        <v>11000</v>
       </c>
       <c r="G13" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3002,18 +2811,15 @@
         <v>10408</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0</v>
+        <v>91.2</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>91.2</v>
+        <v>555368</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>555368</v>
+        <v/>
       </c>
       <c r="G14" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H14" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3030,18 +2836,15 @@
         <v>17355</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>202021</v>
       </c>
       <c r="F15" t="n">
-        <v>202021</v>
+        <v/>
       </c>
       <c r="G15" t="n">
-        <v/>
-      </c>
-      <c r="H15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3058,18 +2861,15 @@
         <v>50478</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>64</v>
+        <v>757086</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>757086</v>
+        <v/>
       </c>
       <c r="G16" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H16" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3086,18 +2886,15 @@
         <v>12494</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>58.3</v>
       </c>
       <c r="E17" t="n">
-        <v>58.3</v>
+        <v>218415</v>
       </c>
       <c r="F17" t="n">
-        <v>218415</v>
+        <v>84800</v>
       </c>
       <c r="G17" t="n">
-        <v>84800</v>
-      </c>
-      <c r="H17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3114,18 +2911,15 @@
         <v>53399</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0</v>
+        <v>76.2</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>76.2</v>
+        <v>1017635</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1017635</v>
+        <v>44800</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>44800</v>
-      </c>
-      <c r="H18" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3142,18 +2936,15 @@
         <v>36195</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>87.09999999999999</v>
+        <v>626503</v>
       </c>
       <c r="F19" t="n">
-        <v>626503</v>
+        <v/>
       </c>
       <c r="G19" t="n">
-        <v/>
-      </c>
-      <c r="H19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3170,18 +2961,15 @@
         <v>29529</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>92.90000000000001</v>
+        <v>1056677</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>1056677</v>
+        <v>64800</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>64800</v>
-      </c>
-      <c r="H20" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3198,18 +2986,15 @@
         <v>24580</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>97.5</v>
       </c>
       <c r="E21" t="n">
-        <v>97.5</v>
+        <v>1409473</v>
       </c>
       <c r="F21" t="n">
-        <v>1409473</v>
+        <v>11000</v>
       </c>
       <c r="G21" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3226,18 +3011,15 @@
         <v>16727</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>70.09999999999999</v>
+        <v>169021</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>169021</v>
+        <v/>
       </c>
       <c r="G22" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H22" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3254,18 +3036,15 @@
         <v>91184</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="E23" t="n">
-        <v>98</v>
+        <v>894458</v>
       </c>
       <c r="F23" t="n">
-        <v>894458</v>
+        <v>5600</v>
       </c>
       <c r="G23" t="n">
-        <v>5600</v>
-      </c>
-      <c r="H23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3282,18 +3061,15 @@
         <v>54771</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>96.8</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>96.8</v>
+        <v>760662</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>760662</v>
+        <v>66000</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>66000</v>
-      </c>
-      <c r="H24" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3310,18 +3086,15 @@
         <v>14169</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>81.5</v>
       </c>
       <c r="E25" t="n">
-        <v>81.5</v>
+        <v>386456</v>
       </c>
       <c r="F25" t="n">
-        <v>386456</v>
+        <v/>
       </c>
       <c r="G25" t="n">
-        <v/>
-      </c>
-      <c r="H25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3338,18 +3111,15 @@
         <v>18400</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>0</v>
+        <v>96.8</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>96.8</v>
+        <v>1159707</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>1159707</v>
+        <v>5250</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>5250</v>
-      </c>
-      <c r="H26" s="4" t="n">
         <v>50</v>
       </c>
     </row>
@@ -3366,18 +3136,15 @@
         <v>24619</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="E27" t="n">
-        <v>79.59999999999999</v>
+        <v>625616</v>
       </c>
       <c r="F27" t="n">
-        <v>625616</v>
+        <v/>
       </c>
       <c r="G27" t="n">
-        <v/>
-      </c>
-      <c r="H27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3394,18 +3161,15 @@
         <v>51847</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>83.90000000000001</v>
+        <v>1398584</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>1398584</v>
+        <v/>
       </c>
       <c r="G28" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H28" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3422,18 +3186,15 @@
         <v>143870</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>87.2</v>
       </c>
       <c r="E29" t="n">
-        <v>87.2</v>
+        <v>1227784</v>
       </c>
       <c r="F29" t="n">
-        <v>1227784</v>
+        <v>42000</v>
       </c>
       <c r="G29" t="n">
-        <v>42000</v>
-      </c>
-      <c r="H29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3450,18 +3211,15 @@
         <v>8518</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>77</v>
+        <v>146552</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>146552</v>
+        <v/>
       </c>
       <c r="G30" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H30" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3478,18 +3236,15 @@
         <v>22170</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>83.8</v>
       </c>
       <c r="E31" t="n">
-        <v>83.8</v>
+        <v>730170</v>
       </c>
       <c r="F31" t="n">
-        <v>730170</v>
+        <v>16500</v>
       </c>
       <c r="G31" t="n">
-        <v>16500</v>
-      </c>
-      <c r="H31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3506,18 +3261,15 @@
         <v>50662</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>98.40000000000001</v>
+        <v>886195</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>886195</v>
+        <v>16000</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>16000</v>
-      </c>
-      <c r="H32" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3534,18 +3286,15 @@
         <v>2892</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>95.5</v>
       </c>
       <c r="E33" t="n">
-        <v>95.5</v>
+        <v>627791</v>
       </c>
       <c r="F33" t="n">
-        <v>627791</v>
+        <v>20500</v>
       </c>
       <c r="G33" t="n">
-        <v>20500</v>
-      </c>
-      <c r="H33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3562,18 +3311,15 @@
         <v>256</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>64.09999999999999</v>
+        <v>3082</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>3082</v>
+        <v/>
       </c>
       <c r="G34" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H34" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3590,18 +3336,15 @@
         <v>4694</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>89.3</v>
       </c>
       <c r="E35" t="n">
-        <v>89.3</v>
+        <v>235091</v>
       </c>
       <c r="F35" t="n">
-        <v>235091</v>
+        <v/>
       </c>
       <c r="G35" t="n">
-        <v/>
-      </c>
-      <c r="H35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3618,18 +3361,15 @@
         <v>27254</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>89.59999999999999</v>
+        <v>663082</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>663082</v>
+        <v>10700</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>10700</v>
-      </c>
-      <c r="H36" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3646,18 +3386,15 @@
         <v>270</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E37" t="n">
-        <v>66.40000000000001</v>
+        <v>82197</v>
       </c>
       <c r="F37" t="n">
-        <v>82197</v>
+        <v/>
       </c>
       <c r="G37" t="n">
-        <v/>
-      </c>
-      <c r="H37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3674,18 +3411,15 @@
         <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0</v>
+        <v>82.5</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>82.5</v>
+        <v>175272</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>175272</v>
+        <v/>
       </c>
       <c r="G38" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H38" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3702,18 +3436,15 @@
         <v>5831</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="E39" t="n">
-        <v>79.59999999999999</v>
+        <v>110623</v>
       </c>
       <c r="F39" t="n">
-        <v>110623</v>
+        <v>37500</v>
       </c>
       <c r="G39" t="n">
-        <v>37500</v>
-      </c>
-      <c r="H39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3730,18 +3461,15 @@
         <v>2</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0</v>
+        <v>89.3</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>89.3</v>
+        <v>13686</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>13686</v>
+        <v/>
       </c>
       <c r="G40" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H40" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3758,18 +3486,15 @@
         <v>22265</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>0</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>84.40000000000001</v>
+        <v>844921</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>844921</v>
+        <v>23100</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>23100</v>
-      </c>
-      <c r="H41" s="4" t="n">
         <v>65</v>
       </c>
     </row>
@@ -3786,18 +3511,15 @@
         <v>44886</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>0</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>79.09999999999999</v>
+        <v>797216</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>797216</v>
+        <v>8600</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>8600</v>
-      </c>
-      <c r="H42" s="4" t="n">
         <v>60</v>
       </c>
     </row>
@@ -3814,18 +3536,15 @@
         <v>5716</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>90.2</v>
       </c>
       <c r="E43" t="n">
-        <v>90.2</v>
+        <v>321395</v>
       </c>
       <c r="F43" t="n">
-        <v>321395</v>
+        <v>79800</v>
       </c>
       <c r="G43" t="n">
-        <v>79800</v>
-      </c>
-      <c r="H43" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3842,18 +3561,15 @@
         <v>34699</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>75.59999999999999</v>
+        <v>240355</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>240355</v>
+        <v/>
       </c>
       <c r="G44" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H44" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3870,18 +3586,15 @@
         <v>15893</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>0</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>96.09999999999999</v>
+        <v>835349</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>835349</v>
+        <v>6960</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>6960</v>
-      </c>
-      <c r="H45" s="4" t="n">
         <v>80</v>
       </c>
     </row>
@@ -3898,18 +3611,15 @@
         <v>3832</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>700785</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>700785</v>
+        <v>5500</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>5500</v>
-      </c>
-      <c r="H46" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3926,18 +3636,15 @@
         <v>664</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>81.3</v>
       </c>
       <c r="E47" t="n">
-        <v>81.3</v>
+        <v>473743</v>
       </c>
       <c r="F47" t="n">
-        <v>473743</v>
+        <v/>
       </c>
       <c r="G47" t="n">
-        <v/>
-      </c>
-      <c r="H47" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3954,18 +3661,15 @@
         <v>8551</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>0</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>92.40000000000001</v>
+        <v>295218</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>295218</v>
+        <v>9460</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>9460</v>
-      </c>
-      <c r="H48" s="4" t="n">
         <v>78</v>
       </c>
     </row>
@@ -3982,18 +3686,15 @@
         <v>17281</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="E49" t="n">
-        <v>97.40000000000001</v>
+        <v>867404</v>
       </c>
       <c r="F49" t="n">
-        <v>867404</v>
+        <v>24800</v>
       </c>
       <c r="G49" t="n">
-        <v>24800</v>
-      </c>
-      <c r="H49" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4010,18 +3711,15 @@
         <v>14439</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>0</v>
+        <v>94.3</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>94.3</v>
+        <v>499828</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>499828</v>
+        <v>11000</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H50" s="4" t="n">
         <v>50</v>
       </c>
     </row>
@@ -4038,18 +3736,15 @@
         <v>9978</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>95.8</v>
       </c>
       <c r="E51" t="n">
-        <v>95.8</v>
+        <v>768779</v>
       </c>
       <c r="F51" t="n">
-        <v>768779</v>
+        <v>21500</v>
       </c>
       <c r="G51" t="n">
-        <v>21500</v>
-      </c>
-      <c r="H51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4066,18 +3761,15 @@
         <v>1028</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>85</v>
+        <v>346404</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>346404</v>
+        <v/>
       </c>
       <c r="G52" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H52" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4094,18 +3786,15 @@
         <v>66954</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>69.5</v>
       </c>
       <c r="E53" t="n">
-        <v>69.5</v>
+        <v>324927</v>
       </c>
       <c r="F53" t="n">
-        <v>324927</v>
+        <v/>
       </c>
       <c r="G53" t="n">
-        <v/>
-      </c>
-      <c r="H53" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4141,7 +3830,117 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일) 이상 상위 50위 유지 게임 — 기준일: 2026-04-27</t>
+          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>게임명</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>유지 일수</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>평균 순위</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>최고 순위</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>평균 동접</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>최근 동접</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>평균 긍정리뷰(%)</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>최근 긍정리뷰(%)</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>총 리뷰수</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>현재 가격(₩)</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>최대 할인율(%)</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>첫 관측일</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>최근 관측일</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>아직 14일 분량의 데이터가 쌓이지 않았습니다. 매일 자동 수집이 진행되면 이 시트가 채워집니다.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-04-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-04-28
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -573,7 +573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -651,7 +651,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -690,7 +690,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -729,7 +729,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -846,7 +846,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -885,7 +885,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -924,7 +924,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -963,7 +963,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1002,7 +1002,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1041,7 +1041,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1080,7 +1080,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1119,7 +1119,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1158,7 +1158,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1197,7 +1197,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1236,7 +1236,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1275,7 +1275,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1314,7 +1314,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1353,7 +1353,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1392,7 +1392,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1431,7 +1431,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1470,7 +1470,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1509,7 +1509,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1536,10 +1536,10 @@
         <v>1071135</v>
       </c>
       <c r="I27" t="n">
-        <v>42000</v>
+        <v>21000</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K27" t="n">
         <v>42000</v>
@@ -1548,7 +1548,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1587,7 +1587,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1626,7 +1626,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1665,7 +1665,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1704,7 +1704,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1743,7 +1743,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1782,7 +1782,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1821,7 +1821,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1860,7 +1860,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1899,7 +1899,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1938,7 +1938,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1977,7 +1977,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2016,7 +2016,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2055,7 +2055,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2094,7 +2094,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2133,7 +2133,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2172,7 +2172,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2211,7 +2211,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2250,7 +2250,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2289,7 +2289,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2328,7 +2328,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2367,7 +2367,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2406,7 +2406,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2445,7 +2445,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2507,7 +2507,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-04-27</t>
+          <t>Steam 인기 차트 — 2026-04-28</t>
         </is>
       </c>
     </row>
@@ -3174,28 +3174,28 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Rust</t>
         </is>
       </c>
-      <c r="C29" t="n">
+      <c r="C29" s="4" t="n">
         <v>143870</v>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="4" t="n">
         <v>87.2</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="4" t="n">
         <v>1227784</v>
       </c>
-      <c r="F29" t="n">
-        <v>42000</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0</v>
+      <c r="F29" s="4" t="n">
+        <v>21000</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="30">
@@ -3830,7 +3830,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-04-27</t>
+          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-04-28</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-04-27</t>
+          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-04-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-04-29
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -573,7 +573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -651,7 +651,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -690,7 +690,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -729,7 +729,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -846,7 +846,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -885,7 +885,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -924,7 +924,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -963,7 +963,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1002,7 +1002,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1041,7 +1041,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1080,7 +1080,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1119,7 +1119,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1158,7 +1158,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1197,7 +1197,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1236,7 +1236,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1275,7 +1275,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1314,7 +1314,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1353,7 +1353,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1392,7 +1392,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1431,7 +1431,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1470,7 +1470,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1509,7 +1509,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1548,7 +1548,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1587,7 +1587,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1626,7 +1626,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1665,7 +1665,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1704,7 +1704,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1743,7 +1743,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1782,7 +1782,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1821,7 +1821,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1860,7 +1860,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1899,7 +1899,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1938,7 +1938,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1977,7 +1977,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2016,7 +2016,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2055,7 +2055,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2094,7 +2094,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2133,7 +2133,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2172,7 +2172,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2211,7 +2211,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2250,7 +2250,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2289,7 +2289,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2328,7 +2328,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2367,7 +2367,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2406,7 +2406,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2445,7 +2445,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2507,7 +2507,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-04-28</t>
+          <t>Steam 인기 차트 — 2026-04-29</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-04-28</t>
+          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-04-29</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-04-28</t>
+          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-04-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-01
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2591,10 +2591,10 @@
         <v>471451</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>11000</v>
+        <v>22000</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>22000</v>
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4307,10 +4307,10 @@
         <v>256362</v>
       </c>
       <c r="J87" t="n">
-        <v>33000</v>
+        <v>9900</v>
       </c>
       <c r="K87" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L87" t="n">
         <v>33000</v>
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4395,10 +4395,10 @@
         <v>195724</v>
       </c>
       <c r="J89" t="n">
-        <v>32000</v>
+        <v>8000</v>
       </c>
       <c r="K89" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="L89" t="n">
         <v>32000</v>
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4483,10 +4483,10 @@
         <v>304053</v>
       </c>
       <c r="J91" t="n">
-        <v>65000</v>
+        <v>6500</v>
       </c>
       <c r="K91" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L91" t="n">
         <v>65000</v>
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4791,10 +4791,10 @@
         <v>225479</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>29400</v>
+        <v>42000</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>42000</v>
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-04-30</t>
+          <t>Steam 인기 차트 — 2026-05-01</t>
         </is>
       </c>
     </row>
@@ -6380,33 +6380,33 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="n">
+      <c r="A50" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Valheim</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Early Access</t>
         </is>
       </c>
-      <c r="D50" s="4" t="n">
+      <c r="D50" s="2" t="n">
         <v>14439</v>
       </c>
-      <c r="E50" s="4" t="n">
+      <c r="E50" s="2" t="n">
         <v>94.3</v>
       </c>
-      <c r="F50" s="4" t="n">
+      <c r="F50" s="2" t="n">
         <v>499828</v>
       </c>
-      <c r="G50" s="4" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H50" s="4" t="n">
-        <v>50</v>
+      <c r="G50" s="2" t="n">
+        <v>22000</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -7550,33 +7550,33 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="n">
+      <c r="A89" s="4" t="n">
         <v>86</v>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="4" t="inlineStr">
         <is>
           <t>Cities: Skylines</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="4" t="inlineStr">
         <is>
           <t>Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D89" t="n">
+      <c r="D89" s="4" t="n">
         <v>8842</v>
       </c>
-      <c r="E89" t="n">
+      <c r="E89" s="4" t="n">
         <v>93</v>
       </c>
-      <c r="F89" t="n">
+      <c r="F89" s="4" t="n">
         <v>275770</v>
       </c>
-      <c r="G89" t="n">
-        <v>33000</v>
-      </c>
-      <c r="H89" t="n">
-        <v>0</v>
+      <c r="G89" s="4" t="n">
+        <v>9900</v>
+      </c>
+      <c r="H89" s="4" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="90">
@@ -7610,33 +7610,33 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="n">
+      <c r="A91" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="4" t="inlineStr">
         <is>
           <t>Sid Meier's Civilization® V</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="4" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="D91" t="n">
+      <c r="D91" s="4" t="n">
         <v>12206</v>
       </c>
-      <c r="E91" t="n">
+      <c r="E91" s="4" t="n">
         <v>95.8</v>
       </c>
-      <c r="F91" t="n">
+      <c r="F91" s="4" t="n">
         <v>204265</v>
       </c>
-      <c r="G91" t="n">
-        <v>32000</v>
-      </c>
-      <c r="H91" t="n">
-        <v>0</v>
+      <c r="G91" s="4" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H91" s="4" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="92">
@@ -7670,33 +7670,33 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="n">
+      <c r="A93" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>Sid Meier’s Civilization® VI</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="D93" t="n">
+      <c r="D93" s="4" t="n">
         <v>25420</v>
       </c>
-      <c r="E93" t="n">
+      <c r="E93" s="4" t="n">
         <v>86.90000000000001</v>
       </c>
-      <c r="F93" t="n">
+      <c r="F93" s="4" t="n">
         <v>349920</v>
       </c>
-      <c r="G93" t="n">
-        <v>65000</v>
-      </c>
-      <c r="H93" t="n">
-        <v>0</v>
+      <c r="G93" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="H93" s="4" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="94">
@@ -7880,33 +7880,33 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="4" t="n">
+      <c r="A100" s="2" t="n">
         <v>97</v>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B100" s="2" t="inlineStr">
         <is>
           <t>Satisfactory</t>
         </is>
       </c>
-      <c r="C100" s="4" t="inlineStr">
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>Adventure, Indie, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D100" s="4" t="n">
+      <c r="D100" s="2" t="n">
         <v>12596</v>
       </c>
-      <c r="E100" s="4" t="n">
+      <c r="E100" s="2" t="n">
         <v>97.2</v>
       </c>
-      <c r="F100" s="4" t="n">
+      <c r="F100" s="2" t="n">
         <v>232064</v>
       </c>
-      <c r="G100" s="4" t="n">
-        <v>29400</v>
-      </c>
-      <c r="H100" s="4" t="n">
-        <v>30</v>
+      <c r="G100" s="2" t="n">
+        <v>42000</v>
+      </c>
+      <c r="H100" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-04-30</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-01</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-04-30</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-01</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-04-30</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-02
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-01</t>
+          <t>Steam 인기 차트 — 2026-05-02</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-01</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-02</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-01</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-02</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-01</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-03
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -3999,19 +3999,19 @@
         <v>181110</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>36700</v>
+        <v>19560</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>36700</v>
+        <v>48900</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-02</t>
+          <t>Steam 인기 차트 — 2026-05-03</t>
         </is>
       </c>
     </row>
@@ -7340,33 +7340,33 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="4" t="n">
         <v>79</v>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B82" s="4" t="inlineStr">
         <is>
           <t>Hunt: Showdown 1896</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="C82" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D82" s="2" t="n">
+      <c r="D82" s="4" t="n">
         <v>6300</v>
       </c>
-      <c r="E82" s="2" t="n">
+      <c r="E82" s="4" t="n">
         <v>73</v>
       </c>
-      <c r="F82" s="2" t="n">
+      <c r="F82" s="4" t="n">
         <v>248220</v>
       </c>
-      <c r="G82" s="2" t="n">
-        <v>36700</v>
-      </c>
-      <c r="H82" s="2" t="n">
-        <v>0</v>
+      <c r="G82" s="4" t="n">
+        <v>19560</v>
+      </c>
+      <c r="H82" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="83">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-02</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-03</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-02</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-03</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-02</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-04
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2195,10 +2195,10 @@
         <v>713071</v>
       </c>
       <c r="J39" t="n">
-        <v>23100</v>
+        <v>66000</v>
       </c>
       <c r="K39" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
         <v>66000</v>
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2371,10 +2371,10 @@
         <v>802993</v>
       </c>
       <c r="J43" t="n">
-        <v>6960</v>
+        <v>34800</v>
       </c>
       <c r="K43" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L43" t="n">
         <v>34800</v>
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-03</t>
+          <t>Steam 인기 차트 — 2026-05-04</t>
         </is>
       </c>
     </row>
@@ -6110,33 +6110,33 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n">
+      <c r="A41" t="n">
         <v>38</v>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>Cyberpunk 2077</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>RPG</t>
         </is>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="D41" t="n">
         <v>22265</v>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="E41" t="n">
         <v>84.40000000000001</v>
       </c>
-      <c r="F41" s="4" t="n">
+      <c r="F41" t="n">
         <v>844921</v>
       </c>
-      <c r="G41" s="4" t="n">
-        <v>23100</v>
-      </c>
-      <c r="H41" s="4" t="n">
-        <v>65</v>
+      <c r="G41" t="n">
+        <v>66000</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -6230,33 +6230,33 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="n">
+      <c r="A45" t="n">
         <v>42</v>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>The Witcher 3: Wild Hunt</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>RPG</t>
         </is>
       </c>
-      <c r="D45" s="4" t="n">
+      <c r="D45" t="n">
         <v>15893</v>
       </c>
-      <c r="E45" s="4" t="n">
+      <c r="E45" t="n">
         <v>96.09999999999999</v>
       </c>
-      <c r="F45" s="4" t="n">
+      <c r="F45" t="n">
         <v>835349</v>
       </c>
-      <c r="G45" s="4" t="n">
-        <v>6960</v>
-      </c>
-      <c r="H45" s="4" t="n">
-        <v>80</v>
+      <c r="G45" t="n">
+        <v>34800</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-03</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-04</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-03</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-04</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-03</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-05
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1449,10 +1449,10 @@
         <v>736688</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>66000</v>
+        <v>49500</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>66000</v>
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2503,19 +2503,19 @@
         <v>272900</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>9460</v>
+        <v>21000</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>43000</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3735,10 +3735,10 @@
         <v>202253</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>20500</v>
+        <v>6150</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>20500</v>
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-04</t>
+          <t>Steam 인기 차트 — 2026-05-05</t>
         </is>
       </c>
     </row>
@@ -5602,33 +5602,33 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Baldur's Gate 3</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Adventure, RPG, Strategy</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D24" s="4" t="n">
         <v>54771</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="4" t="n">
         <v>96.8</v>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="F24" s="4" t="n">
         <v>760662</v>
       </c>
-      <c r="G24" s="2" t="n">
-        <v>66000</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>0</v>
+      <c r="G24" s="4" t="n">
+        <v>49500</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="25">
@@ -6320,33 +6320,33 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="n">
+      <c r="A48" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Borderlands 2</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D48" s="4" t="n">
+      <c r="D48" s="2" t="n">
         <v>8551</v>
       </c>
-      <c r="E48" s="4" t="n">
+      <c r="E48" s="2" t="n">
         <v>92.40000000000001</v>
       </c>
-      <c r="F48" s="4" t="n">
+      <c r="F48" s="2" t="n">
         <v>295218</v>
       </c>
-      <c r="G48" s="4" t="n">
-        <v>9460</v>
-      </c>
-      <c r="H48" s="4" t="n">
-        <v>78</v>
+      <c r="G48" s="2" t="n">
+        <v>21000</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -7160,33 +7160,33 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="4" t="n">
         <v>73</v>
       </c>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="B76" s="4" t="inlineStr">
         <is>
           <t>Human Fall Flat</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
+      <c r="C76" s="4" t="inlineStr">
         <is>
           <t>Adventure, Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D76" s="2" t="n">
+      <c r="D76" s="4" t="n">
         <v>950</v>
       </c>
-      <c r="E76" s="2" t="n">
+      <c r="E76" s="4" t="n">
         <v>94.7</v>
       </c>
-      <c r="F76" s="2" t="n">
+      <c r="F76" s="4" t="n">
         <v>213640</v>
       </c>
-      <c r="G76" s="2" t="n">
-        <v>20500</v>
-      </c>
-      <c r="H76" s="2" t="n">
-        <v>0</v>
+      <c r="G76" s="4" t="n">
+        <v>6150</v>
+      </c>
+      <c r="H76" s="4" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="77">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-04</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-05</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-04</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-05</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-04</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-06
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2635,10 +2635,10 @@
         <v>736611</v>
       </c>
       <c r="J49" t="n">
-        <v>21500</v>
+        <v>15050</v>
       </c>
       <c r="K49" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L49" t="n">
         <v>21500</v>
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-05</t>
+          <t>Steam 인기 차트 — 2026-05-06</t>
         </is>
       </c>
     </row>
@@ -6410,33 +6410,33 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>Phasmophobia</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Action, Indie, Early Access</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D51" s="4" t="n">
         <v>9978</v>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="4" t="n">
         <v>95.8</v>
       </c>
-      <c r="F51" t="n">
+      <c r="F51" s="4" t="n">
         <v>768779</v>
       </c>
-      <c r="G51" t="n">
-        <v>21500</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0</v>
+      <c r="G51" s="4" t="n">
+        <v>15050</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="52">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-05</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-06</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-05</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-06</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-05</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-07
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-06</t>
+          <t>Steam 인기 차트 — 2026-05-07</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-06</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-07</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-06</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-07</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-06</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-08
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1537,10 +1537,10 @@
         <v>1122546</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>5250</v>
+        <v>10500</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>10500</v>
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2239,10 +2239,10 @@
         <v>630223</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>8600</v>
+        <v>21500</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>21500</v>
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3119,10 +3119,10 @@
         <v>139186</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>3300</v>
+        <v>66000</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>66000</v>
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -3999,19 +3999,19 @@
         <v>181110</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>19560</v>
+        <v>36700</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>48900</v>
+        <v>36700</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4307,10 +4307,10 @@
         <v>256362</v>
       </c>
       <c r="J87" t="n">
-        <v>9900</v>
+        <v>33000</v>
       </c>
       <c r="K87" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L87" t="n">
         <v>33000</v>
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4659,10 +4659,10 @@
         <v>177352</v>
       </c>
       <c r="J95" t="n">
-        <v>2750</v>
+        <v>55000</v>
       </c>
       <c r="K95" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="L95" t="n">
         <v>55000</v>
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-07</t>
+          <t>Steam 인기 차트 — 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -5662,33 +5662,33 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Garry's Mod</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="D26" s="2" t="n">
         <v>18400</v>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="E26" s="2" t="n">
         <v>96.8</v>
       </c>
-      <c r="F26" s="4" t="n">
+      <c r="F26" s="2" t="n">
         <v>1159707</v>
       </c>
-      <c r="G26" s="4" t="n">
-        <v>5250</v>
-      </c>
-      <c r="H26" s="4" t="n">
-        <v>50</v>
+      <c r="G26" s="2" t="n">
+        <v>10500</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -6140,33 +6140,33 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n">
+      <c r="A42" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Dead by Daylight</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D42" s="4" t="n">
+      <c r="D42" s="2" t="n">
         <v>44886</v>
       </c>
-      <c r="E42" s="4" t="n">
+      <c r="E42" s="2" t="n">
         <v>79.09999999999999</v>
       </c>
-      <c r="F42" s="4" t="n">
+      <c r="F42" s="2" t="n">
         <v>797216</v>
       </c>
-      <c r="G42" s="4" t="n">
-        <v>8600</v>
-      </c>
-      <c r="H42" s="4" t="n">
-        <v>60</v>
+      <c r="G42" s="2" t="n">
+        <v>21500</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -6740,33 +6740,33 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="n">
+      <c r="A62" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>Battlefield™ 2042</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Casual</t>
         </is>
       </c>
-      <c r="D62" s="4" t="n">
+      <c r="D62" s="2" t="n">
         <v>2774</v>
       </c>
-      <c r="E62" s="4" t="n">
+      <c r="E62" s="2" t="n">
         <v>46.7</v>
       </c>
-      <c r="F62" s="4" t="n">
+      <c r="F62" s="2" t="n">
         <v>297774</v>
       </c>
-      <c r="G62" s="4" t="n">
-        <v>3300</v>
-      </c>
-      <c r="H62" s="4" t="n">
-        <v>95</v>
+      <c r="G62" s="2" t="n">
+        <v>66000</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -7340,33 +7340,33 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="4" t="n">
+      <c r="A82" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="B82" s="4" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>Hunt: Showdown 1896</t>
         </is>
       </c>
-      <c r="C82" s="4" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D82" s="4" t="n">
+      <c r="D82" s="2" t="n">
         <v>6300</v>
       </c>
-      <c r="E82" s="4" t="n">
+      <c r="E82" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="F82" s="4" t="n">
+      <c r="F82" s="2" t="n">
         <v>248220</v>
       </c>
-      <c r="G82" s="4" t="n">
-        <v>19560</v>
-      </c>
-      <c r="H82" s="4" t="n">
-        <v>60</v>
+      <c r="G82" s="2" t="n">
+        <v>36700</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -7550,33 +7550,33 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="4" t="n">
+      <c r="A89" t="n">
         <v>86</v>
       </c>
-      <c r="B89" s="4" t="inlineStr">
+      <c r="B89" t="inlineStr">
         <is>
           <t>Cities: Skylines</t>
         </is>
       </c>
-      <c r="C89" s="4" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D89" s="4" t="n">
+      <c r="D89" t="n">
         <v>8842</v>
       </c>
-      <c r="E89" s="4" t="n">
+      <c r="E89" t="n">
         <v>93</v>
       </c>
-      <c r="F89" s="4" t="n">
+      <c r="F89" t="n">
         <v>275770</v>
       </c>
-      <c r="G89" s="4" t="n">
-        <v>9900</v>
-      </c>
-      <c r="H89" s="4" t="n">
-        <v>70</v>
+      <c r="G89" t="n">
+        <v>33000</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -7790,33 +7790,33 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="4" t="n">
+      <c r="A97" t="n">
         <v>94</v>
       </c>
-      <c r="B97" s="4" t="inlineStr">
+      <c r="B97" t="inlineStr">
         <is>
           <t>Battlefield™ V</t>
         </is>
       </c>
-      <c r="C97" s="4" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D97" s="4" t="n">
+      <c r="D97" t="n">
         <v>6327</v>
       </c>
-      <c r="E97" s="4" t="n">
+      <c r="E97" t="n">
         <v>70.90000000000001</v>
       </c>
-      <c r="F97" s="4" t="n">
+      <c r="F97" t="n">
         <v>250288</v>
       </c>
-      <c r="G97" s="4" t="n">
-        <v>2750</v>
-      </c>
-      <c r="H97" s="4" t="n">
-        <v>95</v>
+      <c r="G97" t="n">
+        <v>55000</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-07</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-07</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-07</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-09
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-08</t>
+          <t>Steam 인기 차트 — 2026-05-09</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-08</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-09</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-08</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-09</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-08</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-10
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-09</t>
+          <t>Steam 인기 차트 — 2026-05-10</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-09</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-10</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-09</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-10</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-09</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-11
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-10</t>
+          <t>Steam 인기 차트 — 2026-05-11</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-10</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-11</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-10</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-11</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-10</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-12
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1449,10 +1449,10 @@
         <v>736688</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>49500</v>
+        <v>66000</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>66000</v>
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1669,10 +1669,10 @@
         <v>1071135</v>
       </c>
       <c r="J27" t="n">
-        <v>21000</v>
+        <v>42000</v>
       </c>
       <c r="K27" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
         <v>42000</v>
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3075,10 +3075,10 @@
         <v>676667</v>
       </c>
       <c r="J59" t="n">
-        <v>73000</v>
+        <v>18250</v>
       </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="L59" t="n">
         <v>73000</v>
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4703,10 +4703,10 @@
         <v>179154</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>7490</v>
+        <v>10700</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>10700</v>
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-11</t>
+          <t>Steam 인기 차트 — 2026-05-12</t>
         </is>
       </c>
     </row>
@@ -5602,33 +5602,33 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Baldur's Gate 3</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Adventure, RPG, Strategy</t>
         </is>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="D24" s="2" t="n">
         <v>54771</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" s="2" t="n">
         <v>96.8</v>
       </c>
-      <c r="F24" s="4" t="n">
+      <c r="F24" s="2" t="n">
         <v>760662</v>
       </c>
-      <c r="G24" s="4" t="n">
-        <v>49500</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>25</v>
+      <c r="G24" s="2" t="n">
+        <v>66000</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -5752,33 +5752,33 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n">
+      <c r="A29" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Rust</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Massively Multiplayer, RPG</t>
         </is>
       </c>
-      <c r="D29" s="4" t="n">
+      <c r="D29" t="n">
         <v>143870</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" t="n">
         <v>87.2</v>
       </c>
-      <c r="F29" s="4" t="n">
+      <c r="F29" t="n">
         <v>1227784</v>
       </c>
-      <c r="G29" s="4" t="n">
-        <v>21000</v>
-      </c>
-      <c r="H29" s="4" t="n">
-        <v>50</v>
+      <c r="G29" t="n">
+        <v>42000</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -6710,33 +6710,33 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="n">
+      <c r="A61" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>Red Dead Redemption 2</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure</t>
         </is>
       </c>
-      <c r="D61" t="n">
+      <c r="D61" s="4" t="n">
         <v>29885</v>
       </c>
-      <c r="E61" t="n">
+      <c r="E61" s="4" t="n">
         <v>92.2</v>
       </c>
-      <c r="F61" t="n">
+      <c r="F61" s="4" t="n">
         <v>733542</v>
       </c>
-      <c r="G61" t="n">
-        <v>73000</v>
-      </c>
-      <c r="H61" t="n">
-        <v>0</v>
+      <c r="G61" s="4" t="n">
+        <v>18250</v>
+      </c>
+      <c r="H61" s="4" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="62">
@@ -7820,33 +7820,33 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="4" t="n">
+      <c r="A98" s="2" t="n">
         <v>95</v>
       </c>
-      <c r="B98" s="4" t="inlineStr">
+      <c r="B98" s="2" t="inlineStr">
         <is>
           <t>R.E.P.O.</t>
         </is>
       </c>
-      <c r="C98" s="4" t="inlineStr">
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>Action, Early Access</t>
         </is>
       </c>
-      <c r="D98" s="4" t="n">
+      <c r="D98" s="2" t="n">
         <v>32349</v>
       </c>
-      <c r="E98" s="4" t="n">
+      <c r="E98" s="2" t="n">
         <v>96.5</v>
       </c>
-      <c r="F98" s="4" t="n">
+      <c r="F98" s="2" t="n">
         <v>185642</v>
       </c>
-      <c r="G98" s="4" t="n">
-        <v>7490</v>
-      </c>
-      <c r="H98" s="4" t="n">
-        <v>30</v>
+      <c r="G98" s="2" t="n">
+        <v>10700</v>
+      </c>
+      <c r="H98" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-11</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-12</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-11</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-12</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-11</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-13
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-12</t>
+          <t>Steam 인기 차트 — 2026-05-13</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-12</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-13</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-12</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-13</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-12</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-14
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1975,10 +1975,10 @@
         <v>594327</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>10700</v>
+        <v>5350</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>10700</v>
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-13</t>
+          <t>Steam 인기 차트 — 2026-05-14</t>
         </is>
       </c>
     </row>
@@ -5960,33 +5960,33 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>PAYDAY 2</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D36" s="4" t="n">
         <v>27254</v>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E36" s="4" t="n">
         <v>89.59999999999999</v>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="F36" s="4" t="n">
         <v>663082</v>
       </c>
-      <c r="G36" s="2" t="n">
-        <v>10700</v>
-      </c>
-      <c r="H36" s="2" t="n">
-        <v>0</v>
+      <c r="G36" s="4" t="n">
+        <v>5350</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="37">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-13</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-14</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-13</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-14</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-13</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-15
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1801,10 +1801,10 @@
         <v>872384</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>16000</v>
+        <v>8000</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>16000</v>
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2547,10 +2547,10 @@
         <v>844480</v>
       </c>
       <c r="J47" t="n">
-        <v>24800</v>
+        <v>6200</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="L47" t="n">
         <v>24800</v>
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3691,10 +3691,10 @@
         <v>435687</v>
       </c>
       <c r="J73" t="n">
-        <v>27400</v>
+        <v>5480</v>
       </c>
       <c r="K73" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="L73" t="n">
         <v>27400</v>
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4395,10 +4395,10 @@
         <v>195724</v>
       </c>
       <c r="J89" t="n">
-        <v>8000</v>
+        <v>32000</v>
       </c>
       <c r="K89" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="L89" t="n">
         <v>32000</v>
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4483,10 +4483,10 @@
         <v>304053</v>
       </c>
       <c r="J91" t="n">
-        <v>6500</v>
+        <v>65000</v>
       </c>
       <c r="K91" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L91" t="n">
         <v>65000</v>
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-14</t>
+          <t>Steam 인기 차트 — 2026-05-15</t>
         </is>
       </c>
     </row>
@@ -5842,33 +5842,33 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Stardew Valley</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Indie, RPG, Simulation</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n">
+      <c r="D32" s="4" t="n">
         <v>50662</v>
       </c>
-      <c r="E32" s="2" t="n">
+      <c r="E32" s="4" t="n">
         <v>98.40000000000001</v>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="F32" s="4" t="n">
         <v>886195</v>
       </c>
-      <c r="G32" s="2" t="n">
-        <v>16000</v>
-      </c>
-      <c r="H32" s="2" t="n">
-        <v>0</v>
+      <c r="G32" s="4" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="33">
@@ -6350,33 +6350,33 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>Euro Truck Simulator 2</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Indie, Simulation</t>
         </is>
       </c>
-      <c r="D49" t="n">
+      <c r="D49" s="4" t="n">
         <v>17281</v>
       </c>
-      <c r="E49" t="n">
+      <c r="E49" s="4" t="n">
         <v>97.40000000000001</v>
       </c>
-      <c r="F49" t="n">
+      <c r="F49" s="4" t="n">
         <v>867404</v>
       </c>
-      <c r="G49" t="n">
-        <v>24800</v>
-      </c>
-      <c r="H49" t="n">
-        <v>0</v>
+      <c r="G49" s="4" t="n">
+        <v>6200</v>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="50">
@@ -7130,33 +7130,33 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="n">
+      <c r="A75" s="4" t="n">
         <v>72</v>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="4" t="inlineStr">
         <is>
           <t>Dying Light</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="4" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D75" t="n">
+      <c r="D75" s="4" t="n">
         <v>4953</v>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="4" t="n">
         <v>95.2</v>
       </c>
-      <c r="F75" t="n">
+      <c r="F75" s="4" t="n">
         <v>457632</v>
       </c>
-      <c r="G75" t="n">
-        <v>27400</v>
-      </c>
-      <c r="H75" t="n">
-        <v>0</v>
+      <c r="G75" s="4" t="n">
+        <v>5480</v>
+      </c>
+      <c r="H75" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="76">
@@ -7610,33 +7610,33 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="4" t="n">
+      <c r="A91" t="n">
         <v>88</v>
       </c>
-      <c r="B91" s="4" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>Sid Meier's Civilization® V</t>
         </is>
       </c>
-      <c r="C91" s="4" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="D91" s="4" t="n">
+      <c r="D91" t="n">
         <v>12206</v>
       </c>
-      <c r="E91" s="4" t="n">
+      <c r="E91" t="n">
         <v>95.8</v>
       </c>
-      <c r="F91" s="4" t="n">
+      <c r="F91" t="n">
         <v>204265</v>
       </c>
-      <c r="G91" s="4" t="n">
-        <v>8000</v>
-      </c>
-      <c r="H91" s="4" t="n">
-        <v>75</v>
+      <c r="G91" t="n">
+        <v>32000</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -7670,33 +7670,33 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="4" t="n">
+      <c r="A93" t="n">
         <v>90</v>
       </c>
-      <c r="B93" s="4" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>Sid Meier’s Civilization® VI</t>
         </is>
       </c>
-      <c r="C93" s="4" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="D93" s="4" t="n">
+      <c r="D93" t="n">
         <v>25420</v>
       </c>
-      <c r="E93" s="4" t="n">
+      <c r="E93" t="n">
         <v>86.90000000000001</v>
       </c>
-      <c r="F93" s="4" t="n">
+      <c r="F93" t="n">
         <v>349920</v>
       </c>
-      <c r="G93" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="H93" s="4" t="n">
-        <v>90</v>
+      <c r="G93" t="n">
+        <v>65000</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-14</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-15</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-14</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-15</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-14</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-16
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-15</t>
+          <t>Steam 인기 차트 — 2026-05-16</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-15</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-16</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-15</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-16</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-15</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-18
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-16</t>
+          <t>Steam 인기 차트 — 2026-05-18</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-16</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-18</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-16</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-18</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-16</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-19
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3735,10 +3735,10 @@
         <v>202253</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>6150</v>
+        <v>20500</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>20500</v>
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-18</t>
+          <t>Steam 인기 차트 — 2026-05-19</t>
         </is>
       </c>
     </row>
@@ -7160,33 +7160,33 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="4" t="n">
+      <c r="A76" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="B76" s="4" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>Human Fall Flat</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>Adventure, Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D76" s="4" t="n">
+      <c r="D76" s="2" t="n">
         <v>950</v>
       </c>
-      <c r="E76" s="4" t="n">
+      <c r="E76" s="2" t="n">
         <v>94.7</v>
       </c>
-      <c r="F76" s="4" t="n">
+      <c r="F76" s="2" t="n">
         <v>213640</v>
       </c>
-      <c r="G76" s="4" t="n">
-        <v>6150</v>
-      </c>
-      <c r="H76" s="4" t="n">
-        <v>70</v>
+      <c r="G76" s="2" t="n">
+        <v>20500</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-18</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-19</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-18</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-19</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-18</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-20
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1757,10 +1757,10 @@
         <v>612177</v>
       </c>
       <c r="J29" t="n">
-        <v>16500</v>
+        <v>10890</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="L29" t="n">
         <v>16500</v>
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2635,10 +2635,10 @@
         <v>736611</v>
       </c>
       <c r="J49" t="n">
-        <v>15050</v>
+        <v>21500</v>
       </c>
       <c r="K49" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L49" t="n">
         <v>21500</v>
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-19</t>
+          <t>Steam 인기 차트 — 2026-05-20</t>
         </is>
       </c>
     </row>
@@ -5812,33 +5812,33 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>ARK: Survival Evolved</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Massively Multiplayer, RPG</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="4" t="n">
         <v>22170</v>
       </c>
-      <c r="E31" t="n">
+      <c r="E31" s="4" t="n">
         <v>83.8</v>
       </c>
-      <c r="F31" t="n">
+      <c r="F31" s="4" t="n">
         <v>730170</v>
       </c>
-      <c r="G31" t="n">
-        <v>16500</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0</v>
+      <c r="G31" s="4" t="n">
+        <v>10890</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="32">
@@ -6410,33 +6410,33 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="n">
+      <c r="A51" t="n">
         <v>48</v>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Phasmophobia</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Action, Indie, Early Access</t>
         </is>
       </c>
-      <c r="D51" s="4" t="n">
+      <c r="D51" t="n">
         <v>9978</v>
       </c>
-      <c r="E51" s="4" t="n">
+      <c r="E51" t="n">
         <v>95.8</v>
       </c>
-      <c r="F51" s="4" t="n">
+      <c r="F51" t="n">
         <v>768779</v>
       </c>
-      <c r="G51" s="4" t="n">
-        <v>15050</v>
-      </c>
-      <c r="H51" s="4" t="n">
-        <v>30</v>
+      <c r="G51" t="n">
+        <v>21500</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-19</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-20</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-19</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-20</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-19</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-21
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-20</t>
+          <t>Steam 인기 차트 — 2026-05-21</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-20</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-21</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-20</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-21</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-20</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-22
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1801,10 +1801,10 @@
         <v>872384</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>8000</v>
+        <v>16000</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>16000</v>
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3031,10 +3031,10 @@
         <v>473422</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>11000</v>
+        <v>7150</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>11000</v>
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4615,10 +4615,10 @@
         <v>26360</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>53000</v>
+        <v>21200</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>53000</v>
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4879,10 +4879,10 @@
         <v>293127</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>26000</v>
+        <v>8580</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>26000</v>
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-21</t>
+          <t>Steam 인기 차트 — 2026-05-22</t>
         </is>
       </c>
     </row>
@@ -5842,33 +5842,33 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Stardew Valley</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Indie, RPG, Simulation</t>
         </is>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="D32" s="2" t="n">
         <v>50662</v>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="E32" s="2" t="n">
         <v>98.40000000000001</v>
       </c>
-      <c r="F32" s="4" t="n">
+      <c r="F32" s="2" t="n">
         <v>886195</v>
       </c>
-      <c r="G32" s="4" t="n">
-        <v>8000</v>
-      </c>
-      <c r="H32" s="4" t="n">
-        <v>50</v>
+      <c r="G32" s="2" t="n">
+        <v>16000</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -6680,33 +6680,33 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="4" t="n">
         <v>57</v>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>Lethal Company</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Early Access</t>
         </is>
       </c>
-      <c r="D60" s="2" t="n">
+      <c r="D60" s="4" t="n">
         <v>6199</v>
       </c>
-      <c r="E60" s="2" t="n">
+      <c r="E60" s="4" t="n">
         <v>97.2</v>
       </c>
-      <c r="F60" s="2" t="n">
+      <c r="F60" s="4" t="n">
         <v>487160</v>
       </c>
-      <c r="G60" s="2" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H60" s="2" t="n">
-        <v>0</v>
+      <c r="G60" s="4" t="n">
+        <v>7150</v>
+      </c>
+      <c r="H60" s="4" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="61">
@@ -7760,33 +7760,33 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="4" t="n">
         <v>93</v>
       </c>
-      <c r="B96" s="2" t="inlineStr">
+      <c r="B96" s="4" t="inlineStr">
         <is>
           <t>Warhammer 40,000: Rogue Trader</t>
         </is>
       </c>
-      <c r="C96" s="2" t="inlineStr">
+      <c r="C96" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Strategy</t>
         </is>
       </c>
-      <c r="D96" s="2" t="n">
+      <c r="D96" s="4" t="n">
         <v>3582</v>
       </c>
-      <c r="E96" s="2" t="n">
+      <c r="E96" s="4" t="n">
         <v>85.59999999999999</v>
       </c>
-      <c r="F96" s="2" t="n">
+      <c r="F96" s="4" t="n">
         <v>30805</v>
       </c>
-      <c r="G96" s="2" t="n">
-        <v>53000</v>
-      </c>
-      <c r="H96" s="2" t="n">
-        <v>0</v>
+      <c r="G96" s="4" t="n">
+        <v>21200</v>
+      </c>
+      <c r="H96" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="97">
@@ -7940,33 +7940,33 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="4" t="n">
         <v>99</v>
       </c>
-      <c r="B102" s="2" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>Risk of Rain 2</t>
         </is>
       </c>
-      <c r="C102" s="2" t="inlineStr">
+      <c r="C102" s="4" t="inlineStr">
         <is>
           <t>Action, Indie</t>
         </is>
       </c>
-      <c r="D102" s="2" t="n">
+      <c r="D102" s="4" t="n">
         <v>7902</v>
       </c>
-      <c r="E102" s="2" t="n">
+      <c r="E102" s="4" t="n">
         <v>93.5</v>
       </c>
-      <c r="F102" s="2" t="n">
+      <c r="F102" s="4" t="n">
         <v>313577</v>
       </c>
-      <c r="G102" s="2" t="n">
-        <v>26000</v>
-      </c>
-      <c r="H102" s="2" t="n">
-        <v>0</v>
+      <c r="G102" s="4" t="n">
+        <v>8580</v>
+      </c>
+      <c r="H102" s="4" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="103">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-21</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-22</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-21</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-22</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-21</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-23
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-22</t>
+          <t>Steam 인기 차트 — 2026-05-23</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-22</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-23</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-22</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-23</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-22</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-24
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-23</t>
+          <t>Steam 인기 차트 — 2026-05-24</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-23</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-24</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-23</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-24</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-23</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-25
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2547,10 +2547,10 @@
         <v>844480</v>
       </c>
       <c r="J47" t="n">
-        <v>6200</v>
+        <v>24800</v>
       </c>
       <c r="K47" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="L47" t="n">
         <v>24800</v>
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-24</t>
+          <t>Steam 인기 차트 — 2026-05-25</t>
         </is>
       </c>
     </row>
@@ -6350,33 +6350,33 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="n">
+      <c r="A49" t="n">
         <v>46</v>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>Euro Truck Simulator 2</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>Indie, Simulation</t>
         </is>
       </c>
-      <c r="D49" s="4" t="n">
+      <c r="D49" t="n">
         <v>17281</v>
       </c>
-      <c r="E49" s="4" t="n">
+      <c r="E49" t="n">
         <v>97.40000000000001</v>
       </c>
-      <c r="F49" s="4" t="n">
+      <c r="F49" t="n">
         <v>867404</v>
       </c>
-      <c r="G49" s="4" t="n">
-        <v>6200</v>
-      </c>
-      <c r="H49" s="4" t="n">
-        <v>75</v>
+      <c r="G49" t="n">
+        <v>24800</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-24</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-25</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-24</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-25</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-24</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-26
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3075,10 +3075,10 @@
         <v>676667</v>
       </c>
       <c r="J59" t="n">
-        <v>18250</v>
+        <v>73000</v>
       </c>
       <c r="K59" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="L59" t="n">
         <v>73000</v>
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-25</t>
+          <t>Steam 인기 차트 — 2026-05-26</t>
         </is>
       </c>
     </row>
@@ -6710,33 +6710,33 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="n">
+      <c r="A61" t="n">
         <v>58</v>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>Red Dead Redemption 2</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>Action, Adventure</t>
         </is>
       </c>
-      <c r="D61" s="4" t="n">
+      <c r="D61" t="n">
         <v>29885</v>
       </c>
-      <c r="E61" s="4" t="n">
+      <c r="E61" t="n">
         <v>92.2</v>
       </c>
-      <c r="F61" s="4" t="n">
+      <c r="F61" t="n">
         <v>733542</v>
       </c>
-      <c r="G61" s="4" t="n">
-        <v>18250</v>
-      </c>
-      <c r="H61" s="4" t="n">
-        <v>75</v>
+      <c r="G61" t="n">
+        <v>73000</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-25</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-26</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-25</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-26</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-25</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-27
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -705,10 +705,10 @@
         <v>358266</v>
       </c>
       <c r="J5" t="n">
-        <v>32000</v>
+        <v>24000</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="L5" t="n">
         <v>32000</v>
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2811,10 +2811,10 @@
         <v>143086</v>
       </c>
       <c r="J53" t="n">
-        <v>10500</v>
+        <v>7870</v>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="L53" t="n">
         <v>10500</v>
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-26</t>
+          <t>Steam 인기 차트 — 2026-05-27</t>
         </is>
       </c>
     </row>
@@ -5096,33 +5096,33 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Palworld</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Early Access</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="4" t="n">
         <v>18028</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="4" t="n">
         <v>94.09999999999999</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="4" t="n">
         <v>380709</v>
       </c>
-      <c r="G7" t="n">
-        <v>32000</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
+      <c r="G7" s="4" t="n">
+        <v>24000</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -6530,33 +6530,33 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="n">
+      <c r="A55" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>Half-Life</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D55" t="n">
+      <c r="D55" s="4" t="n">
         <v>634</v>
       </c>
-      <c r="E55" t="n">
+      <c r="E55" s="4" t="n">
         <v>96.5</v>
       </c>
-      <c r="F55" t="n">
+      <c r="F55" s="4" t="n">
         <v>148221</v>
       </c>
-      <c r="G55" t="n">
-        <v>10500</v>
-      </c>
-      <c r="H55" t="n">
-        <v>0</v>
+      <c r="G55" s="4" t="n">
+        <v>7870</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="56">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-26</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-27</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-26</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-27</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-26</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-28
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1975,10 +1975,10 @@
         <v>594327</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>5350</v>
+        <v>10700</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>10700</v>
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2283,10 +2283,10 @@
         <v>289966</v>
       </c>
       <c r="J41" t="n">
-        <v>79800</v>
+        <v>11970</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="L41" t="n">
         <v>79800</v>
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4263,10 +4263,10 @@
         <v>93489</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>27000</v>
+        <v>5400</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>27000</v>
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-27</t>
+          <t>Steam 인기 차트 — 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -5960,33 +5960,33 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n">
+      <c r="A36" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>PAYDAY 2</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D36" s="4" t="n">
+      <c r="D36" s="2" t="n">
         <v>27254</v>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="E36" s="2" t="n">
         <v>89.59999999999999</v>
       </c>
-      <c r="F36" s="4" t="n">
+      <c r="F36" s="2" t="n">
         <v>663082</v>
       </c>
-      <c r="G36" s="4" t="n">
-        <v>5350</v>
-      </c>
-      <c r="H36" s="4" t="n">
-        <v>50</v>
+      <c r="G36" s="2" t="n">
+        <v>10700</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -6170,33 +6170,33 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>Hogwarts Legacy</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, RPG</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D43" s="4" t="n">
         <v>5716</v>
       </c>
-      <c r="E43" t="n">
+      <c r="E43" s="4" t="n">
         <v>90.2</v>
       </c>
-      <c r="F43" t="n">
+      <c r="F43" s="4" t="n">
         <v>321395</v>
       </c>
-      <c r="G43" t="n">
-        <v>79800</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
+      <c r="G43" s="4" t="n">
+        <v>11970</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="44">
@@ -7520,33 +7520,33 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="4" t="n">
         <v>85</v>
       </c>
-      <c r="B88" s="2" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>Grim Dawn</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C88" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D88" s="2" t="n">
+      <c r="D88" s="4" t="n">
         <v>2376</v>
       </c>
-      <c r="E88" s="2" t="n">
+      <c r="E88" s="4" t="n">
         <v>93.7</v>
       </c>
-      <c r="F88" s="2" t="n">
+      <c r="F88" s="4" t="n">
         <v>99730</v>
       </c>
-      <c r="G88" s="2" t="n">
-        <v>27000</v>
-      </c>
-      <c r="H88" s="2" t="n">
-        <v>0</v>
+      <c r="G88" s="4" t="n">
+        <v>5400</v>
+      </c>
+      <c r="H88" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="89">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-27</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-27</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-27</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-29
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3031,10 +3031,10 @@
         <v>473422</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>7150</v>
+        <v>11000</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>11000</v>
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3691,10 +3691,10 @@
         <v>435687</v>
       </c>
       <c r="J73" t="n">
-        <v>5480</v>
+        <v>27400</v>
       </c>
       <c r="K73" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L73" t="n">
         <v>27400</v>
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4615,10 +4615,10 @@
         <v>26360</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>21200</v>
+        <v>53000</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>53000</v>
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-28</t>
+          <t>Steam 인기 차트 — 2026-05-29</t>
         </is>
       </c>
     </row>
@@ -6680,33 +6680,33 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="n">
+      <c r="A60" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>Lethal Company</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Early Access</t>
         </is>
       </c>
-      <c r="D60" s="4" t="n">
+      <c r="D60" s="2" t="n">
         <v>6199</v>
       </c>
-      <c r="E60" s="4" t="n">
+      <c r="E60" s="2" t="n">
         <v>97.2</v>
       </c>
-      <c r="F60" s="4" t="n">
+      <c r="F60" s="2" t="n">
         <v>487160</v>
       </c>
-      <c r="G60" s="4" t="n">
-        <v>7150</v>
-      </c>
-      <c r="H60" s="4" t="n">
-        <v>35</v>
+      <c r="G60" s="2" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -7130,33 +7130,33 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="4" t="n">
+      <c r="A75" t="n">
         <v>72</v>
       </c>
-      <c r="B75" s="4" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>Dying Light</t>
         </is>
       </c>
-      <c r="C75" s="4" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D75" s="4" t="n">
+      <c r="D75" t="n">
         <v>4953</v>
       </c>
-      <c r="E75" s="4" t="n">
+      <c r="E75" t="n">
         <v>95.2</v>
       </c>
-      <c r="F75" s="4" t="n">
+      <c r="F75" t="n">
         <v>457632</v>
       </c>
-      <c r="G75" s="4" t="n">
-        <v>5480</v>
-      </c>
-      <c r="H75" s="4" t="n">
-        <v>80</v>
+      <c r="G75" t="n">
+        <v>27400</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -7760,33 +7760,33 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="n">
+      <c r="A96" s="2" t="n">
         <v>93</v>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>Warhammer 40,000: Rogue Trader</t>
         </is>
       </c>
-      <c r="C96" s="4" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Strategy</t>
         </is>
       </c>
-      <c r="D96" s="4" t="n">
+      <c r="D96" s="2" t="n">
         <v>3582</v>
       </c>
-      <c r="E96" s="4" t="n">
+      <c r="E96" s="2" t="n">
         <v>85.59999999999999</v>
       </c>
-      <c r="F96" s="4" t="n">
+      <c r="F96" s="2" t="n">
         <v>30805</v>
       </c>
-      <c r="G96" s="4" t="n">
-        <v>21200</v>
-      </c>
-      <c r="H96" s="4" t="n">
-        <v>60</v>
+      <c r="G96" s="2" t="n">
+        <v>53000</v>
+      </c>
+      <c r="H96" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-28</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-29</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-28</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-29</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-28</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-30
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-29</t>
+          <t>Steam 인기 차트 — 2026-05-30</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-29</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-30</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-29</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-30</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-29</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-05-31
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2415,10 +2415,10 @@
         <v>643681</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>5500</v>
+        <v>3300</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>5500</v>
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-30</t>
+          <t>Steam 인기 차트 — 2026-05-31</t>
         </is>
       </c>
     </row>
@@ -6260,33 +6260,33 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Among Us</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Casual</t>
         </is>
       </c>
-      <c r="D46" s="2" t="n">
+      <c r="D46" s="4" t="n">
         <v>3832</v>
       </c>
-      <c r="E46" s="2" t="n">
+      <c r="E46" s="4" t="n">
         <v>91.90000000000001</v>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="F46" s="4" t="n">
         <v>700785</v>
       </c>
-      <c r="G46" s="2" t="n">
-        <v>5500</v>
-      </c>
-      <c r="H46" s="2" t="n">
-        <v>0</v>
+      <c r="G46" s="4" t="n">
+        <v>3300</v>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="47">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-30</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-31</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-30</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-31</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-30</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-01
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-31</t>
+          <t>Steam 인기 차트 — 2026-06-01</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-05-31</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-01</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-05-31</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-01</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-05-31</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-02
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4791,10 +4791,10 @@
         <v>225479</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>42000</v>
+        <v>29400</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>42000</v>
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-01</t>
+          <t>Steam 인기 차트 — 2026-06-02</t>
         </is>
       </c>
     </row>
@@ -7880,33 +7880,33 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="4" t="n">
         <v>97</v>
       </c>
-      <c r="B100" s="2" t="inlineStr">
+      <c r="B100" s="4" t="inlineStr">
         <is>
           <t>Satisfactory</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
+      <c r="C100" s="4" t="inlineStr">
         <is>
           <t>Adventure, Indie, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D100" s="2" t="n">
+      <c r="D100" s="4" t="n">
         <v>12596</v>
       </c>
-      <c r="E100" s="2" t="n">
+      <c r="E100" s="4" t="n">
         <v>97.2</v>
       </c>
-      <c r="F100" s="2" t="n">
+      <c r="F100" s="4" t="n">
         <v>232064</v>
       </c>
-      <c r="G100" s="2" t="n">
-        <v>42000</v>
-      </c>
-      <c r="H100" s="2" t="n">
-        <v>0</v>
+      <c r="G100" s="4" t="n">
+        <v>29400</v>
+      </c>
+      <c r="H100" s="4" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="101">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-01</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-02</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-01</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-02</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-01</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-03
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1757,10 +1757,10 @@
         <v>612177</v>
       </c>
       <c r="J29" t="n">
-        <v>10890</v>
+        <v>16500</v>
       </c>
       <c r="K29" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
         <v>16500</v>
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2811,10 +2811,10 @@
         <v>143086</v>
       </c>
       <c r="J53" t="n">
-        <v>7870</v>
+        <v>10500</v>
       </c>
       <c r="K53" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="L53" t="n">
         <v>10500</v>
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-02</t>
+          <t>Steam 인기 차트 — 2026-06-03</t>
         </is>
       </c>
     </row>
@@ -5812,33 +5812,33 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="A31" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>ARK: Survival Evolved</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Massively Multiplayer, RPG</t>
         </is>
       </c>
-      <c r="D31" s="4" t="n">
+      <c r="D31" t="n">
         <v>22170</v>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="E31" t="n">
         <v>83.8</v>
       </c>
-      <c r="F31" s="4" t="n">
+      <c r="F31" t="n">
         <v>730170</v>
       </c>
-      <c r="G31" s="4" t="n">
-        <v>10890</v>
-      </c>
-      <c r="H31" s="4" t="n">
-        <v>34</v>
+      <c r="G31" t="n">
+        <v>16500</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -6530,33 +6530,33 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="n">
+      <c r="A55" t="n">
         <v>52</v>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>Half-Life</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D55" s="4" t="n">
+      <c r="D55" t="n">
         <v>634</v>
       </c>
-      <c r="E55" s="4" t="n">
+      <c r="E55" t="n">
         <v>96.5</v>
       </c>
-      <c r="F55" s="4" t="n">
+      <c r="F55" t="n">
         <v>148221</v>
       </c>
-      <c r="G55" s="4" t="n">
-        <v>7870</v>
-      </c>
-      <c r="H55" s="4" t="n">
-        <v>25</v>
+      <c r="G55" t="n">
+        <v>10500</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-02</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-03</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-02</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-03</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-02</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-04
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4263,10 +4263,10 @@
         <v>93489</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>5400</v>
+        <v>27000</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>27000</v>
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-03</t>
+          <t>Steam 인기 차트 — 2026-06-04</t>
         </is>
       </c>
     </row>
@@ -7520,33 +7520,33 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="4" t="n">
+      <c r="A88" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="B88" s="4" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>Grim Dawn</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D88" s="4" t="n">
+      <c r="D88" s="2" t="n">
         <v>2376</v>
       </c>
-      <c r="E88" s="4" t="n">
+      <c r="E88" s="2" t="n">
         <v>93.7</v>
       </c>
-      <c r="F88" s="4" t="n">
+      <c r="F88" s="2" t="n">
         <v>99730</v>
       </c>
-      <c r="G88" s="4" t="n">
-        <v>5400</v>
-      </c>
-      <c r="H88" s="4" t="n">
-        <v>80</v>
+      <c r="G88" s="2" t="n">
+        <v>27000</v>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="89">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-03</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-04</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-03</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-04</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-03</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-05
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1143,10 +1143,10 @@
         <v>127273</v>
       </c>
       <c r="J15" t="n">
-        <v>84800</v>
+        <v>35620</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="L15" t="n">
         <v>84800</v>
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1845,10 +1845,10 @@
         <v>599805</v>
       </c>
       <c r="J31" t="n">
-        <v>20500</v>
+        <v>4510</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="L31" t="n">
         <v>20500</v>
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2855,10 +2855,10 @@
         <v>434239</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>36800</v>
+        <v>9570</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>36800</v>
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4219,10 +4219,10 @@
         <v>222495</v>
       </c>
       <c r="J85" t="n">
-        <v>32000</v>
+        <v>9600</v>
       </c>
       <c r="K85" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L85" t="n">
         <v>32000</v>
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4879,10 +4879,10 @@
         <v>293127</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>8580</v>
+        <v>26000</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>26000</v>
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-04</t>
+          <t>Steam 인기 차트 — 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -5394,33 +5394,33 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Monster Hunter Wilds</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, RPG</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="4" t="n">
         <v>12494</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="4" t="n">
         <v>58.3</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="4" t="n">
         <v>218415</v>
       </c>
-      <c r="G17" t="n">
-        <v>84800</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
+      <c r="G17" s="4" t="n">
+        <v>35620</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>58</v>
       </c>
     </row>
     <row r="18">
@@ -5872,33 +5872,33 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>The Forest</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" s="4" t="n">
         <v>2892</v>
       </c>
-      <c r="E33" t="n">
+      <c r="E33" s="4" t="n">
         <v>95.5</v>
       </c>
-      <c r="F33" t="n">
+      <c r="F33" s="4" t="n">
         <v>627791</v>
       </c>
-      <c r="G33" t="n">
-        <v>20500</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
+      <c r="G33" s="4" t="n">
+        <v>4510</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>78</v>
       </c>
     </row>
     <row r="34">
@@ -6560,33 +6560,33 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>Monster Hunter: World</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D56" s="2" t="n">
+      <c r="D56" s="4" t="n">
         <v>11923</v>
       </c>
-      <c r="E56" s="2" t="n">
+      <c r="E56" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="F56" s="2" t="n">
+      <c r="F56" s="4" t="n">
         <v>493390</v>
       </c>
-      <c r="G56" s="2" t="n">
-        <v>36800</v>
-      </c>
-      <c r="H56" s="2" t="n">
-        <v>0</v>
+      <c r="G56" s="4" t="n">
+        <v>9570</v>
+      </c>
+      <c r="H56" s="4" t="n">
+        <v>74</v>
       </c>
     </row>
     <row r="57">
@@ -7490,33 +7490,33 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="n">
+      <c r="A87" s="4" t="n">
         <v>84</v>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>Sons Of The Forest</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D87" t="n">
+      <c r="D87" s="4" t="n">
         <v>4450</v>
       </c>
-      <c r="E87" t="n">
+      <c r="E87" s="4" t="n">
         <v>87.8</v>
       </c>
-      <c r="F87" t="n">
+      <c r="F87" s="4" t="n">
         <v>253546</v>
       </c>
-      <c r="G87" t="n">
-        <v>32000</v>
-      </c>
-      <c r="H87" t="n">
-        <v>0</v>
+      <c r="G87" s="4" t="n">
+        <v>9600</v>
+      </c>
+      <c r="H87" s="4" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="88">
@@ -7940,33 +7940,33 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="4" t="n">
+      <c r="A102" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="B102" s="4" t="inlineStr">
+      <c r="B102" s="2" t="inlineStr">
         <is>
           <t>Risk of Rain 2</t>
         </is>
       </c>
-      <c r="C102" s="4" t="inlineStr">
+      <c r="C102" s="2" t="inlineStr">
         <is>
           <t>Action, Indie</t>
         </is>
       </c>
-      <c r="D102" s="4" t="n">
+      <c r="D102" s="2" t="n">
         <v>7902</v>
       </c>
-      <c r="E102" s="4" t="n">
+      <c r="E102" s="2" t="n">
         <v>93.5</v>
       </c>
-      <c r="F102" s="4" t="n">
+      <c r="F102" s="2" t="n">
         <v>313577</v>
       </c>
-      <c r="G102" s="4" t="n">
-        <v>8580</v>
-      </c>
-      <c r="H102" s="4" t="n">
-        <v>67</v>
+      <c r="G102" s="2" t="n">
+        <v>26000</v>
+      </c>
+      <c r="H102" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-04</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-04</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-04</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-06
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-05</t>
+          <t>Steam 인기 차트 — 2026-06-06</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-05</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-06</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-05</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-06</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-05</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-07
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-06</t>
+          <t>Steam 인기 차트 — 2026-06-07</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-06</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-07</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-06</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-07</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-06</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-08
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-07</t>
+          <t>Steam 인기 차트 — 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-07</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-07</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-07</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-09
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1537,10 +1537,10 @@
         <v>1122546</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>10500</v>
+        <v>5250</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>10500</v>
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2283,10 +2283,10 @@
         <v>289966</v>
       </c>
       <c r="J41" t="n">
-        <v>11970</v>
+        <v>79800</v>
       </c>
       <c r="K41" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="L41" t="n">
         <v>79800</v>
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -3999,10 +3999,10 @@
         <v>181110</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>36700</v>
+        <v>14680</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>36700</v>
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4087,10 +4087,10 @@
         <v>266</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>16500</v>
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4791,10 +4791,10 @@
         <v>225479</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>29400</v>
+        <v>42000</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>42000</v>
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-08</t>
+          <t>Steam 인기 차트 — 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -5662,33 +5662,33 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Garry's Mod</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n">
+      <c r="D26" s="4" t="n">
         <v>18400</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="4" t="n">
         <v>96.8</v>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="F26" s="4" t="n">
         <v>1159707</v>
       </c>
-      <c r="G26" s="2" t="n">
-        <v>10500</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>0</v>
+      <c r="G26" s="4" t="n">
+        <v>5250</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="27">
@@ -6170,33 +6170,33 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n">
+      <c r="A43" t="n">
         <v>40</v>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Hogwarts Legacy</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Action, Adventure, RPG</t>
         </is>
       </c>
-      <c r="D43" s="4" t="n">
+      <c r="D43" t="n">
         <v>5716</v>
       </c>
-      <c r="E43" s="4" t="n">
+      <c r="E43" t="n">
         <v>90.2</v>
       </c>
-      <c r="F43" s="4" t="n">
+      <c r="F43" t="n">
         <v>321395</v>
       </c>
-      <c r="G43" s="4" t="n">
-        <v>11970</v>
-      </c>
-      <c r="H43" s="4" t="n">
-        <v>85</v>
+      <c r="G43" t="n">
+        <v>79800</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -7340,33 +7340,33 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="4" t="n">
         <v>79</v>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B82" s="4" t="inlineStr">
         <is>
           <t>Hunt: Showdown 1896</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="C82" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D82" s="2" t="n">
+      <c r="D82" s="4" t="n">
         <v>6300</v>
       </c>
-      <c r="E82" s="2" t="n">
+      <c r="E82" s="4" t="n">
         <v>73</v>
       </c>
-      <c r="F82" s="2" t="n">
+      <c r="F82" s="4" t="n">
         <v>248220</v>
       </c>
-      <c r="G82" s="2" t="n">
-        <v>36700</v>
-      </c>
-      <c r="H82" s="2" t="n">
-        <v>0</v>
+      <c r="G82" s="4" t="n">
+        <v>14680</v>
+      </c>
+      <c r="H82" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="83">
@@ -7400,33 +7400,33 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="4" t="n">
         <v>81</v>
       </c>
-      <c r="B84" s="2" t="inlineStr">
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>CyberCorp</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
+      <c r="C84" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D84" s="2" t="n">
+      <c r="D84" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E84" s="2" t="n">
+      <c r="E84" s="4" t="n">
         <v>82.59999999999999</v>
       </c>
-      <c r="F84" s="2" t="n">
+      <c r="F84" s="4" t="n">
         <v>322</v>
       </c>
-      <c r="G84" s="2" t="n">
-        <v>16500</v>
-      </c>
-      <c r="H84" s="2" t="n">
-        <v>0</v>
+      <c r="G84" s="4" t="n">
+        <v>9900</v>
+      </c>
+      <c r="H84" s="4" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="85">
@@ -7880,33 +7880,33 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="4" t="n">
+      <c r="A100" s="2" t="n">
         <v>97</v>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B100" s="2" t="inlineStr">
         <is>
           <t>Satisfactory</t>
         </is>
       </c>
-      <c r="C100" s="4" t="inlineStr">
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>Adventure, Indie, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D100" s="4" t="n">
+      <c r="D100" s="2" t="n">
         <v>12596</v>
       </c>
-      <c r="E100" s="4" t="n">
+      <c r="E100" s="2" t="n">
         <v>97.2</v>
       </c>
-      <c r="F100" s="4" t="n">
+      <c r="F100" s="2" t="n">
         <v>232064</v>
       </c>
-      <c r="G100" s="4" t="n">
-        <v>29400</v>
-      </c>
-      <c r="H100" s="4" t="n">
-        <v>30</v>
+      <c r="G100" s="2" t="n">
+        <v>42000</v>
+      </c>
+      <c r="H100" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-08</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-08</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-08</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-10
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -705,10 +705,10 @@
         <v>358266</v>
       </c>
       <c r="J5" t="n">
-        <v>24000</v>
+        <v>32000</v>
       </c>
       <c r="K5" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>32000</v>
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-09</t>
+          <t>Steam 인기 차트 — 2026-06-10</t>
         </is>
       </c>
     </row>
@@ -5096,33 +5096,33 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Palworld</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Early Access</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" t="n">
         <v>18028</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" t="n">
         <v>94.09999999999999</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" t="n">
         <v>380709</v>
       </c>
-      <c r="G7" s="4" t="n">
-        <v>24000</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>25</v>
+      <c r="G7" t="n">
+        <v>32000</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-09</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-10</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-09</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-10</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-09</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-11
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4703,10 +4703,10 @@
         <v>179154</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>10700</v>
+        <v>7490</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>10700</v>
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-10</t>
+          <t>Steam 인기 차트 — 2026-06-11</t>
         </is>
       </c>
     </row>
@@ -7820,33 +7820,33 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="4" t="n">
         <v>95</v>
       </c>
-      <c r="B98" s="2" t="inlineStr">
+      <c r="B98" s="4" t="inlineStr">
         <is>
           <t>R.E.P.O.</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr">
+      <c r="C98" s="4" t="inlineStr">
         <is>
           <t>Action, Early Access</t>
         </is>
       </c>
-      <c r="D98" s="2" t="n">
+      <c r="D98" s="4" t="n">
         <v>32349</v>
       </c>
-      <c r="E98" s="2" t="n">
+      <c r="E98" s="4" t="n">
         <v>96.5</v>
       </c>
-      <c r="F98" s="2" t="n">
+      <c r="F98" s="4" t="n">
         <v>185642</v>
       </c>
-      <c r="G98" s="2" t="n">
-        <v>10700</v>
-      </c>
-      <c r="H98" s="2" t="n">
-        <v>0</v>
+      <c r="G98" s="4" t="n">
+        <v>7490</v>
+      </c>
+      <c r="H98" s="4" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="99">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-10</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-11</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-10</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-11</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-10</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-12
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1669,10 +1669,10 @@
         <v>1071135</v>
       </c>
       <c r="J27" t="n">
-        <v>42000</v>
+        <v>21000</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L27" t="n">
         <v>42000</v>
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1845,10 +1845,10 @@
         <v>599805</v>
       </c>
       <c r="J31" t="n">
-        <v>4510</v>
+        <v>20500</v>
       </c>
       <c r="K31" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
         <v>20500</v>
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2503,10 +2503,10 @@
         <v>272900</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>21000</v>
+        <v>5250</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>21000</v>
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3647,10 +3647,10 @@
         <v>475393</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>15500</v>
+        <v>1550</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>15500</v>
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4219,10 +4219,10 @@
         <v>222495</v>
       </c>
       <c r="J85" t="n">
-        <v>9600</v>
+        <v>32000</v>
       </c>
       <c r="K85" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L85" t="n">
         <v>32000</v>
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4307,10 +4307,10 @@
         <v>256362</v>
       </c>
       <c r="J87" t="n">
-        <v>33000</v>
+        <v>9900</v>
       </c>
       <c r="K87" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L87" t="n">
         <v>33000</v>
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-11</t>
+          <t>Steam 인기 차트 — 2026-06-12</t>
         </is>
       </c>
     </row>
@@ -5752,33 +5752,33 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Rust</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Massively Multiplayer, RPG</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="4" t="n">
         <v>143870</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="4" t="n">
         <v>87.2</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" s="4" t="n">
         <v>1227784</v>
       </c>
-      <c r="G29" t="n">
-        <v>42000</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0</v>
+      <c r="G29" s="4" t="n">
+        <v>21000</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="30">
@@ -5872,33 +5872,33 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n">
+      <c r="A33" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>The Forest</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D33" t="n">
         <v>2892</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E33" t="n">
         <v>95.5</v>
       </c>
-      <c r="F33" s="4" t="n">
+      <c r="F33" t="n">
         <v>627791</v>
       </c>
-      <c r="G33" s="4" t="n">
-        <v>4510</v>
-      </c>
-      <c r="H33" s="4" t="n">
-        <v>78</v>
+      <c r="G33" t="n">
+        <v>20500</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -6320,33 +6320,33 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>Borderlands 2</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D48" s="2" t="n">
+      <c r="D48" s="4" t="n">
         <v>8551</v>
       </c>
-      <c r="E48" s="2" t="n">
+      <c r="E48" s="4" t="n">
         <v>92.40000000000001</v>
       </c>
-      <c r="F48" s="2" t="n">
+      <c r="F48" s="4" t="n">
         <v>295218</v>
       </c>
-      <c r="G48" s="2" t="n">
-        <v>21000</v>
-      </c>
-      <c r="H48" s="2" t="n">
-        <v>0</v>
+      <c r="G48" s="4" t="n">
+        <v>5250</v>
+      </c>
+      <c r="H48" s="4" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="49">
@@ -7100,33 +7100,33 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>Don't Starve Together</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D74" s="2" t="n">
+      <c r="D74" s="4" t="n">
         <v>30542</v>
       </c>
-      <c r="E74" s="2" t="n">
+      <c r="E74" s="4" t="n">
         <v>95.3</v>
       </c>
-      <c r="F74" s="2" t="n">
+      <c r="F74" s="4" t="n">
         <v>499061</v>
       </c>
-      <c r="G74" s="2" t="n">
-        <v>15500</v>
-      </c>
-      <c r="H74" s="2" t="n">
-        <v>0</v>
+      <c r="G74" s="4" t="n">
+        <v>1550</v>
+      </c>
+      <c r="H74" s="4" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="75">
@@ -7490,33 +7490,33 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="4" t="n">
+      <c r="A87" t="n">
         <v>84</v>
       </c>
-      <c r="B87" s="4" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>Sons Of The Forest</t>
         </is>
       </c>
-      <c r="C87" s="4" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D87" s="4" t="n">
+      <c r="D87" t="n">
         <v>4450</v>
       </c>
-      <c r="E87" s="4" t="n">
+      <c r="E87" t="n">
         <v>87.8</v>
       </c>
-      <c r="F87" s="4" t="n">
+      <c r="F87" t="n">
         <v>253546</v>
       </c>
-      <c r="G87" s="4" t="n">
-        <v>9600</v>
-      </c>
-      <c r="H87" s="4" t="n">
-        <v>70</v>
+      <c r="G87" t="n">
+        <v>32000</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -7550,33 +7550,33 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="n">
+      <c r="A89" s="4" t="n">
         <v>86</v>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="4" t="inlineStr">
         <is>
           <t>Cities: Skylines</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="4" t="inlineStr">
         <is>
           <t>Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D89" t="n">
+      <c r="D89" s="4" t="n">
         <v>8842</v>
       </c>
-      <c r="E89" t="n">
+      <c r="E89" s="4" t="n">
         <v>93</v>
       </c>
-      <c r="F89" t="n">
+      <c r="F89" s="4" t="n">
         <v>275770</v>
       </c>
-      <c r="G89" t="n">
-        <v>33000</v>
-      </c>
-      <c r="H89" t="n">
-        <v>0</v>
+      <c r="G89" s="4" t="n">
+        <v>9900</v>
+      </c>
+      <c r="H89" s="4" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="90">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-11</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-12</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-11</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-12</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-11</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-13
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-12</t>
+          <t>Steam 인기 차트 — 2026-06-13</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-12</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-13</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-12</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-13</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-12</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-14
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2415,10 +2415,10 @@
         <v>643681</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>3300</v>
+        <v>5500</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>5500</v>
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-13</t>
+          <t>Steam 인기 차트 — 2026-06-14</t>
         </is>
       </c>
     </row>
@@ -6260,33 +6260,33 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="n">
+      <c r="A46" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Among Us</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Casual</t>
         </is>
       </c>
-      <c r="D46" s="4" t="n">
+      <c r="D46" s="2" t="n">
         <v>3832</v>
       </c>
-      <c r="E46" s="4" t="n">
+      <c r="E46" s="2" t="n">
         <v>91.90000000000001</v>
       </c>
-      <c r="F46" s="4" t="n">
+      <c r="F46" s="2" t="n">
         <v>700785</v>
       </c>
-      <c r="G46" s="4" t="n">
-        <v>3300</v>
-      </c>
-      <c r="H46" s="4" t="n">
-        <v>40</v>
+      <c r="G46" s="2" t="n">
+        <v>5500</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-13</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-14</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-13</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-14</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-13</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-15
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-14</t>
+          <t>Steam 인기 차트 — 2026-06-15</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-14</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-15</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-14</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-15</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-14</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-16
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4395,10 +4395,10 @@
         <v>195724</v>
       </c>
       <c r="J89" t="n">
-        <v>32000</v>
+        <v>8000</v>
       </c>
       <c r="K89" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="L89" t="n">
         <v>32000</v>
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4483,10 +4483,10 @@
         <v>304053</v>
       </c>
       <c r="J91" t="n">
-        <v>65000</v>
+        <v>6500</v>
       </c>
       <c r="K91" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L91" t="n">
         <v>65000</v>
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-15</t>
+          <t>Steam 인기 차트 — 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -7610,33 +7610,33 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="n">
+      <c r="A91" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="4" t="inlineStr">
         <is>
           <t>Sid Meier's Civilization® V</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="4" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="D91" t="n">
+      <c r="D91" s="4" t="n">
         <v>12206</v>
       </c>
-      <c r="E91" t="n">
+      <c r="E91" s="4" t="n">
         <v>95.8</v>
       </c>
-      <c r="F91" t="n">
+      <c r="F91" s="4" t="n">
         <v>204265</v>
       </c>
-      <c r="G91" t="n">
-        <v>32000</v>
-      </c>
-      <c r="H91" t="n">
-        <v>0</v>
+      <c r="G91" s="4" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H91" s="4" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="92">
@@ -7670,33 +7670,33 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="n">
+      <c r="A93" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>Sid Meier’s Civilization® VI</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="D93" t="n">
+      <c r="D93" s="4" t="n">
         <v>25420</v>
       </c>
-      <c r="E93" t="n">
+      <c r="E93" s="4" t="n">
         <v>86.90000000000001</v>
       </c>
-      <c r="F93" t="n">
+      <c r="F93" s="4" t="n">
         <v>349920</v>
       </c>
-      <c r="G93" t="n">
-        <v>65000</v>
-      </c>
-      <c r="H93" t="n">
-        <v>0</v>
+      <c r="G93" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="H93" s="4" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="94">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-15</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-15</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-15</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-17
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2239,10 +2239,10 @@
         <v>630223</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>21500</v>
+        <v>8600</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>21500</v>
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-16</t>
+          <t>Steam 인기 차트 — 2026-06-17</t>
         </is>
       </c>
     </row>
@@ -6140,33 +6140,33 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>Dead by Daylight</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D42" s="2" t="n">
+      <c r="D42" s="4" t="n">
         <v>44886</v>
       </c>
-      <c r="E42" s="2" t="n">
+      <c r="E42" s="4" t="n">
         <v>79.09999999999999</v>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="F42" s="4" t="n">
         <v>797216</v>
       </c>
-      <c r="G42" s="2" t="n">
-        <v>21500</v>
-      </c>
-      <c r="H42" s="2" t="n">
-        <v>0</v>
+      <c r="G42" s="4" t="n">
+        <v>8600</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="43">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-16</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-17</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-16</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-17</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-16</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-18
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2107,10 +2107,10 @@
         <v>88027</v>
       </c>
       <c r="J37" t="n">
-        <v>37500</v>
+        <v>30000</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L37" t="n">
         <v>37500</v>
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-17</t>
+          <t>Steam 인기 차트 — 2026-06-18</t>
         </is>
       </c>
     </row>
@@ -6050,33 +6050,33 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Last Epoch</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D39" s="4" t="n">
         <v>5831</v>
       </c>
-      <c r="E39" t="n">
+      <c r="E39" s="4" t="n">
         <v>79.59999999999999</v>
       </c>
-      <c r="F39" t="n">
+      <c r="F39" s="4" t="n">
         <v>110623</v>
       </c>
-      <c r="G39" t="n">
-        <v>37500</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0</v>
+      <c r="G39" s="4" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="40">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-17</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-18</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-17</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-18</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-17</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-19
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1143,10 +1143,10 @@
         <v>127273</v>
       </c>
       <c r="J15" t="n">
-        <v>35620</v>
+        <v>84800</v>
       </c>
       <c r="K15" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>84800</v>
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2195,10 +2195,10 @@
         <v>713071</v>
       </c>
       <c r="J39" t="n">
-        <v>66000</v>
+        <v>19800</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L39" t="n">
         <v>66000</v>
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2371,10 +2371,10 @@
         <v>802993</v>
       </c>
       <c r="J43" t="n">
-        <v>34800</v>
+        <v>3480</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L43" t="n">
         <v>34800</v>
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2855,10 +2855,10 @@
         <v>434239</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>9570</v>
+        <v>36800</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>36800</v>
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3119,10 +3119,10 @@
         <v>139186</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>66000</v>
+        <v>3300</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>66000</v>
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3735,10 +3735,10 @@
         <v>202253</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>20500</v>
+        <v>6150</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>20500</v>
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4175,10 +4175,10 @@
         <v>256128</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>36000</v>
+        <v>10800</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>36000</v>
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4659,10 +4659,10 @@
         <v>177352</v>
       </c>
       <c r="J95" t="n">
-        <v>55000</v>
+        <v>2750</v>
       </c>
       <c r="K95" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="L95" t="n">
         <v>55000</v>
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4747,10 +4747,10 @@
         <v>330349</v>
       </c>
       <c r="J97" t="n">
-        <v>59000</v>
+        <v>26550</v>
       </c>
       <c r="K97" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="L97" t="n">
         <v>59000</v>
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-18</t>
+          <t>Steam 인기 차트 — 2026-06-19</t>
         </is>
       </c>
     </row>
@@ -5394,33 +5394,33 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n">
+      <c r="A17" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Monster Hunter Wilds</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Action, Adventure, RPG</t>
         </is>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" t="n">
         <v>12494</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" t="n">
         <v>58.3</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="F17" t="n">
         <v>218415</v>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>35620</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>58</v>
+      <c r="G17" t="n">
+        <v>84800</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -6110,33 +6110,33 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>Cyberpunk 2077</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>RPG</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="D41" s="4" t="n">
         <v>22265</v>
       </c>
-      <c r="E41" t="n">
+      <c r="E41" s="4" t="n">
         <v>84.40000000000001</v>
       </c>
-      <c r="F41" t="n">
+      <c r="F41" s="4" t="n">
         <v>844921</v>
       </c>
-      <c r="G41" t="n">
-        <v>66000</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0</v>
+      <c r="G41" s="4" t="n">
+        <v>19800</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="42">
@@ -6230,33 +6230,33 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>The Witcher 3: Wild Hunt</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>RPG</t>
         </is>
       </c>
-      <c r="D45" t="n">
+      <c r="D45" s="4" t="n">
         <v>15893</v>
       </c>
-      <c r="E45" t="n">
+      <c r="E45" s="4" t="n">
         <v>96.09999999999999</v>
       </c>
-      <c r="F45" t="n">
+      <c r="F45" s="4" t="n">
         <v>835349</v>
       </c>
-      <c r="G45" t="n">
-        <v>34800</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0</v>
+      <c r="G45" s="4" t="n">
+        <v>3480</v>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="46">
@@ -6560,33 +6560,33 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="n">
+      <c r="A56" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Monster Hunter: World</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D56" s="4" t="n">
+      <c r="D56" s="2" t="n">
         <v>11923</v>
       </c>
-      <c r="E56" s="4" t="n">
+      <c r="E56" s="2" t="n">
         <v>88</v>
       </c>
-      <c r="F56" s="4" t="n">
+      <c r="F56" s="2" t="n">
         <v>493390</v>
       </c>
-      <c r="G56" s="4" t="n">
-        <v>9570</v>
-      </c>
-      <c r="H56" s="4" t="n">
-        <v>74</v>
+      <c r="G56" s="2" t="n">
+        <v>36800</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -6740,33 +6740,33 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>Battlefield™ 2042</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Casual</t>
         </is>
       </c>
-      <c r="D62" s="2" t="n">
+      <c r="D62" s="4" t="n">
         <v>2774</v>
       </c>
-      <c r="E62" s="2" t="n">
+      <c r="E62" s="4" t="n">
         <v>46.7</v>
       </c>
-      <c r="F62" s="2" t="n">
+      <c r="F62" s="4" t="n">
         <v>297774</v>
       </c>
-      <c r="G62" s="2" t="n">
-        <v>66000</v>
-      </c>
-      <c r="H62" s="2" t="n">
-        <v>0</v>
+      <c r="G62" s="4" t="n">
+        <v>3300</v>
+      </c>
+      <c r="H62" s="4" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="63">
@@ -7160,33 +7160,33 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="4" t="n">
         <v>73</v>
       </c>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="B76" s="4" t="inlineStr">
         <is>
           <t>Human Fall Flat</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
+      <c r="C76" s="4" t="inlineStr">
         <is>
           <t>Adventure, Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D76" s="2" t="n">
+      <c r="D76" s="4" t="n">
         <v>950</v>
       </c>
-      <c r="E76" s="2" t="n">
+      <c r="E76" s="4" t="n">
         <v>94.7</v>
       </c>
-      <c r="F76" s="2" t="n">
+      <c r="F76" s="4" t="n">
         <v>213640</v>
       </c>
-      <c r="G76" s="2" t="n">
-        <v>20500</v>
-      </c>
-      <c r="H76" s="2" t="n">
-        <v>0</v>
+      <c r="G76" s="4" t="n">
+        <v>6150</v>
+      </c>
+      <c r="H76" s="4" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="77">
@@ -7460,33 +7460,33 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="4" t="n">
         <v>83</v>
       </c>
-      <c r="B86" s="2" t="inlineStr">
+      <c r="B86" s="4" t="inlineStr">
         <is>
           <t>Arma 3</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr">
+      <c r="C86" s="4" t="inlineStr">
         <is>
           <t>Action, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D86" s="2" t="n">
+      <c r="D86" s="4" t="n">
         <v>7181</v>
       </c>
-      <c r="E86" s="2" t="n">
+      <c r="E86" s="4" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="F86" s="2" t="n">
+      <c r="F86" s="4" t="n">
         <v>283264</v>
       </c>
-      <c r="G86" s="2" t="n">
-        <v>36000</v>
-      </c>
-      <c r="H86" s="2" t="n">
-        <v>0</v>
+      <c r="G86" s="4" t="n">
+        <v>10800</v>
+      </c>
+      <c r="H86" s="4" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="87">
@@ -7790,33 +7790,33 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="n">
+      <c r="A97" s="4" t="n">
         <v>94</v>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B97" s="4" t="inlineStr">
         <is>
           <t>Battlefield™ V</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C97" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D97" t="n">
+      <c r="D97" s="4" t="n">
         <v>6327</v>
       </c>
-      <c r="E97" t="n">
+      <c r="E97" s="4" t="n">
         <v>70.90000000000001</v>
       </c>
-      <c r="F97" t="n">
+      <c r="F97" s="4" t="n">
         <v>250288</v>
       </c>
-      <c r="G97" t="n">
-        <v>55000</v>
-      </c>
-      <c r="H97" t="n">
-        <v>0</v>
+      <c r="G97" s="4" t="n">
+        <v>2750</v>
+      </c>
+      <c r="H97" s="4" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="98">
@@ -7850,33 +7850,33 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="n">
+      <c r="A99" s="4" t="n">
         <v>96</v>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B99" s="4" t="inlineStr">
         <is>
           <t>DayZ</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C99" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Massively Multiplayer</t>
         </is>
       </c>
-      <c r="D99" t="n">
+      <c r="D99" s="4" t="n">
         <v>37066</v>
       </c>
-      <c r="E99" t="n">
+      <c r="E99" s="4" t="n">
         <v>76.8</v>
       </c>
-      <c r="F99" t="n">
+      <c r="F99" s="4" t="n">
         <v>430252</v>
       </c>
-      <c r="G99" t="n">
-        <v>59000</v>
-      </c>
-      <c r="H99" t="n">
-        <v>0</v>
+      <c r="G99" s="4" t="n">
+        <v>26550</v>
+      </c>
+      <c r="H99" s="4" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="100">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-18</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-19</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-18</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-19</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-18</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-20
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-19</t>
+          <t>Steam 인기 차트 — 2026-06-20</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-19</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-20</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-19</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-20</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-19</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-21
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-20</t>
+          <t>Steam 인기 차트 — 2026-06-21</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-20</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-21</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-20</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-21</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-20</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-22
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-21</t>
+          <t>Steam 인기 차트 — 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-21</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-21</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-21</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-23
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1537,10 +1537,10 @@
         <v>1122546</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>5250</v>
+        <v>10500</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>10500</v>
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -3999,10 +3999,10 @@
         <v>181110</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>14680</v>
+        <v>36700</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>36700</v>
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4087,10 +4087,10 @@
         <v>266</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>9900</v>
+        <v>16500</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>16500</v>
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-22</t>
+          <t>Steam 인기 차트 — 2026-06-23</t>
         </is>
       </c>
     </row>
@@ -5662,33 +5662,33 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Garry's Mod</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="D26" s="2" t="n">
         <v>18400</v>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="E26" s="2" t="n">
         <v>96.8</v>
       </c>
-      <c r="F26" s="4" t="n">
+      <c r="F26" s="2" t="n">
         <v>1159707</v>
       </c>
-      <c r="G26" s="4" t="n">
-        <v>5250</v>
-      </c>
-      <c r="H26" s="4" t="n">
-        <v>50</v>
+      <c r="G26" s="2" t="n">
+        <v>10500</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -7340,33 +7340,33 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="4" t="n">
+      <c r="A82" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="B82" s="4" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>Hunt: Showdown 1896</t>
         </is>
       </c>
-      <c r="C82" s="4" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D82" s="4" t="n">
+      <c r="D82" s="2" t="n">
         <v>6300</v>
       </c>
-      <c r="E82" s="4" t="n">
+      <c r="E82" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="F82" s="4" t="n">
+      <c r="F82" s="2" t="n">
         <v>248220</v>
       </c>
-      <c r="G82" s="4" t="n">
-        <v>14680</v>
-      </c>
-      <c r="H82" s="4" t="n">
-        <v>60</v>
+      <c r="G82" s="2" t="n">
+        <v>36700</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -7400,33 +7400,33 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="n">
+      <c r="A84" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="B84" s="4" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>CyberCorp</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D84" s="4" t="n">
+      <c r="D84" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E84" s="4" t="n">
+      <c r="E84" s="2" t="n">
         <v>82.59999999999999</v>
       </c>
-      <c r="F84" s="4" t="n">
+      <c r="F84" s="2" t="n">
         <v>322</v>
       </c>
-      <c r="G84" s="4" t="n">
-        <v>9900</v>
-      </c>
-      <c r="H84" s="4" t="n">
-        <v>40</v>
+      <c r="G84" s="2" t="n">
+        <v>16500</v>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-22</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-23</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-22</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-23</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-22</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-24
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-23</t>
+          <t>Steam 인기 차트 — 2026-06-24</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-23</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-24</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-23</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-24</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-23</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-25
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4703,10 +4703,10 @@
         <v>179154</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>7490</v>
+        <v>10700</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>10700</v>
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-24</t>
+          <t>Steam 인기 차트 — 2026-06-25</t>
         </is>
       </c>
     </row>
@@ -7820,33 +7820,33 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="4" t="n">
+      <c r="A98" s="2" t="n">
         <v>95</v>
       </c>
-      <c r="B98" s="4" t="inlineStr">
+      <c r="B98" s="2" t="inlineStr">
         <is>
           <t>R.E.P.O.</t>
         </is>
       </c>
-      <c r="C98" s="4" t="inlineStr">
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>Action, Early Access</t>
         </is>
       </c>
-      <c r="D98" s="4" t="n">
+      <c r="D98" s="2" t="n">
         <v>32349</v>
       </c>
-      <c r="E98" s="4" t="n">
+      <c r="E98" s="2" t="n">
         <v>96.5</v>
       </c>
-      <c r="F98" s="4" t="n">
+      <c r="F98" s="2" t="n">
         <v>185642</v>
       </c>
-      <c r="G98" s="4" t="n">
-        <v>7490</v>
-      </c>
-      <c r="H98" s="4" t="n">
-        <v>30</v>
+      <c r="G98" s="2" t="n">
+        <v>10700</v>
+      </c>
+      <c r="H98" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-24</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-25</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-24</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-25</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-24</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-26
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -705,10 +705,10 @@
         <v>358266</v>
       </c>
       <c r="J5" t="n">
-        <v>32000</v>
+        <v>22400</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L5" t="n">
         <v>32000</v>
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -969,10 +969,10 @@
         <v>940221</v>
       </c>
       <c r="J11" t="n">
-        <v>11000</v>
+        <v>2200</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="L11" t="n">
         <v>11000</v>
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1143,10 +1143,10 @@
         <v>127273</v>
       </c>
       <c r="J15" t="n">
-        <v>84800</v>
+        <v>35620</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="L15" t="n">
         <v>84800</v>
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1187,10 +1187,10 @@
         <v>775883</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>44800</v>
+        <v>33600</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>44800</v>
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1319,10 +1319,10 @@
         <v>1373979</v>
       </c>
       <c r="J19" t="n">
-        <v>11000</v>
+        <v>5500</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L19" t="n">
         <v>11000</v>
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1405,10 +1405,10 @@
         <v>876898</v>
       </c>
       <c r="J21" t="n">
-        <v>5600</v>
+        <v>4480</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L21" t="n">
         <v>5600</v>
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1449,10 +1449,10 @@
         <v>736688</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>66000</v>
+        <v>49500</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>66000</v>
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1537,10 +1537,10 @@
         <v>1122546</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>10500</v>
+        <v>5250</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>10500</v>
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1801,10 +1801,10 @@
         <v>872384</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>16000</v>
+        <v>9600</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>16000</v>
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1845,10 +1845,10 @@
         <v>599805</v>
       </c>
       <c r="J31" t="n">
-        <v>20500</v>
+        <v>4510</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="L31" t="n">
         <v>20500</v>
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1975,10 +1975,10 @@
         <v>594327</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>10700</v>
+        <v>3210</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>10700</v>
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2283,10 +2283,10 @@
         <v>289966</v>
       </c>
       <c r="J41" t="n">
-        <v>79800</v>
+        <v>11970</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="L41" t="n">
         <v>79800</v>
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2415,10 +2415,10 @@
         <v>643681</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>5500</v>
+        <v>3300</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>5500</v>
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2547,10 +2547,10 @@
         <v>844480</v>
       </c>
       <c r="J47" t="n">
-        <v>24800</v>
+        <v>6200</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="L47" t="n">
         <v>24800</v>
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2591,10 +2591,10 @@
         <v>471451</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>22000</v>
+        <v>11000</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>22000</v>
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2635,10 +2635,10 @@
         <v>736611</v>
       </c>
       <c r="J49" t="n">
-        <v>21500</v>
+        <v>15050</v>
       </c>
       <c r="K49" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L49" t="n">
         <v>21500</v>
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2811,10 +2811,10 @@
         <v>143086</v>
       </c>
       <c r="J53" t="n">
-        <v>10500</v>
+        <v>2100</v>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="L53" t="n">
         <v>10500</v>
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2855,10 +2855,10 @@
         <v>434239</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>36800</v>
+        <v>9570</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>36800</v>
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2987,10 +2987,10 @@
         <v>355171</v>
       </c>
       <c r="J57" t="n">
-        <v>21500</v>
+        <v>14400</v>
       </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="L57" t="n">
         <v>21500</v>
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3075,10 +3075,10 @@
         <v>676667</v>
       </c>
       <c r="J59" t="n">
-        <v>73000</v>
+        <v>18250</v>
       </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="L59" t="n">
         <v>73000</v>
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3207,10 +3207,10 @@
         <v>323198</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>21000</v>
+        <v>14070</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>21000</v>
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3339,10 +3339,10 @@
         <v>243818</v>
       </c>
       <c r="J65" t="n">
-        <v>10500</v>
+        <v>2100</v>
       </c>
       <c r="K65" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="L65" t="n">
         <v>10500</v>
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3383,10 +3383,10 @@
         <v>175426</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>11000</v>
+        <v>2200</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>11000</v>
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3427,10 +3427,10 @@
         <v>200803</v>
       </c>
       <c r="J67" t="n">
-        <v>21500</v>
+        <v>12900</v>
       </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L67" t="n">
         <v>21500</v>
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3515,10 +3515,10 @@
         <v>175024</v>
       </c>
       <c r="J69" t="n">
-        <v>11000</v>
+        <v>2200</v>
       </c>
       <c r="K69" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="L69" t="n">
         <v>11000</v>
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3691,10 +3691,10 @@
         <v>435687</v>
       </c>
       <c r="J73" t="n">
-        <v>27400</v>
+        <v>2740</v>
       </c>
       <c r="K73" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L73" t="n">
         <v>27400</v>
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3779,10 +3779,10 @@
         <v>327889</v>
       </c>
       <c r="J75" t="n">
-        <v>47000</v>
+        <v>25850</v>
       </c>
       <c r="K75" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="L75" t="n">
         <v>47000</v>
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3823,10 +3823,10 @@
         <v>13442</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>10500</v>
+        <v>2100</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>10500</v>
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -3999,10 +3999,10 @@
         <v>181110</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>36700</v>
+        <v>14680</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>36700</v>
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4043,10 +4043,10 @@
         <v>307041</v>
       </c>
       <c r="J81" t="n">
-        <v>75000</v>
+        <v>37500</v>
       </c>
       <c r="K81" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L81" t="n">
         <v>75000</v>
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4087,10 +4087,10 @@
         <v>266</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>16500</v>
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4131,10 +4131,10 @@
         <v>239721</v>
       </c>
       <c r="J83" t="n">
-        <v>11000</v>
+        <v>2200</v>
       </c>
       <c r="K83" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="L83" t="n">
         <v>11000</v>
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4219,10 +4219,10 @@
         <v>222495</v>
       </c>
       <c r="J85" t="n">
-        <v>32000</v>
+        <v>9600</v>
       </c>
       <c r="K85" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L85" t="n">
         <v>32000</v>
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4263,10 +4263,10 @@
         <v>93489</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>27000</v>
+        <v>2700</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>27000</v>
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4351,10 +4351,10 @@
         <v>232360</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>60000</v>
+        <v>24000</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>60000</v>
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4527,10 +4527,10 @@
         <v>326054</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>22000</v>
+        <v>8800</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>22000</v>
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4615,10 +4615,10 @@
         <v>26360</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>53000</v>
+        <v>21200</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>53000</v>
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4703,10 +4703,10 @@
         <v>179154</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>10700</v>
+        <v>6950</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>10700</v>
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4747,10 +4747,10 @@
         <v>330349</v>
       </c>
       <c r="J97" t="n">
-        <v>26550</v>
+        <v>29500</v>
       </c>
       <c r="K97" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="L97" t="n">
         <v>59000</v>
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4791,10 +4791,10 @@
         <v>225479</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>42000</v>
+        <v>29400</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>42000</v>
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4879,10 +4879,10 @@
         <v>293127</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>26000</v>
+        <v>8580</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>26000</v>
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-25</t>
+          <t>Steam 인기 차트 — 2026-06-26</t>
         </is>
       </c>
     </row>
@@ -5096,33 +5096,33 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Palworld</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Early Access</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="4" t="n">
         <v>18028</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="4" t="n">
         <v>94.09999999999999</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="4" t="n">
         <v>380709</v>
       </c>
-      <c r="G7" t="n">
-        <v>32000</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
+      <c r="G7" s="4" t="n">
+        <v>22400</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="8">
@@ -5276,33 +5276,33 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Left 4 Dead 2</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="4" t="n">
         <v>25122</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="4" t="n">
         <v>97.5</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="4" t="n">
         <v>963983</v>
       </c>
-      <c r="G13" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
+      <c r="G13" s="4" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="14">
@@ -5394,63 +5394,63 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Monster Hunter Wilds</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, RPG</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="4" t="n">
         <v>12494</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="4" t="n">
         <v>58.3</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="4" t="n">
         <v>218415</v>
       </c>
-      <c r="G17" t="n">
-        <v>84800</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
+      <c r="G17" s="4" t="n">
+        <v>35620</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>58</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>HELLDIVERS™ 2</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="4" t="n">
         <v>53399</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="4" t="n">
         <v>76.2</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="F18" s="4" t="n">
         <v>1017635</v>
       </c>
-      <c r="G18" s="2" t="n">
-        <v>44800</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>0</v>
+      <c r="G18" s="4" t="n">
+        <v>33600</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="19">
@@ -5514,33 +5514,33 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Terraria</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D21" s="4" t="n">
         <v>24580</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="4" t="n">
         <v>97.5</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="4" t="n">
         <v>1409473</v>
       </c>
-      <c r="G21" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
+      <c r="G21" s="4" t="n">
+        <v>5500</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="22">
@@ -5572,63 +5572,63 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Wallpaper Engine</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Casual, Indie, Animation &amp; Modeling, Design &amp; Illustration, Photo Editing, Utilities</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" s="4" t="n">
         <v>91184</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="4" t="n">
         <v>98</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" s="4" t="n">
         <v>894458</v>
       </c>
-      <c r="G23" t="n">
-        <v>5600</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
+      <c r="G23" s="4" t="n">
+        <v>4480</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Baldur's Gate 3</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Adventure, RPG, Strategy</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D24" s="4" t="n">
         <v>54771</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="4" t="n">
         <v>96.8</v>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="F24" s="4" t="n">
         <v>760662</v>
       </c>
-      <c r="G24" s="2" t="n">
-        <v>66000</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>0</v>
+      <c r="G24" s="4" t="n">
+        <v>49500</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="25">
@@ -5662,33 +5662,33 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Garry's Mod</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n">
+      <c r="D26" s="4" t="n">
         <v>18400</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="4" t="n">
         <v>96.8</v>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="F26" s="4" t="n">
         <v>1159707</v>
       </c>
-      <c r="G26" s="2" t="n">
-        <v>10500</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>0</v>
+      <c r="G26" s="4" t="n">
+        <v>5250</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="27">
@@ -5842,63 +5842,63 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Stardew Valley</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Indie, RPG, Simulation</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n">
+      <c r="D32" s="4" t="n">
         <v>50662</v>
       </c>
-      <c r="E32" s="2" t="n">
+      <c r="E32" s="4" t="n">
         <v>98.40000000000001</v>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="F32" s="4" t="n">
         <v>886195</v>
       </c>
-      <c r="G32" s="2" t="n">
-        <v>16000</v>
-      </c>
-      <c r="H32" s="2" t="n">
-        <v>0</v>
+      <c r="G32" s="4" t="n">
+        <v>9600</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>The Forest</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" s="4" t="n">
         <v>2892</v>
       </c>
-      <c r="E33" t="n">
+      <c r="E33" s="4" t="n">
         <v>95.5</v>
       </c>
-      <c r="F33" t="n">
+      <c r="F33" s="4" t="n">
         <v>627791</v>
       </c>
-      <c r="G33" t="n">
-        <v>20500</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
+      <c r="G33" s="4" t="n">
+        <v>4510</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>78</v>
       </c>
     </row>
     <row r="34">
@@ -5960,33 +5960,33 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>PAYDAY 2</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D36" s="4" t="n">
         <v>27254</v>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E36" s="4" t="n">
         <v>89.59999999999999</v>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="F36" s="4" t="n">
         <v>663082</v>
       </c>
-      <c r="G36" s="2" t="n">
-        <v>10700</v>
-      </c>
-      <c r="H36" s="2" t="n">
-        <v>0</v>
+      <c r="G36" s="4" t="n">
+        <v>3210</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="37">
@@ -6170,33 +6170,33 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>Hogwarts Legacy</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, RPG</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D43" s="4" t="n">
         <v>5716</v>
       </c>
-      <c r="E43" t="n">
+      <c r="E43" s="4" t="n">
         <v>90.2</v>
       </c>
-      <c r="F43" t="n">
+      <c r="F43" s="4" t="n">
         <v>321395</v>
       </c>
-      <c r="G43" t="n">
-        <v>79800</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
+      <c r="G43" s="4" t="n">
+        <v>11970</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="44">
@@ -6260,33 +6260,33 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Among Us</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Casual</t>
         </is>
       </c>
-      <c r="D46" s="2" t="n">
+      <c r="D46" s="4" t="n">
         <v>3832</v>
       </c>
-      <c r="E46" s="2" t="n">
+      <c r="E46" s="4" t="n">
         <v>91.90000000000001</v>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="F46" s="4" t="n">
         <v>700785</v>
       </c>
-      <c r="G46" s="2" t="n">
-        <v>5500</v>
-      </c>
-      <c r="H46" s="2" t="n">
-        <v>0</v>
+      <c r="G46" s="4" t="n">
+        <v>3300</v>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="47">
@@ -6350,93 +6350,93 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>Euro Truck Simulator 2</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Indie, Simulation</t>
         </is>
       </c>
-      <c r="D49" t="n">
+      <c r="D49" s="4" t="n">
         <v>17281</v>
       </c>
-      <c r="E49" t="n">
+      <c r="E49" s="4" t="n">
         <v>97.40000000000001</v>
       </c>
-      <c r="F49" t="n">
+      <c r="F49" s="4" t="n">
         <v>867404</v>
       </c>
-      <c r="G49" t="n">
-        <v>24800</v>
-      </c>
-      <c r="H49" t="n">
-        <v>0</v>
+      <c r="G49" s="4" t="n">
+        <v>6200</v>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>Valheim</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Early Access</t>
         </is>
       </c>
-      <c r="D50" s="2" t="n">
+      <c r="D50" s="4" t="n">
         <v>14439</v>
       </c>
-      <c r="E50" s="2" t="n">
+      <c r="E50" s="4" t="n">
         <v>94.3</v>
       </c>
-      <c r="F50" s="2" t="n">
+      <c r="F50" s="4" t="n">
         <v>499828</v>
       </c>
-      <c r="G50" s="2" t="n">
-        <v>22000</v>
-      </c>
-      <c r="H50" s="2" t="n">
-        <v>0</v>
+      <c r="G50" s="4" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H50" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>Phasmophobia</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Action, Indie, Early Access</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D51" s="4" t="n">
         <v>9978</v>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="4" t="n">
         <v>95.8</v>
       </c>
-      <c r="F51" t="n">
+      <c r="F51" s="4" t="n">
         <v>768779</v>
       </c>
-      <c r="G51" t="n">
-        <v>21500</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0</v>
+      <c r="G51" s="4" t="n">
+        <v>15050</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="52">
@@ -6530,63 +6530,63 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="n">
+      <c r="A55" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>Half-Life</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D55" t="n">
+      <c r="D55" s="4" t="n">
         <v>634</v>
       </c>
-      <c r="E55" t="n">
+      <c r="E55" s="4" t="n">
         <v>96.5</v>
       </c>
-      <c r="F55" t="n">
+      <c r="F55" s="4" t="n">
         <v>148221</v>
       </c>
-      <c r="G55" t="n">
-        <v>10500</v>
-      </c>
-      <c r="H55" t="n">
-        <v>0</v>
+      <c r="G55" s="4" t="n">
+        <v>2100</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>Monster Hunter: World</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D56" s="2" t="n">
+      <c r="D56" s="4" t="n">
         <v>11923</v>
       </c>
-      <c r="E56" s="2" t="n">
+      <c r="E56" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="F56" s="2" t="n">
+      <c r="F56" s="4" t="n">
         <v>493390</v>
       </c>
-      <c r="G56" s="2" t="n">
-        <v>36800</v>
-      </c>
-      <c r="H56" s="2" t="n">
-        <v>0</v>
+      <c r="G56" s="4" t="n">
+        <v>9570</v>
+      </c>
+      <c r="H56" s="4" t="n">
+        <v>74</v>
       </c>
     </row>
     <row r="57">
@@ -6650,33 +6650,33 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="n">
+      <c r="A59" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>Project Zomboid</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>Indie, RPG, Simulation, Early Access</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D59" s="4" t="n">
         <v>22864</v>
       </c>
-      <c r="E59" t="n">
+      <c r="E59" s="4" t="n">
         <v>94.2</v>
       </c>
-      <c r="F59" t="n">
+      <c r="F59" s="4" t="n">
         <v>377063</v>
       </c>
-      <c r="G59" t="n">
-        <v>21500</v>
-      </c>
-      <c r="H59" t="n">
-        <v>0</v>
+      <c r="G59" s="4" t="n">
+        <v>14400</v>
+      </c>
+      <c r="H59" s="4" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="60">
@@ -6710,33 +6710,33 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="n">
+      <c r="A61" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>Red Dead Redemption 2</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure</t>
         </is>
       </c>
-      <c r="D61" t="n">
+      <c r="D61" s="4" t="n">
         <v>29885</v>
       </c>
-      <c r="E61" t="n">
+      <c r="E61" s="4" t="n">
         <v>92.2</v>
       </c>
-      <c r="F61" t="n">
+      <c r="F61" s="4" t="n">
         <v>733542</v>
       </c>
-      <c r="G61" t="n">
-        <v>73000</v>
-      </c>
-      <c r="H61" t="n">
-        <v>0</v>
+      <c r="G61" s="4" t="n">
+        <v>18250</v>
+      </c>
+      <c r="H61" s="4" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="62">
@@ -6800,33 +6800,33 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="4" t="n">
         <v>61</v>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>Raft</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D64" s="2" t="n">
+      <c r="D64" s="4" t="n">
         <v>4701</v>
       </c>
-      <c r="E64" s="2" t="n">
+      <c r="E64" s="4" t="n">
         <v>93.3</v>
       </c>
-      <c r="F64" s="2" t="n">
+      <c r="F64" s="4" t="n">
         <v>346359</v>
       </c>
-      <c r="G64" s="2" t="n">
-        <v>21000</v>
-      </c>
-      <c r="H64" s="2" t="n">
-        <v>0</v>
+      <c r="G64" s="4" t="n">
+        <v>14070</v>
+      </c>
+      <c r="H64" s="4" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="65">
@@ -6890,93 +6890,93 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="n">
+      <c r="A67" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>Counter-Strike</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D67" t="n">
+      <c r="D67" s="4" t="n">
         <v>7323</v>
       </c>
-      <c r="E67" t="n">
+      <c r="E67" s="4" t="n">
         <v>97.40000000000001</v>
       </c>
-      <c r="F67" t="n">
+      <c r="F67" s="4" t="n">
         <v>250245</v>
       </c>
-      <c r="G67" t="n">
-        <v>10500</v>
-      </c>
-      <c r="H67" t="n">
-        <v>0</v>
+      <c r="G67" s="4" t="n">
+        <v>2100</v>
+      </c>
+      <c r="H67" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B68" s="4" t="inlineStr">
         <is>
           <t>Counter-Strike: Source</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D68" s="2" t="n">
+      <c r="D68" s="4" t="n">
         <v>6187</v>
       </c>
-      <c r="E68" s="2" t="n">
+      <c r="E68" s="4" t="n">
         <v>96.3</v>
       </c>
-      <c r="F68" s="2" t="n">
+      <c r="F68" s="4" t="n">
         <v>182234</v>
       </c>
-      <c r="G68" s="2" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>0</v>
+      <c r="G68" s="4" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H68" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="n">
+      <c r="A69" s="4" t="n">
         <v>66</v>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="4" t="inlineStr">
         <is>
           <t>Schedule I</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>Action, Indie, Simulation, Strategy, Early Access</t>
         </is>
       </c>
-      <c r="D69" t="n">
+      <c r="D69" s="4" t="n">
         <v>22757</v>
       </c>
-      <c r="E69" t="n">
+      <c r="E69" s="4" t="n">
         <v>98.40000000000001</v>
       </c>
-      <c r="F69" t="n">
+      <c r="F69" s="4" t="n">
         <v>204041</v>
       </c>
-      <c r="G69" t="n">
-        <v>21500</v>
-      </c>
-      <c r="H69" t="n">
-        <v>0</v>
+      <c r="G69" s="4" t="n">
+        <v>12900</v>
+      </c>
+      <c r="H69" s="4" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="70">
@@ -7010,33 +7010,33 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="n">
+      <c r="A71" s="4" t="n">
         <v>68</v>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D71" t="n">
+      <c r="D71" s="4" t="n">
         <v>638</v>
       </c>
-      <c r="E71" t="n">
+      <c r="E71" s="4" t="n">
         <v>98.5</v>
       </c>
-      <c r="F71" t="n">
+      <c r="F71" s="4" t="n">
         <v>177741</v>
       </c>
-      <c r="G71" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H71" t="n">
-        <v>0</v>
+      <c r="G71" s="4" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H71" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="72">
@@ -7130,33 +7130,33 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="n">
+      <c r="A75" s="4" t="n">
         <v>72</v>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="4" t="inlineStr">
         <is>
           <t>Dying Light</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="4" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D75" t="n">
+      <c r="D75" s="4" t="n">
         <v>4953</v>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="4" t="n">
         <v>95.2</v>
       </c>
-      <c r="F75" t="n">
+      <c r="F75" s="4" t="n">
         <v>457632</v>
       </c>
-      <c r="G75" t="n">
-        <v>27400</v>
-      </c>
-      <c r="H75" t="n">
-        <v>0</v>
+      <c r="G75" s="4" t="n">
+        <v>2740</v>
+      </c>
+      <c r="H75" s="4" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="76">
@@ -7190,63 +7190,63 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="n">
+      <c r="A77" s="4" t="n">
         <v>74</v>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="4" t="inlineStr">
         <is>
           <t>7 Days to Die</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D77" t="n">
+      <c r="D77" s="4" t="n">
         <v>17045</v>
       </c>
-      <c r="E77" t="n">
+      <c r="E77" s="4" t="n">
         <v>88.59999999999999</v>
       </c>
-      <c r="F77" t="n">
+      <c r="F77" s="4" t="n">
         <v>370046</v>
       </c>
-      <c r="G77" t="n">
-        <v>47000</v>
-      </c>
-      <c r="H77" t="n">
-        <v>0</v>
+      <c r="G77" s="4" t="n">
+        <v>25850</v>
+      </c>
+      <c r="H77" s="4" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
         <is>
           <t>Counter-Strike: Condition Zero</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D78" s="2" t="n">
+      <c r="D78" s="4" t="n">
         <v>83</v>
       </c>
-      <c r="E78" s="2" t="n">
+      <c r="E78" s="4" t="n">
         <v>89.8</v>
       </c>
-      <c r="F78" s="2" t="n">
+      <c r="F78" s="4" t="n">
         <v>14977</v>
       </c>
-      <c r="G78" s="2" t="n">
-        <v>10500</v>
-      </c>
-      <c r="H78" s="2" t="n">
-        <v>0</v>
+      <c r="G78" s="4" t="n">
+        <v>2100</v>
+      </c>
+      <c r="H78" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="79">
@@ -7340,123 +7340,123 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="4" t="n">
         <v>79</v>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B82" s="4" t="inlineStr">
         <is>
           <t>Hunt: Showdown 1896</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="C82" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D82" s="2" t="n">
+      <c r="D82" s="4" t="n">
         <v>6300</v>
       </c>
-      <c r="E82" s="2" t="n">
+      <c r="E82" s="4" t="n">
         <v>73</v>
       </c>
-      <c r="F82" s="2" t="n">
+      <c r="F82" s="4" t="n">
         <v>248220</v>
       </c>
-      <c r="G82" s="2" t="n">
-        <v>36700</v>
-      </c>
-      <c r="H82" s="2" t="n">
-        <v>0</v>
+      <c r="G82" s="4" t="n">
+        <v>14680</v>
+      </c>
+      <c r="H82" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="n">
+      <c r="A83" s="4" t="n">
         <v>80</v>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="4" t="inlineStr">
         <is>
           <t>Sekiro™: Shadows Die Twice - GOTY Edition</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C83" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure</t>
         </is>
       </c>
-      <c r="D83" t="n">
+      <c r="D83" s="4" t="n">
         <v>6767</v>
       </c>
-      <c r="E83" t="n">
+      <c r="E83" s="4" t="n">
         <v>95.3</v>
       </c>
-      <c r="F83" t="n">
+      <c r="F83" s="4" t="n">
         <v>322234</v>
       </c>
-      <c r="G83" t="n">
-        <v>75000</v>
-      </c>
-      <c r="H83" t="n">
-        <v>0</v>
+      <c r="G83" s="4" t="n">
+        <v>37500</v>
+      </c>
+      <c r="H83" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="4" t="n">
         <v>81</v>
       </c>
-      <c r="B84" s="2" t="inlineStr">
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>CyberCorp</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
+      <c r="C84" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D84" s="2" t="n">
+      <c r="D84" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E84" s="2" t="n">
+      <c r="E84" s="4" t="n">
         <v>82.59999999999999</v>
       </c>
-      <c r="F84" s="2" t="n">
+      <c r="F84" s="4" t="n">
         <v>322</v>
       </c>
-      <c r="G84" s="2" t="n">
-        <v>16500</v>
-      </c>
-      <c r="H84" s="2" t="n">
-        <v>0</v>
+      <c r="G84" s="4" t="n">
+        <v>9900</v>
+      </c>
+      <c r="H84" s="4" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="n">
+      <c r="A85" s="4" t="n">
         <v>82</v>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="4" t="inlineStr">
         <is>
           <t>Half-Life 2</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="4" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D85" t="n">
+      <c r="D85" s="4" t="n">
         <v>1555</v>
       </c>
-      <c r="E85" t="n">
+      <c r="E85" s="4" t="n">
         <v>97.59999999999999</v>
       </c>
-      <c r="F85" t="n">
+      <c r="F85" s="4" t="n">
         <v>245627</v>
       </c>
-      <c r="G85" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H85" t="n">
-        <v>0</v>
+      <c r="G85" s="4" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H85" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="86">
@@ -7490,63 +7490,63 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="n">
+      <c r="A87" s="4" t="n">
         <v>84</v>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>Sons Of The Forest</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D87" t="n">
+      <c r="D87" s="4" t="n">
         <v>4450</v>
       </c>
-      <c r="E87" t="n">
+      <c r="E87" s="4" t="n">
         <v>87.8</v>
       </c>
-      <c r="F87" t="n">
+      <c r="F87" s="4" t="n">
         <v>253546</v>
       </c>
-      <c r="G87" t="n">
-        <v>32000</v>
-      </c>
-      <c r="H87" t="n">
-        <v>0</v>
+      <c r="G87" s="4" t="n">
+        <v>9600</v>
+      </c>
+      <c r="H87" s="4" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="4" t="n">
         <v>85</v>
       </c>
-      <c r="B88" s="2" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>Grim Dawn</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C88" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D88" s="2" t="n">
+      <c r="D88" s="4" t="n">
         <v>2376</v>
       </c>
-      <c r="E88" s="2" t="n">
+      <c r="E88" s="4" t="n">
         <v>93.7</v>
       </c>
-      <c r="F88" s="2" t="n">
+      <c r="F88" s="4" t="n">
         <v>99730</v>
       </c>
-      <c r="G88" s="2" t="n">
-        <v>27000</v>
-      </c>
-      <c r="H88" s="2" t="n">
-        <v>0</v>
+      <c r="G88" s="4" t="n">
+        <v>2700</v>
+      </c>
+      <c r="H88" s="4" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="89">
@@ -7580,33 +7580,33 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="B90" s="2" t="inlineStr">
+      <c r="B90" s="4" t="inlineStr">
         <is>
           <t>Mount &amp; Blade II: Bannerlord</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C90" s="4" t="inlineStr">
         <is>
           <t>Action, Indie, RPG, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D90" s="2" t="n">
+      <c r="D90" s="4" t="n">
         <v>14477</v>
       </c>
-      <c r="E90" s="2" t="n">
+      <c r="E90" s="4" t="n">
         <v>87.90000000000001</v>
       </c>
-      <c r="F90" s="2" t="n">
+      <c r="F90" s="4" t="n">
         <v>264391</v>
       </c>
-      <c r="G90" s="2" t="n">
-        <v>60000</v>
-      </c>
-      <c r="H90" s="2" t="n">
-        <v>0</v>
+      <c r="G90" s="4" t="n">
+        <v>24000</v>
+      </c>
+      <c r="H90" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="91">
@@ -7700,33 +7700,33 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="4" t="n">
         <v>91</v>
       </c>
-      <c r="B94" s="2" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>Fallout 4</t>
         </is>
       </c>
-      <c r="C94" s="2" t="inlineStr">
+      <c r="C94" s="4" t="inlineStr">
         <is>
           <t>RPG</t>
         </is>
       </c>
-      <c r="D94" s="2" t="n">
+      <c r="D94" s="4" t="n">
         <v>11179</v>
       </c>
-      <c r="E94" s="2" t="n">
+      <c r="E94" s="4" t="n">
         <v>83.09999999999999</v>
       </c>
-      <c r="F94" s="2" t="n">
+      <c r="F94" s="4" t="n">
         <v>392287</v>
       </c>
-      <c r="G94" s="2" t="n">
-        <v>22000</v>
-      </c>
-      <c r="H94" s="2" t="n">
-        <v>0</v>
+      <c r="G94" s="4" t="n">
+        <v>8800</v>
+      </c>
+      <c r="H94" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="95">
@@ -7760,33 +7760,33 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="4" t="n">
         <v>93</v>
       </c>
-      <c r="B96" s="2" t="inlineStr">
+      <c r="B96" s="4" t="inlineStr">
         <is>
           <t>Warhammer 40,000: Rogue Trader</t>
         </is>
       </c>
-      <c r="C96" s="2" t="inlineStr">
+      <c r="C96" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Strategy</t>
         </is>
       </c>
-      <c r="D96" s="2" t="n">
+      <c r="D96" s="4" t="n">
         <v>3582</v>
       </c>
-      <c r="E96" s="2" t="n">
+      <c r="E96" s="4" t="n">
         <v>85.59999999999999</v>
       </c>
-      <c r="F96" s="2" t="n">
+      <c r="F96" s="4" t="n">
         <v>30805</v>
       </c>
-      <c r="G96" s="2" t="n">
-        <v>53000</v>
-      </c>
-      <c r="H96" s="2" t="n">
-        <v>0</v>
+      <c r="G96" s="4" t="n">
+        <v>21200</v>
+      </c>
+      <c r="H96" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="97">
@@ -7820,33 +7820,33 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="4" t="n">
         <v>95</v>
       </c>
-      <c r="B98" s="2" t="inlineStr">
+      <c r="B98" s="4" t="inlineStr">
         <is>
           <t>R.E.P.O.</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr">
+      <c r="C98" s="4" t="inlineStr">
         <is>
           <t>Action, Early Access</t>
         </is>
       </c>
-      <c r="D98" s="2" t="n">
+      <c r="D98" s="4" t="n">
         <v>32349</v>
       </c>
-      <c r="E98" s="2" t="n">
+      <c r="E98" s="4" t="n">
         <v>96.5</v>
       </c>
-      <c r="F98" s="2" t="n">
+      <c r="F98" s="4" t="n">
         <v>185642</v>
       </c>
-      <c r="G98" s="2" t="n">
-        <v>10700</v>
-      </c>
-      <c r="H98" s="2" t="n">
-        <v>0</v>
+      <c r="G98" s="4" t="n">
+        <v>6950</v>
+      </c>
+      <c r="H98" s="4" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="99">
@@ -7873,40 +7873,40 @@
         <v>430252</v>
       </c>
       <c r="G99" s="4" t="n">
-        <v>26550</v>
+        <v>29500</v>
       </c>
       <c r="H99" s="4" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="4" t="n">
         <v>97</v>
       </c>
-      <c r="B100" s="2" t="inlineStr">
+      <c r="B100" s="4" t="inlineStr">
         <is>
           <t>Satisfactory</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
+      <c r="C100" s="4" t="inlineStr">
         <is>
           <t>Adventure, Indie, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D100" s="2" t="n">
+      <c r="D100" s="4" t="n">
         <v>12596</v>
       </c>
-      <c r="E100" s="2" t="n">
+      <c r="E100" s="4" t="n">
         <v>97.2</v>
       </c>
-      <c r="F100" s="2" t="n">
+      <c r="F100" s="4" t="n">
         <v>232064</v>
       </c>
-      <c r="G100" s="2" t="n">
-        <v>42000</v>
-      </c>
-      <c r="H100" s="2" t="n">
-        <v>0</v>
+      <c r="G100" s="4" t="n">
+        <v>29400</v>
+      </c>
+      <c r="H100" s="4" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="101">
@@ -7940,33 +7940,33 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="4" t="n">
         <v>99</v>
       </c>
-      <c r="B102" s="2" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>Risk of Rain 2</t>
         </is>
       </c>
-      <c r="C102" s="2" t="inlineStr">
+      <c r="C102" s="4" t="inlineStr">
         <is>
           <t>Action, Indie</t>
         </is>
       </c>
-      <c r="D102" s="2" t="n">
+      <c r="D102" s="4" t="n">
         <v>7902</v>
       </c>
-      <c r="E102" s="2" t="n">
+      <c r="E102" s="4" t="n">
         <v>93.5</v>
       </c>
-      <c r="F102" s="2" t="n">
+      <c r="F102" s="4" t="n">
         <v>313577</v>
       </c>
-      <c r="G102" s="2" t="n">
-        <v>26000</v>
-      </c>
-      <c r="H102" s="2" t="n">
-        <v>0</v>
+      <c r="G102" s="4" t="n">
+        <v>8580</v>
+      </c>
+      <c r="H102" s="4" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="103">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-25</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-26</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-25</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-26</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-25</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-27
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-26</t>
+          <t>Steam 인기 차트 — 2026-06-27</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-26</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-27</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-26</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-27</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-26</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-28
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1757,10 +1757,10 @@
         <v>612177</v>
       </c>
       <c r="J29" t="n">
-        <v>16500</v>
+        <v>10890</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="L29" t="n">
         <v>16500</v>
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-27</t>
+          <t>Steam 인기 차트 — 2026-06-28</t>
         </is>
       </c>
     </row>
@@ -5812,33 +5812,33 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>ARK: Survival Evolved</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Massively Multiplayer, RPG</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="4" t="n">
         <v>22170</v>
       </c>
-      <c r="E31" t="n">
+      <c r="E31" s="4" t="n">
         <v>83.8</v>
       </c>
-      <c r="F31" t="n">
+      <c r="F31" s="4" t="n">
         <v>730170</v>
       </c>
-      <c r="G31" t="n">
-        <v>16500</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0</v>
+      <c r="G31" s="4" t="n">
+        <v>10890</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="32">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-27</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-28</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-27</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-28</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-27</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-29
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-28</t>
+          <t>Steam 인기 차트 — 2026-06-29</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-28</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-29</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-28</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-29</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-28</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-06-30
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-29</t>
+          <t>Steam 인기 차트 — 2026-06-30</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-29</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-30</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-29</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-30</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-29</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-01
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-06-30</t>
+          <t>Steam 인기 차트 — 2026-07-01</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-06-30</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-01</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-06-30</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-01</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-06-30</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-02
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Action, RPG</t>
+          <t>Action, Adventure, RPG</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-01</t>
+          <t>Steam 인기 차트 — 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -7140,7 +7140,7 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Action, RPG</t>
+          <t>Action, Adventure, RPG</t>
         </is>
       </c>
       <c r="D75" s="4" t="n">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-01</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-01</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-01</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-03
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-02</t>
+          <t>Steam 인기 차트 — 2026-07-03</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-02</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-03</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-02</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-03</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-02</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-04
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-03</t>
+          <t>Steam 인기 차트 — 2026-07-04</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-03</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-04</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-03</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-04</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-03</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-05
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-04</t>
+          <t>Steam 인기 차트 — 2026-07-05</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-04</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-05</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-04</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-05</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-04</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-06
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-05</t>
+          <t>Steam 인기 차트 — 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-05</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-05</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-05</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-07
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-06</t>
+          <t>Steam 인기 차트 — 2026-07-07</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-06</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-07</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-06</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-07</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-06</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-08
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-07</t>
+          <t>Steam 인기 차트 — 2026-07-08</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-07</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-08</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-07</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-08</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-07</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-09
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-08</t>
+          <t>Steam 인기 차트 — 2026-07-09</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-08</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-09</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-08</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-09</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-08</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-10
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -969,10 +969,10 @@
         <v>940221</v>
       </c>
       <c r="J11" t="n">
-        <v>2200</v>
+        <v>11000</v>
       </c>
       <c r="K11" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>11000</v>
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1143,10 +1143,10 @@
         <v>127273</v>
       </c>
       <c r="J15" t="n">
-        <v>35620</v>
+        <v>84800</v>
       </c>
       <c r="K15" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>84800</v>
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1187,10 +1187,10 @@
         <v>775883</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>33600</v>
+        <v>44800</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>44800</v>
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1319,10 +1319,10 @@
         <v>1373979</v>
       </c>
       <c r="J19" t="n">
-        <v>5500</v>
+        <v>11000</v>
       </c>
       <c r="K19" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
         <v>11000</v>
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1405,10 +1405,10 @@
         <v>876898</v>
       </c>
       <c r="J21" t="n">
-        <v>4480</v>
+        <v>5600</v>
       </c>
       <c r="K21" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
         <v>5600</v>
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1449,10 +1449,10 @@
         <v>736688</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>49500</v>
+        <v>66000</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>66000</v>
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1537,10 +1537,10 @@
         <v>1122546</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>5250</v>
+        <v>10500</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>10500</v>
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1669,10 +1669,10 @@
         <v>1071135</v>
       </c>
       <c r="J27" t="n">
-        <v>21000</v>
+        <v>42000</v>
       </c>
       <c r="K27" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
         <v>42000</v>
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1801,10 +1801,10 @@
         <v>872384</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>9600</v>
+        <v>16000</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>16000</v>
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1845,10 +1845,10 @@
         <v>599805</v>
       </c>
       <c r="J31" t="n">
-        <v>4510</v>
+        <v>20500</v>
       </c>
       <c r="K31" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
         <v>20500</v>
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1975,10 +1975,10 @@
         <v>594327</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>3210</v>
+        <v>10700</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>10700</v>
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2107,10 +2107,10 @@
         <v>88027</v>
       </c>
       <c r="J37" t="n">
-        <v>30000</v>
+        <v>37500</v>
       </c>
       <c r="K37" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
         <v>37500</v>
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2195,10 +2195,10 @@
         <v>713071</v>
       </c>
       <c r="J39" t="n">
-        <v>19800</v>
+        <v>66000</v>
       </c>
       <c r="K39" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
         <v>66000</v>
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2239,10 +2239,10 @@
         <v>630223</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>8600</v>
+        <v>21500</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>21500</v>
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2283,10 +2283,10 @@
         <v>289966</v>
       </c>
       <c r="J41" t="n">
-        <v>11970</v>
+        <v>79800</v>
       </c>
       <c r="K41" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="L41" t="n">
         <v>79800</v>
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2371,10 +2371,10 @@
         <v>802993</v>
       </c>
       <c r="J43" t="n">
-        <v>3480</v>
+        <v>34800</v>
       </c>
       <c r="K43" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L43" t="n">
         <v>34800</v>
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2415,10 +2415,10 @@
         <v>643681</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>3300</v>
+        <v>5500</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>5500</v>
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2503,10 +2503,10 @@
         <v>272900</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>5250</v>
+        <v>21000</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>21000</v>
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2591,10 +2591,10 @@
         <v>471451</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>11000</v>
+        <v>22000</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>22000</v>
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2635,10 +2635,10 @@
         <v>736611</v>
       </c>
       <c r="J49" t="n">
-        <v>15050</v>
+        <v>21500</v>
       </c>
       <c r="K49" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L49" t="n">
         <v>21500</v>
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2811,10 +2811,10 @@
         <v>143086</v>
       </c>
       <c r="J53" t="n">
-        <v>2100</v>
+        <v>10500</v>
       </c>
       <c r="K53" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L53" t="n">
         <v>10500</v>
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2855,10 +2855,10 @@
         <v>434239</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>9570</v>
+        <v>36800</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>36800</v>
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2987,10 +2987,10 @@
         <v>355171</v>
       </c>
       <c r="J57" t="n">
-        <v>14400</v>
+        <v>21500</v>
       </c>
       <c r="K57" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="L57" t="n">
         <v>21500</v>
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3119,10 +3119,10 @@
         <v>139186</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>3300</v>
+        <v>66000</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>66000</v>
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3207,10 +3207,10 @@
         <v>323198</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>14070</v>
+        <v>21000</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>21000</v>
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3339,10 +3339,10 @@
         <v>243818</v>
       </c>
       <c r="J65" t="n">
-        <v>2100</v>
+        <v>10500</v>
       </c>
       <c r="K65" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L65" t="n">
         <v>10500</v>
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3383,10 +3383,10 @@
         <v>175426</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>2200</v>
+        <v>11000</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>11000</v>
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3427,10 +3427,10 @@
         <v>200803</v>
       </c>
       <c r="J67" t="n">
-        <v>12900</v>
+        <v>21500</v>
       </c>
       <c r="K67" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="L67" t="n">
         <v>21500</v>
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3515,10 +3515,10 @@
         <v>175024</v>
       </c>
       <c r="J69" t="n">
-        <v>2200</v>
+        <v>11000</v>
       </c>
       <c r="K69" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L69" t="n">
         <v>11000</v>
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3647,10 +3647,10 @@
         <v>475393</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>1550</v>
+        <v>15500</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>15500</v>
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3691,10 +3691,10 @@
         <v>435687</v>
       </c>
       <c r="J73" t="n">
-        <v>2740</v>
+        <v>27400</v>
       </c>
       <c r="K73" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L73" t="n">
         <v>27400</v>
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3735,10 +3735,10 @@
         <v>202253</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>6150</v>
+        <v>20500</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>20500</v>
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3779,10 +3779,10 @@
         <v>327889</v>
       </c>
       <c r="J75" t="n">
-        <v>25850</v>
+        <v>47000</v>
       </c>
       <c r="K75" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="L75" t="n">
         <v>47000</v>
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3823,10 +3823,10 @@
         <v>13442</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>2100</v>
+        <v>10500</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>10500</v>
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -3999,10 +3999,10 @@
         <v>181110</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>14680</v>
+        <v>36700</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>36700</v>
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4043,10 +4043,10 @@
         <v>307041</v>
       </c>
       <c r="J81" t="n">
-        <v>37500</v>
+        <v>75000</v>
       </c>
       <c r="K81" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L81" t="n">
         <v>75000</v>
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4087,10 +4087,10 @@
         <v>266</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>9900</v>
+        <v>16500</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>16500</v>
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4131,10 +4131,10 @@
         <v>239721</v>
       </c>
       <c r="J83" t="n">
-        <v>2200</v>
+        <v>11000</v>
       </c>
       <c r="K83" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L83" t="n">
         <v>11000</v>
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4175,10 +4175,10 @@
         <v>256128</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>10800</v>
+        <v>36000</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>36000</v>
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4219,10 +4219,10 @@
         <v>222495</v>
       </c>
       <c r="J85" t="n">
-        <v>9600</v>
+        <v>32000</v>
       </c>
       <c r="K85" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L85" t="n">
         <v>32000</v>
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4263,10 +4263,10 @@
         <v>93489</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>2700</v>
+        <v>5400</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>27000</v>
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4307,10 +4307,10 @@
         <v>256362</v>
       </c>
       <c r="J87" t="n">
-        <v>9900</v>
+        <v>33000</v>
       </c>
       <c r="K87" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L87" t="n">
         <v>33000</v>
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4351,10 +4351,10 @@
         <v>232360</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>24000</v>
+        <v>60000</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>60000</v>
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4395,10 +4395,10 @@
         <v>195724</v>
       </c>
       <c r="J89" t="n">
-        <v>8000</v>
+        <v>32000</v>
       </c>
       <c r="K89" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="L89" t="n">
         <v>32000</v>
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4483,10 +4483,10 @@
         <v>304053</v>
       </c>
       <c r="J91" t="n">
-        <v>6500</v>
+        <v>65000</v>
       </c>
       <c r="K91" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L91" t="n">
         <v>65000</v>
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4527,10 +4527,10 @@
         <v>326054</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>8800</v>
+        <v>22000</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>22000</v>
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4659,10 +4659,10 @@
         <v>177352</v>
       </c>
       <c r="J95" t="n">
-        <v>2750</v>
+        <v>55000</v>
       </c>
       <c r="K95" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="L95" t="n">
         <v>55000</v>
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4703,10 +4703,10 @@
         <v>179154</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>6950</v>
+        <v>10700</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>10700</v>
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4747,10 +4747,10 @@
         <v>330349</v>
       </c>
       <c r="J97" t="n">
-        <v>29500</v>
+        <v>59000</v>
       </c>
       <c r="K97" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L97" t="n">
         <v>59000</v>
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4791,10 +4791,10 @@
         <v>225479</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>29400</v>
+        <v>42000</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>42000</v>
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4879,10 +4879,10 @@
         <v>293127</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>8580</v>
+        <v>26000</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>26000</v>
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-09</t>
+          <t>Steam 인기 차트 — 2026-07-10</t>
         </is>
       </c>
     </row>
@@ -5276,33 +5276,33 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n">
+      <c r="A13" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Left 4 Dead 2</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" t="n">
         <v>25122</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" t="n">
         <v>97.5</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F13" t="n">
         <v>963983</v>
       </c>
-      <c r="G13" s="4" t="n">
-        <v>2200</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>80</v>
+      <c r="G13" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -5394,63 +5394,63 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n">
+      <c r="A17" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Monster Hunter Wilds</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Action, Adventure, RPG</t>
         </is>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" t="n">
         <v>12494</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" t="n">
         <v>58.3</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="F17" t="n">
         <v>218415</v>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>35620</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>58</v>
+      <c r="G17" t="n">
+        <v>84800</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>HELLDIVERS™ 2</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="2" t="n">
         <v>53399</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="2" t="n">
         <v>76.2</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="F18" s="2" t="n">
         <v>1017635</v>
       </c>
-      <c r="G18" s="4" t="n">
-        <v>33600</v>
-      </c>
-      <c r="H18" s="4" t="n">
-        <v>25</v>
+      <c r="G18" s="2" t="n">
+        <v>44800</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -5514,33 +5514,33 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Terraria</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" t="n">
         <v>24580</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" t="n">
         <v>97.5</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="F21" t="n">
         <v>1409473</v>
       </c>
-      <c r="G21" s="4" t="n">
-        <v>5500</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>50</v>
+      <c r="G21" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -5572,63 +5572,63 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n">
+      <c r="A23" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Wallpaper Engine</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Casual, Indie, Animation &amp; Modeling, Design &amp; Illustration, Photo Editing, Utilities</t>
         </is>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="D23" t="n">
         <v>91184</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" t="n">
         <v>98</v>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="F23" t="n">
         <v>894458</v>
       </c>
-      <c r="G23" s="4" t="n">
-        <v>4480</v>
-      </c>
-      <c r="H23" s="4" t="n">
-        <v>20</v>
+      <c r="G23" t="n">
+        <v>5600</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Baldur's Gate 3</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Adventure, RPG, Strategy</t>
         </is>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="D24" s="2" t="n">
         <v>54771</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" s="2" t="n">
         <v>96.8</v>
       </c>
-      <c r="F24" s="4" t="n">
+      <c r="F24" s="2" t="n">
         <v>760662</v>
       </c>
-      <c r="G24" s="4" t="n">
-        <v>49500</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>25</v>
+      <c r="G24" s="2" t="n">
+        <v>66000</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -5662,33 +5662,33 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Garry's Mod</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="D26" s="2" t="n">
         <v>18400</v>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="E26" s="2" t="n">
         <v>96.8</v>
       </c>
-      <c r="F26" s="4" t="n">
+      <c r="F26" s="2" t="n">
         <v>1159707</v>
       </c>
-      <c r="G26" s="4" t="n">
-        <v>5250</v>
-      </c>
-      <c r="H26" s="4" t="n">
-        <v>50</v>
+      <c r="G26" s="2" t="n">
+        <v>10500</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -5752,33 +5752,33 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n">
+      <c r="A29" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Rust</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Massively Multiplayer, RPG</t>
         </is>
       </c>
-      <c r="D29" s="4" t="n">
+      <c r="D29" t="n">
         <v>143870</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" t="n">
         <v>87.2</v>
       </c>
-      <c r="F29" s="4" t="n">
+      <c r="F29" t="n">
         <v>1227784</v>
       </c>
-      <c r="G29" s="4" t="n">
-        <v>21000</v>
-      </c>
-      <c r="H29" s="4" t="n">
-        <v>50</v>
+      <c r="G29" t="n">
+        <v>42000</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -5842,63 +5842,63 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Stardew Valley</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Indie, RPG, Simulation</t>
         </is>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="D32" s="2" t="n">
         <v>50662</v>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="E32" s="2" t="n">
         <v>98.40000000000001</v>
       </c>
-      <c r="F32" s="4" t="n">
+      <c r="F32" s="2" t="n">
         <v>886195</v>
       </c>
-      <c r="G32" s="4" t="n">
-        <v>9600</v>
-      </c>
-      <c r="H32" s="4" t="n">
-        <v>40</v>
+      <c r="G32" s="2" t="n">
+        <v>16000</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n">
+      <c r="A33" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>The Forest</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D33" t="n">
         <v>2892</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E33" t="n">
         <v>95.5</v>
       </c>
-      <c r="F33" s="4" t="n">
+      <c r="F33" t="n">
         <v>627791</v>
       </c>
-      <c r="G33" s="4" t="n">
-        <v>4510</v>
-      </c>
-      <c r="H33" s="4" t="n">
-        <v>78</v>
+      <c r="G33" t="n">
+        <v>20500</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -5960,33 +5960,33 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n">
+      <c r="A36" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>PAYDAY 2</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D36" s="4" t="n">
+      <c r="D36" s="2" t="n">
         <v>27254</v>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="E36" s="2" t="n">
         <v>89.59999999999999</v>
       </c>
-      <c r="F36" s="4" t="n">
+      <c r="F36" s="2" t="n">
         <v>663082</v>
       </c>
-      <c r="G36" s="4" t="n">
-        <v>3210</v>
-      </c>
-      <c r="H36" s="4" t="n">
-        <v>70</v>
+      <c r="G36" s="2" t="n">
+        <v>10700</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -6050,33 +6050,33 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n">
+      <c r="A39" t="n">
         <v>36</v>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>Last Epoch</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D39" s="4" t="n">
+      <c r="D39" t="n">
         <v>5831</v>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="E39" t="n">
         <v>79.59999999999999</v>
       </c>
-      <c r="F39" s="4" t="n">
+      <c r="F39" t="n">
         <v>110623</v>
       </c>
-      <c r="G39" s="4" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H39" s="4" t="n">
-        <v>20</v>
+      <c r="G39" t="n">
+        <v>37500</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -6110,93 +6110,93 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n">
+      <c r="A41" t="n">
         <v>38</v>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>Cyberpunk 2077</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>RPG</t>
         </is>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="D41" t="n">
         <v>22265</v>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="E41" t="n">
         <v>84.40000000000001</v>
       </c>
-      <c r="F41" s="4" t="n">
+      <c r="F41" t="n">
         <v>844921</v>
       </c>
-      <c r="G41" s="4" t="n">
-        <v>19800</v>
-      </c>
-      <c r="H41" s="4" t="n">
-        <v>70</v>
+      <c r="G41" t="n">
+        <v>66000</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n">
+      <c r="A42" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Dead by Daylight</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D42" s="4" t="n">
+      <c r="D42" s="2" t="n">
         <v>44886</v>
       </c>
-      <c r="E42" s="4" t="n">
+      <c r="E42" s="2" t="n">
         <v>79.09999999999999</v>
       </c>
-      <c r="F42" s="4" t="n">
+      <c r="F42" s="2" t="n">
         <v>797216</v>
       </c>
-      <c r="G42" s="4" t="n">
-        <v>8600</v>
-      </c>
-      <c r="H42" s="4" t="n">
-        <v>60</v>
+      <c r="G42" s="2" t="n">
+        <v>21500</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n">
+      <c r="A43" t="n">
         <v>40</v>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Hogwarts Legacy</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Action, Adventure, RPG</t>
         </is>
       </c>
-      <c r="D43" s="4" t="n">
+      <c r="D43" t="n">
         <v>5716</v>
       </c>
-      <c r="E43" s="4" t="n">
+      <c r="E43" t="n">
         <v>90.2</v>
       </c>
-      <c r="F43" s="4" t="n">
+      <c r="F43" t="n">
         <v>321395</v>
       </c>
-      <c r="G43" s="4" t="n">
-        <v>11970</v>
-      </c>
-      <c r="H43" s="4" t="n">
-        <v>85</v>
+      <c r="G43" t="n">
+        <v>79800</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -6230,63 +6230,63 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="n">
+      <c r="A45" t="n">
         <v>42</v>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>The Witcher 3: Wild Hunt</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>RPG</t>
         </is>
       </c>
-      <c r="D45" s="4" t="n">
+      <c r="D45" t="n">
         <v>15893</v>
       </c>
-      <c r="E45" s="4" t="n">
+      <c r="E45" t="n">
         <v>96.09999999999999</v>
       </c>
-      <c r="F45" s="4" t="n">
+      <c r="F45" t="n">
         <v>835349</v>
       </c>
-      <c r="G45" s="4" t="n">
-        <v>3480</v>
-      </c>
-      <c r="H45" s="4" t="n">
-        <v>90</v>
+      <c r="G45" t="n">
+        <v>34800</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="n">
+      <c r="A46" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Among Us</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Casual</t>
         </is>
       </c>
-      <c r="D46" s="4" t="n">
+      <c r="D46" s="2" t="n">
         <v>3832</v>
       </c>
-      <c r="E46" s="4" t="n">
+      <c r="E46" s="2" t="n">
         <v>91.90000000000001</v>
       </c>
-      <c r="F46" s="4" t="n">
+      <c r="F46" s="2" t="n">
         <v>700785</v>
       </c>
-      <c r="G46" s="4" t="n">
-        <v>3300</v>
-      </c>
-      <c r="H46" s="4" t="n">
-        <v>40</v>
+      <c r="G46" s="2" t="n">
+        <v>5500</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -6320,33 +6320,33 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="n">
+      <c r="A48" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Borderlands 2</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D48" s="4" t="n">
+      <c r="D48" s="2" t="n">
         <v>8551</v>
       </c>
-      <c r="E48" s="4" t="n">
+      <c r="E48" s="2" t="n">
         <v>92.40000000000001</v>
       </c>
-      <c r="F48" s="4" t="n">
+      <c r="F48" s="2" t="n">
         <v>295218</v>
       </c>
-      <c r="G48" s="4" t="n">
-        <v>5250</v>
-      </c>
-      <c r="H48" s="4" t="n">
-        <v>75</v>
+      <c r="G48" s="2" t="n">
+        <v>21000</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -6380,63 +6380,63 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="n">
+      <c r="A50" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Valheim</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Early Access</t>
         </is>
       </c>
-      <c r="D50" s="4" t="n">
+      <c r="D50" s="2" t="n">
         <v>14439</v>
       </c>
-      <c r="E50" s="4" t="n">
+      <c r="E50" s="2" t="n">
         <v>94.3</v>
       </c>
-      <c r="F50" s="4" t="n">
+      <c r="F50" s="2" t="n">
         <v>499828</v>
       </c>
-      <c r="G50" s="4" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H50" s="4" t="n">
-        <v>50</v>
+      <c r="G50" s="2" t="n">
+        <v>22000</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="n">
+      <c r="A51" t="n">
         <v>48</v>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Phasmophobia</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Action, Indie, Early Access</t>
         </is>
       </c>
-      <c r="D51" s="4" t="n">
+      <c r="D51" t="n">
         <v>9978</v>
       </c>
-      <c r="E51" s="4" t="n">
+      <c r="E51" t="n">
         <v>95.8</v>
       </c>
-      <c r="F51" s="4" t="n">
+      <c r="F51" t="n">
         <v>768779</v>
       </c>
-      <c r="G51" s="4" t="n">
-        <v>15050</v>
-      </c>
-      <c r="H51" s="4" t="n">
-        <v>30</v>
+      <c r="G51" t="n">
+        <v>21500</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -6530,63 +6530,63 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="n">
+      <c r="A55" t="n">
         <v>52</v>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>Half-Life</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D55" s="4" t="n">
+      <c r="D55" t="n">
         <v>634</v>
       </c>
-      <c r="E55" s="4" t="n">
+      <c r="E55" t="n">
         <v>96.5</v>
       </c>
-      <c r="F55" s="4" t="n">
+      <c r="F55" t="n">
         <v>148221</v>
       </c>
-      <c r="G55" s="4" t="n">
-        <v>2100</v>
-      </c>
-      <c r="H55" s="4" t="n">
-        <v>80</v>
+      <c r="G55" t="n">
+        <v>10500</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="n">
+      <c r="A56" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Monster Hunter: World</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D56" s="4" t="n">
+      <c r="D56" s="2" t="n">
         <v>11923</v>
       </c>
-      <c r="E56" s="4" t="n">
+      <c r="E56" s="2" t="n">
         <v>88</v>
       </c>
-      <c r="F56" s="4" t="n">
+      <c r="F56" s="2" t="n">
         <v>493390</v>
       </c>
-      <c r="G56" s="4" t="n">
-        <v>9570</v>
-      </c>
-      <c r="H56" s="4" t="n">
-        <v>74</v>
+      <c r="G56" s="2" t="n">
+        <v>36800</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -6650,33 +6650,33 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="n">
+      <c r="A59" t="n">
         <v>56</v>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>Project Zomboid</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>Indie, RPG, Simulation, Early Access</t>
         </is>
       </c>
-      <c r="D59" s="4" t="n">
+      <c r="D59" t="n">
         <v>22864</v>
       </c>
-      <c r="E59" s="4" t="n">
+      <c r="E59" t="n">
         <v>94.2</v>
       </c>
-      <c r="F59" s="4" t="n">
+      <c r="F59" t="n">
         <v>377063</v>
       </c>
-      <c r="G59" s="4" t="n">
-        <v>14400</v>
-      </c>
-      <c r="H59" s="4" t="n">
-        <v>33</v>
+      <c r="G59" t="n">
+        <v>21500</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -6740,33 +6740,33 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="n">
+      <c r="A62" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>Battlefield™ 2042</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Casual</t>
         </is>
       </c>
-      <c r="D62" s="4" t="n">
+      <c r="D62" s="2" t="n">
         <v>2774</v>
       </c>
-      <c r="E62" s="4" t="n">
+      <c r="E62" s="2" t="n">
         <v>46.7</v>
       </c>
-      <c r="F62" s="4" t="n">
+      <c r="F62" s="2" t="n">
         <v>297774</v>
       </c>
-      <c r="G62" s="4" t="n">
-        <v>3300</v>
-      </c>
-      <c r="H62" s="4" t="n">
-        <v>95</v>
+      <c r="G62" s="2" t="n">
+        <v>66000</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -6800,33 +6800,33 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="n">
+      <c r="A64" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="B64" s="4" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Raft</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D64" s="4" t="n">
+      <c r="D64" s="2" t="n">
         <v>4701</v>
       </c>
-      <c r="E64" s="4" t="n">
+      <c r="E64" s="2" t="n">
         <v>93.3</v>
       </c>
-      <c r="F64" s="4" t="n">
+      <c r="F64" s="2" t="n">
         <v>346359</v>
       </c>
-      <c r="G64" s="4" t="n">
-        <v>14070</v>
-      </c>
-      <c r="H64" s="4" t="n">
-        <v>33</v>
+      <c r="G64" s="2" t="n">
+        <v>21000</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -6890,93 +6890,93 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="4" t="n">
+      <c r="A67" t="n">
         <v>64</v>
       </c>
-      <c r="B67" s="4" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>Counter-Strike</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D67" s="4" t="n">
+      <c r="D67" t="n">
         <v>7323</v>
       </c>
-      <c r="E67" s="4" t="n">
+      <c r="E67" t="n">
         <v>97.40000000000001</v>
       </c>
-      <c r="F67" s="4" t="n">
+      <c r="F67" t="n">
         <v>250245</v>
       </c>
-      <c r="G67" s="4" t="n">
-        <v>2100</v>
-      </c>
-      <c r="H67" s="4" t="n">
-        <v>80</v>
+      <c r="G67" t="n">
+        <v>10500</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="n">
+      <c r="A68" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>Counter-Strike: Source</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D68" s="4" t="n">
+      <c r="D68" s="2" t="n">
         <v>6187</v>
       </c>
-      <c r="E68" s="4" t="n">
+      <c r="E68" s="2" t="n">
         <v>96.3</v>
       </c>
-      <c r="F68" s="4" t="n">
+      <c r="F68" s="2" t="n">
         <v>182234</v>
       </c>
-      <c r="G68" s="4" t="n">
-        <v>2200</v>
-      </c>
-      <c r="H68" s="4" t="n">
-        <v>80</v>
+      <c r="G68" s="2" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="4" t="n">
+      <c r="A69" t="n">
         <v>66</v>
       </c>
-      <c r="B69" s="4" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>Schedule I</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>Action, Indie, Simulation, Strategy, Early Access</t>
         </is>
       </c>
-      <c r="D69" s="4" t="n">
+      <c r="D69" t="n">
         <v>22757</v>
       </c>
-      <c r="E69" s="4" t="n">
+      <c r="E69" t="n">
         <v>98.40000000000001</v>
       </c>
-      <c r="F69" s="4" t="n">
+      <c r="F69" t="n">
         <v>204041</v>
       </c>
-      <c r="G69" s="4" t="n">
-        <v>12900</v>
-      </c>
-      <c r="H69" s="4" t="n">
-        <v>40</v>
+      <c r="G69" t="n">
+        <v>21500</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -7010,33 +7010,33 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="4" t="n">
+      <c r="A71" t="n">
         <v>68</v>
       </c>
-      <c r="B71" s="4" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D71" s="4" t="n">
+      <c r="D71" t="n">
         <v>638</v>
       </c>
-      <c r="E71" s="4" t="n">
+      <c r="E71" t="n">
         <v>98.5</v>
       </c>
-      <c r="F71" s="4" t="n">
+      <c r="F71" t="n">
         <v>177741</v>
       </c>
-      <c r="G71" s="4" t="n">
-        <v>2200</v>
-      </c>
-      <c r="H71" s="4" t="n">
-        <v>80</v>
+      <c r="G71" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -7100,153 +7100,153 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="4" t="n">
+      <c r="A74" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="B74" s="4" t="inlineStr">
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>Don't Starve Together</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D74" s="4" t="n">
+      <c r="D74" s="2" t="n">
         <v>30542</v>
       </c>
-      <c r="E74" s="4" t="n">
+      <c r="E74" s="2" t="n">
         <v>95.3</v>
       </c>
-      <c r="F74" s="4" t="n">
+      <c r="F74" s="2" t="n">
         <v>499061</v>
       </c>
-      <c r="G74" s="4" t="n">
-        <v>1550</v>
-      </c>
-      <c r="H74" s="4" t="n">
-        <v>90</v>
+      <c r="G74" s="2" t="n">
+        <v>15500</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="4" t="n">
+      <c r="A75" t="n">
         <v>72</v>
       </c>
-      <c r="B75" s="4" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>Dying Light</t>
         </is>
       </c>
-      <c r="C75" s="4" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>Action, Adventure, RPG</t>
         </is>
       </c>
-      <c r="D75" s="4" t="n">
+      <c r="D75" t="n">
         <v>4953</v>
       </c>
-      <c r="E75" s="4" t="n">
+      <c r="E75" t="n">
         <v>95.2</v>
       </c>
-      <c r="F75" s="4" t="n">
+      <c r="F75" t="n">
         <v>457632</v>
       </c>
-      <c r="G75" s="4" t="n">
-        <v>2740</v>
-      </c>
-      <c r="H75" s="4" t="n">
-        <v>90</v>
+      <c r="G75" t="n">
+        <v>27400</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="4" t="n">
+      <c r="A76" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="B76" s="4" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>Human Fall Flat</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>Adventure, Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D76" s="4" t="n">
+      <c r="D76" s="2" t="n">
         <v>950</v>
       </c>
-      <c r="E76" s="4" t="n">
+      <c r="E76" s="2" t="n">
         <v>94.7</v>
       </c>
-      <c r="F76" s="4" t="n">
+      <c r="F76" s="2" t="n">
         <v>213640</v>
       </c>
-      <c r="G76" s="4" t="n">
-        <v>6150</v>
-      </c>
-      <c r="H76" s="4" t="n">
-        <v>70</v>
+      <c r="G76" s="2" t="n">
+        <v>20500</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="4" t="n">
+      <c r="A77" t="n">
         <v>74</v>
       </c>
-      <c r="B77" s="4" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>7 Days to Die</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D77" s="4" t="n">
+      <c r="D77" t="n">
         <v>17045</v>
       </c>
-      <c r="E77" s="4" t="n">
+      <c r="E77" t="n">
         <v>88.59999999999999</v>
       </c>
-      <c r="F77" s="4" t="n">
+      <c r="F77" t="n">
         <v>370046</v>
       </c>
-      <c r="G77" s="4" t="n">
-        <v>25850</v>
-      </c>
-      <c r="H77" s="4" t="n">
-        <v>45</v>
+      <c r="G77" t="n">
+        <v>47000</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="4" t="n">
+      <c r="A78" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="B78" s="4" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>Counter-Strike: Condition Zero</t>
         </is>
       </c>
-      <c r="C78" s="4" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D78" s="4" t="n">
+      <c r="D78" s="2" t="n">
         <v>83</v>
       </c>
-      <c r="E78" s="4" t="n">
+      <c r="E78" s="2" t="n">
         <v>89.8</v>
       </c>
-      <c r="F78" s="4" t="n">
+      <c r="F78" s="2" t="n">
         <v>14977</v>
       </c>
-      <c r="G78" s="4" t="n">
-        <v>2100</v>
-      </c>
-      <c r="H78" s="4" t="n">
-        <v>80</v>
+      <c r="G78" s="2" t="n">
+        <v>10500</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -7340,183 +7340,183 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="4" t="n">
+      <c r="A82" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="B82" s="4" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>Hunt: Showdown 1896</t>
         </is>
       </c>
-      <c r="C82" s="4" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D82" s="4" t="n">
+      <c r="D82" s="2" t="n">
         <v>6300</v>
       </c>
-      <c r="E82" s="4" t="n">
+      <c r="E82" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="F82" s="4" t="n">
+      <c r="F82" s="2" t="n">
         <v>248220</v>
       </c>
-      <c r="G82" s="4" t="n">
-        <v>14680</v>
-      </c>
-      <c r="H82" s="4" t="n">
-        <v>60</v>
+      <c r="G82" s="2" t="n">
+        <v>36700</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="4" t="n">
+      <c r="A83" t="n">
         <v>80</v>
       </c>
-      <c r="B83" s="4" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>Sekiro™: Shadows Die Twice - GOTY Edition</t>
         </is>
       </c>
-      <c r="C83" s="4" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>Action, Adventure</t>
         </is>
       </c>
-      <c r="D83" s="4" t="n">
+      <c r="D83" t="n">
         <v>6767</v>
       </c>
-      <c r="E83" s="4" t="n">
+      <c r="E83" t="n">
         <v>95.3</v>
       </c>
-      <c r="F83" s="4" t="n">
+      <c r="F83" t="n">
         <v>322234</v>
       </c>
-      <c r="G83" s="4" t="n">
-        <v>37500</v>
-      </c>
-      <c r="H83" s="4" t="n">
-        <v>50</v>
+      <c r="G83" t="n">
+        <v>75000</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="n">
+      <c r="A84" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="B84" s="4" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>CyberCorp</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D84" s="4" t="n">
+      <c r="D84" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E84" s="4" t="n">
+      <c r="E84" s="2" t="n">
         <v>82.59999999999999</v>
       </c>
-      <c r="F84" s="4" t="n">
+      <c r="F84" s="2" t="n">
         <v>322</v>
       </c>
-      <c r="G84" s="4" t="n">
-        <v>9900</v>
-      </c>
-      <c r="H84" s="4" t="n">
-        <v>40</v>
+      <c r="G84" s="2" t="n">
+        <v>16500</v>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="4" t="n">
+      <c r="A85" t="n">
         <v>82</v>
       </c>
-      <c r="B85" s="4" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>Half-Life 2</t>
         </is>
       </c>
-      <c r="C85" s="4" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D85" s="4" t="n">
+      <c r="D85" t="n">
         <v>1555</v>
       </c>
-      <c r="E85" s="4" t="n">
+      <c r="E85" t="n">
         <v>97.59999999999999</v>
       </c>
-      <c r="F85" s="4" t="n">
+      <c r="F85" t="n">
         <v>245627</v>
       </c>
-      <c r="G85" s="4" t="n">
-        <v>2200</v>
-      </c>
-      <c r="H85" s="4" t="n">
-        <v>80</v>
+      <c r="G85" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="4" t="n">
+      <c r="A86" s="2" t="n">
         <v>83</v>
       </c>
-      <c r="B86" s="4" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>Arma 3</t>
         </is>
       </c>
-      <c r="C86" s="4" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>Action, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D86" s="4" t="n">
+      <c r="D86" s="2" t="n">
         <v>7181</v>
       </c>
-      <c r="E86" s="4" t="n">
+      <c r="E86" s="2" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="F86" s="4" t="n">
+      <c r="F86" s="2" t="n">
         <v>283264</v>
       </c>
-      <c r="G86" s="4" t="n">
-        <v>10800</v>
-      </c>
-      <c r="H86" s="4" t="n">
-        <v>70</v>
+      <c r="G86" s="2" t="n">
+        <v>36000</v>
+      </c>
+      <c r="H86" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="4" t="n">
+      <c r="A87" t="n">
         <v>84</v>
       </c>
-      <c r="B87" s="4" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>Sons Of The Forest</t>
         </is>
       </c>
-      <c r="C87" s="4" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="D87" s="4" t="n">
+      <c r="D87" t="n">
         <v>4450</v>
       </c>
-      <c r="E87" s="4" t="n">
+      <c r="E87" t="n">
         <v>87.8</v>
       </c>
-      <c r="F87" s="4" t="n">
+      <c r="F87" t="n">
         <v>253546</v>
       </c>
-      <c r="G87" s="4" t="n">
-        <v>9600</v>
-      </c>
-      <c r="H87" s="4" t="n">
-        <v>70</v>
+      <c r="G87" t="n">
+        <v>32000</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -7543,100 +7543,100 @@
         <v>99730</v>
       </c>
       <c r="G88" s="4" t="n">
-        <v>2700</v>
+        <v>5400</v>
       </c>
       <c r="H88" s="4" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="4" t="n">
+      <c r="A89" t="n">
         <v>86</v>
       </c>
-      <c r="B89" s="4" t="inlineStr">
+      <c r="B89" t="inlineStr">
         <is>
           <t>Cities: Skylines</t>
         </is>
       </c>
-      <c r="C89" s="4" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D89" s="4" t="n">
+      <c r="D89" t="n">
         <v>8842</v>
       </c>
-      <c r="E89" s="4" t="n">
+      <c r="E89" t="n">
         <v>93</v>
       </c>
-      <c r="F89" s="4" t="n">
+      <c r="F89" t="n">
         <v>275770</v>
       </c>
-      <c r="G89" s="4" t="n">
-        <v>9900</v>
-      </c>
-      <c r="H89" s="4" t="n">
-        <v>70</v>
+      <c r="G89" t="n">
+        <v>33000</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="4" t="n">
+      <c r="A90" s="2" t="n">
         <v>87</v>
       </c>
-      <c r="B90" s="4" t="inlineStr">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>Mount &amp; Blade II: Bannerlord</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>Action, Indie, RPG, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D90" s="4" t="n">
+      <c r="D90" s="2" t="n">
         <v>14477</v>
       </c>
-      <c r="E90" s="4" t="n">
+      <c r="E90" s="2" t="n">
         <v>87.90000000000001</v>
       </c>
-      <c r="F90" s="4" t="n">
+      <c r="F90" s="2" t="n">
         <v>264391</v>
       </c>
-      <c r="G90" s="4" t="n">
-        <v>24000</v>
-      </c>
-      <c r="H90" s="4" t="n">
-        <v>60</v>
+      <c r="G90" s="2" t="n">
+        <v>60000</v>
+      </c>
+      <c r="H90" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="4" t="n">
+      <c r="A91" t="n">
         <v>88</v>
       </c>
-      <c r="B91" s="4" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>Sid Meier's Civilization® V</t>
         </is>
       </c>
-      <c r="C91" s="4" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="D91" s="4" t="n">
+      <c r="D91" t="n">
         <v>12206</v>
       </c>
-      <c r="E91" s="4" t="n">
+      <c r="E91" t="n">
         <v>95.8</v>
       </c>
-      <c r="F91" s="4" t="n">
+      <c r="F91" t="n">
         <v>204265</v>
       </c>
-      <c r="G91" s="4" t="n">
-        <v>8000</v>
-      </c>
-      <c r="H91" s="4" t="n">
-        <v>75</v>
+      <c r="G91" t="n">
+        <v>32000</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -7670,63 +7670,63 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="4" t="n">
+      <c r="A93" t="n">
         <v>90</v>
       </c>
-      <c r="B93" s="4" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>Sid Meier’s Civilization® VI</t>
         </is>
       </c>
-      <c r="C93" s="4" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="D93" s="4" t="n">
+      <c r="D93" t="n">
         <v>25420</v>
       </c>
-      <c r="E93" s="4" t="n">
+      <c r="E93" t="n">
         <v>86.90000000000001</v>
       </c>
-      <c r="F93" s="4" t="n">
+      <c r="F93" t="n">
         <v>349920</v>
       </c>
-      <c r="G93" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="H93" s="4" t="n">
-        <v>90</v>
+      <c r="G93" t="n">
+        <v>65000</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="4" t="n">
+      <c r="A94" s="2" t="n">
         <v>91</v>
       </c>
-      <c r="B94" s="4" t="inlineStr">
+      <c r="B94" s="2" t="inlineStr">
         <is>
           <t>Fallout 4</t>
         </is>
       </c>
-      <c r="C94" s="4" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>RPG</t>
         </is>
       </c>
-      <c r="D94" s="4" t="n">
+      <c r="D94" s="2" t="n">
         <v>11179</v>
       </c>
-      <c r="E94" s="4" t="n">
+      <c r="E94" s="2" t="n">
         <v>83.09999999999999</v>
       </c>
-      <c r="F94" s="4" t="n">
+      <c r="F94" s="2" t="n">
         <v>392287</v>
       </c>
-      <c r="G94" s="4" t="n">
-        <v>8800</v>
-      </c>
-      <c r="H94" s="4" t="n">
-        <v>60</v>
+      <c r="G94" s="2" t="n">
+        <v>22000</v>
+      </c>
+      <c r="H94" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -7790,123 +7790,123 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="4" t="n">
+      <c r="A97" t="n">
         <v>94</v>
       </c>
-      <c r="B97" s="4" t="inlineStr">
+      <c r="B97" t="inlineStr">
         <is>
           <t>Battlefield™ V</t>
         </is>
       </c>
-      <c r="C97" s="4" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D97" s="4" t="n">
+      <c r="D97" t="n">
         <v>6327</v>
       </c>
-      <c r="E97" s="4" t="n">
+      <c r="E97" t="n">
         <v>70.90000000000001</v>
       </c>
-      <c r="F97" s="4" t="n">
+      <c r="F97" t="n">
         <v>250288</v>
       </c>
-      <c r="G97" s="4" t="n">
-        <v>2750</v>
-      </c>
-      <c r="H97" s="4" t="n">
+      <c r="G97" t="n">
+        <v>55000</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
         <v>95</v>
       </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="4" t="n">
-        <v>95</v>
-      </c>
-      <c r="B98" s="4" t="inlineStr">
+      <c r="B98" s="2" t="inlineStr">
         <is>
           <t>R.E.P.O.</t>
         </is>
       </c>
-      <c r="C98" s="4" t="inlineStr">
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>Action, Early Access</t>
         </is>
       </c>
-      <c r="D98" s="4" t="n">
+      <c r="D98" s="2" t="n">
         <v>32349</v>
       </c>
-      <c r="E98" s="4" t="n">
+      <c r="E98" s="2" t="n">
         <v>96.5</v>
       </c>
-      <c r="F98" s="4" t="n">
+      <c r="F98" s="2" t="n">
         <v>185642</v>
       </c>
-      <c r="G98" s="4" t="n">
-        <v>6950</v>
-      </c>
-      <c r="H98" s="4" t="n">
-        <v>35</v>
+      <c r="G98" s="2" t="n">
+        <v>10700</v>
+      </c>
+      <c r="H98" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="4" t="n">
+      <c r="A99" t="n">
         <v>96</v>
       </c>
-      <c r="B99" s="4" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>DayZ</t>
         </is>
       </c>
-      <c r="C99" s="4" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>Action, Adventure, Massively Multiplayer</t>
         </is>
       </c>
-      <c r="D99" s="4" t="n">
+      <c r="D99" t="n">
         <v>37066</v>
       </c>
-      <c r="E99" s="4" t="n">
+      <c r="E99" t="n">
         <v>76.8</v>
       </c>
-      <c r="F99" s="4" t="n">
+      <c r="F99" t="n">
         <v>430252</v>
       </c>
-      <c r="G99" s="4" t="n">
-        <v>29500</v>
-      </c>
-      <c r="H99" s="4" t="n">
-        <v>50</v>
+      <c r="G99" t="n">
+        <v>59000</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="4" t="n">
+      <c r="A100" s="2" t="n">
         <v>97</v>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B100" s="2" t="inlineStr">
         <is>
           <t>Satisfactory</t>
         </is>
       </c>
-      <c r="C100" s="4" t="inlineStr">
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>Adventure, Indie, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D100" s="4" t="n">
+      <c r="D100" s="2" t="n">
         <v>12596</v>
       </c>
-      <c r="E100" s="4" t="n">
+      <c r="E100" s="2" t="n">
         <v>97.2</v>
       </c>
-      <c r="F100" s="4" t="n">
+      <c r="F100" s="2" t="n">
         <v>232064</v>
       </c>
-      <c r="G100" s="4" t="n">
-        <v>29400</v>
-      </c>
-      <c r="H100" s="4" t="n">
-        <v>30</v>
+      <c r="G100" s="2" t="n">
+        <v>42000</v>
+      </c>
+      <c r="H100" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -7940,33 +7940,33 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="4" t="n">
+      <c r="A102" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="B102" s="4" t="inlineStr">
+      <c r="B102" s="2" t="inlineStr">
         <is>
           <t>Risk of Rain 2</t>
         </is>
       </c>
-      <c r="C102" s="4" t="inlineStr">
+      <c r="C102" s="2" t="inlineStr">
         <is>
           <t>Action, Indie</t>
         </is>
       </c>
-      <c r="D102" s="4" t="n">
+      <c r="D102" s="2" t="n">
         <v>7902</v>
       </c>
-      <c r="E102" s="4" t="n">
+      <c r="E102" s="2" t="n">
         <v>93.5</v>
       </c>
-      <c r="F102" s="4" t="n">
+      <c r="F102" s="2" t="n">
         <v>313577</v>
       </c>
-      <c r="G102" s="4" t="n">
-        <v>8580</v>
-      </c>
-      <c r="H102" s="4" t="n">
-        <v>67</v>
+      <c r="G102" s="2" t="n">
+        <v>26000</v>
+      </c>
+      <c r="H102" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-09</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-10</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-09</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-10</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-09</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-11
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -689,7 +689,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Action, Adventure, Indie, RPG, Early Access</t>
+          <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-10</t>
+          <t>Steam 인기 차트 — 2026-07-11</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Action, Adventure, Indie, RPG, Early Access</t>
+          <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-10</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-11</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-10</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-11</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-10</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-12
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3911,10 +3911,10 @@
         <v>941</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>2200</v>
+        <v>1100</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>2200</v>
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-11</t>
+          <t>Steam 인기 차트 — 2026-07-12</t>
         </is>
       </c>
     </row>
@@ -7280,33 +7280,33 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="4" t="n">
         <v>77</v>
       </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="B80" s="4" t="inlineStr">
         <is>
           <t>Street Warriors Online</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C80" s="4" t="inlineStr">
         <is>
           <t>Action, Massively Multiplayer, Simulation, Sports</t>
         </is>
       </c>
-      <c r="D80" s="2" t="n">
+      <c r="D80" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E80" s="2" t="n">
+      <c r="E80" s="4" t="n">
         <v>57.6</v>
       </c>
-      <c r="F80" s="2" t="n">
+      <c r="F80" s="4" t="n">
         <v>1634</v>
       </c>
-      <c r="G80" s="2" t="n">
-        <v>2200</v>
-      </c>
-      <c r="H80" s="2" t="n">
-        <v>0</v>
+      <c r="G80" s="4" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H80" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="81">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-11</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-12</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-11</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-12</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-11</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-13
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1975,10 +1975,10 @@
         <v>594327</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>10700</v>
+        <v>5350</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>10700</v>
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2591,10 +2591,10 @@
         <v>471451</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>22000</v>
+        <v>11000</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>22000</v>
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4791,10 +4791,10 @@
         <v>225479</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>42000</v>
+        <v>29400</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>42000</v>
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-12</t>
+          <t>Steam 인기 차트 — 2026-07-13</t>
         </is>
       </c>
     </row>
@@ -5960,33 +5960,33 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>PAYDAY 2</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Action, RPG</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D36" s="4" t="n">
         <v>27254</v>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E36" s="4" t="n">
         <v>89.59999999999999</v>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="F36" s="4" t="n">
         <v>663082</v>
       </c>
-      <c r="G36" s="2" t="n">
-        <v>10700</v>
-      </c>
-      <c r="H36" s="2" t="n">
-        <v>0</v>
+      <c r="G36" s="4" t="n">
+        <v>5350</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="37">
@@ -6380,33 +6380,33 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>Valheim</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Early Access</t>
         </is>
       </c>
-      <c r="D50" s="2" t="n">
+      <c r="D50" s="4" t="n">
         <v>14439</v>
       </c>
-      <c r="E50" s="2" t="n">
+      <c r="E50" s="4" t="n">
         <v>94.3</v>
       </c>
-      <c r="F50" s="2" t="n">
+      <c r="F50" s="4" t="n">
         <v>499828</v>
       </c>
-      <c r="G50" s="2" t="n">
-        <v>22000</v>
-      </c>
-      <c r="H50" s="2" t="n">
-        <v>0</v>
+      <c r="G50" s="4" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H50" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="51">
@@ -7880,33 +7880,33 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="4" t="n">
         <v>97</v>
       </c>
-      <c r="B100" s="2" t="inlineStr">
+      <c r="B100" s="4" t="inlineStr">
         <is>
           <t>Satisfactory</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
+      <c r="C100" s="4" t="inlineStr">
         <is>
           <t>Adventure, Indie, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="D100" s="2" t="n">
+      <c r="D100" s="4" t="n">
         <v>12596</v>
       </c>
-      <c r="E100" s="2" t="n">
+      <c r="E100" s="4" t="n">
         <v>97.2</v>
       </c>
-      <c r="F100" s="2" t="n">
+      <c r="F100" s="4" t="n">
         <v>232064</v>
       </c>
-      <c r="G100" s="2" t="n">
-        <v>42000</v>
-      </c>
-      <c r="H100" s="2" t="n">
-        <v>0</v>
+      <c r="G100" s="4" t="n">
+        <v>29400</v>
+      </c>
+      <c r="H100" s="4" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="101">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-12</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-13</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-12</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-13</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-12</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-14
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2415,10 +2415,10 @@
         <v>643681</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>5500</v>
+        <v>3300</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>5500</v>
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4615,10 +4615,10 @@
         <v>26360</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>21200</v>
+        <v>53000</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>53000</v>
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-13</t>
+          <t>Steam 인기 차트 — 2026-07-14</t>
         </is>
       </c>
     </row>
@@ -6260,33 +6260,33 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Among Us</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Casual</t>
         </is>
       </c>
-      <c r="D46" s="2" t="n">
+      <c r="D46" s="4" t="n">
         <v>3832</v>
       </c>
-      <c r="E46" s="2" t="n">
+      <c r="E46" s="4" t="n">
         <v>91.90000000000001</v>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="F46" s="4" t="n">
         <v>700785</v>
       </c>
-      <c r="G46" s="2" t="n">
-        <v>5500</v>
-      </c>
-      <c r="H46" s="2" t="n">
-        <v>0</v>
+      <c r="G46" s="4" t="n">
+        <v>3300</v>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="47">
@@ -7760,33 +7760,33 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="n">
+      <c r="A96" s="2" t="n">
         <v>93</v>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>Warhammer 40,000: Rogue Trader</t>
         </is>
       </c>
-      <c r="C96" s="4" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG, Strategy</t>
         </is>
       </c>
-      <c r="D96" s="4" t="n">
+      <c r="D96" s="2" t="n">
         <v>3582</v>
       </c>
-      <c r="E96" s="4" t="n">
+      <c r="E96" s="2" t="n">
         <v>85.59999999999999</v>
       </c>
-      <c r="F96" s="4" t="n">
+      <c r="F96" s="2" t="n">
         <v>30805</v>
       </c>
-      <c r="G96" s="4" t="n">
-        <v>21200</v>
-      </c>
-      <c r="H96" s="4" t="n">
-        <v>60</v>
+      <c r="G96" s="2" t="n">
+        <v>53000</v>
+      </c>
+      <c r="H96" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-13</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-14</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-13</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-14</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-13</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-15
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3911,10 +3911,10 @@
         <v>941</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>1100</v>
+        <v>2200</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>2200</v>
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-14</t>
+          <t>Steam 인기 차트 — 2026-07-15</t>
         </is>
       </c>
     </row>
@@ -7280,33 +7280,33 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="4" t="n">
+      <c r="A80" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="B80" s="4" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>Street Warriors Online</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>Action, Massively Multiplayer, Simulation, Sports</t>
         </is>
       </c>
-      <c r="D80" s="4" t="n">
+      <c r="D80" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E80" s="4" t="n">
+      <c r="E80" s="2" t="n">
         <v>57.6</v>
       </c>
-      <c r="F80" s="4" t="n">
+      <c r="F80" s="2" t="n">
         <v>1634</v>
       </c>
-      <c r="G80" s="4" t="n">
-        <v>1100</v>
-      </c>
-      <c r="H80" s="4" t="n">
-        <v>50</v>
+      <c r="G80" s="2" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-14</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-15</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-14</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-15</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-14</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-16
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-15</t>
+          <t>Steam 인기 차트 — 2026-07-16</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-15</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-16</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-15</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-16</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-15</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-17
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2635,10 +2635,10 @@
         <v>736611</v>
       </c>
       <c r="J49" t="n">
-        <v>21500</v>
+        <v>15050</v>
       </c>
       <c r="K49" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L49" t="n">
         <v>21500</v>
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4263,10 +4263,10 @@
         <v>93489</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>5400</v>
+        <v>27000</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>27000</v>
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-16</t>
+          <t>Steam 인기 차트 — 2026-07-17</t>
         </is>
       </c>
     </row>
@@ -6410,33 +6410,33 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>Phasmophobia</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Action, Indie, Early Access</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D51" s="4" t="n">
         <v>9978</v>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="4" t="n">
         <v>95.8</v>
       </c>
-      <c r="F51" t="n">
+      <c r="F51" s="4" t="n">
         <v>768779</v>
       </c>
-      <c r="G51" t="n">
-        <v>21500</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0</v>
+      <c r="G51" s="4" t="n">
+        <v>15050</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="52">
@@ -7520,33 +7520,33 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="4" t="n">
+      <c r="A88" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="B88" s="4" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>Grim Dawn</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, RPG</t>
         </is>
       </c>
-      <c r="D88" s="4" t="n">
+      <c r="D88" s="2" t="n">
         <v>2376</v>
       </c>
-      <c r="E88" s="4" t="n">
+      <c r="E88" s="2" t="n">
         <v>93.7</v>
       </c>
-      <c r="F88" s="4" t="n">
+      <c r="F88" s="2" t="n">
         <v>99730</v>
       </c>
-      <c r="G88" s="4" t="n">
-        <v>5400</v>
-      </c>
-      <c r="H88" s="4" t="n">
-        <v>80</v>
+      <c r="G88" s="2" t="n">
+        <v>27000</v>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="89">
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-16</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-17</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-16</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-17</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-16</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-18
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3351,7 +3351,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -3395,7 +3395,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3439,7 +3439,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3483,7 +3483,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3527,7 +3527,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3571,7 +3571,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3615,7 +3615,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3659,7 +3659,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3703,7 +3703,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3747,7 +3747,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3791,7 +3791,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3835,7 +3835,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3879,7 +3879,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3923,7 +3923,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3967,7 +3967,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -4011,7 +4011,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -4055,7 +4055,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -4099,7 +4099,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -4143,7 +4143,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -4187,7 +4187,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -4231,7 +4231,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -4275,7 +4275,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -4319,7 +4319,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -4363,7 +4363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -4407,7 +4407,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -4451,7 +4451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4495,7 +4495,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -4539,7 +4539,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4583,7 +4583,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -4627,7 +4627,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4671,7 +4671,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -4715,7 +4715,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4759,7 +4759,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -4803,7 +4803,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4847,7 +4847,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -4891,7 +4891,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4959,7 +4959,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-07-17</t>
+          <t>Steam 인기 차트 — 2026-07-18</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-17</t>
+          <t>1주(7일)+ 상위 100위 유지 게임 — 기준일: 2026-07-18</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-17</t>
+          <t>2주(14일)+ 상위 100위 유지 게임 — 기준일: 2026-07-18</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-17</t>
+          <t>4주(28일)+ 상위 100위 유지 게임 — 기준일: 2026-07-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-07-19
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -629,7 +629,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -673,7 +673,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -761,7 +761,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -849,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -893,7 +893,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -937,7 +937,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -981,7 +981,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1025,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1067,7 +1067,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1155,7 +1155,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1199,7 +1199,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1243,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1287,7 +1287,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1331,7 +1331,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1417,7 +1417,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1461,7 +1461,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1505,7 +1505,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1549,7 +1549,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1593,7 +1593,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1637,7 +1637,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1681,7 +1681,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1725,7 +1725,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1813,7 +1813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1857,7 +1857,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1901,7 +1901,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1943,7 +1943,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1987,7 +1987,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2031,7 +2031,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2075,7 +2075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2119,7 +2119,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2163,7 +2163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2207,7 +2207,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2251,7 +2251,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2295,7 +2295,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2339,7 +2339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2383,7 +2383,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2427,7 +2427,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2471,7 +2471,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2515,7 +2515,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2559,7 +2559,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2603,7 +2603,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2647,7 +2647,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2691,7 +2691,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2735,7 +2735,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2823,7 +2823,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2867,7 +2867,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2911,7 +2911,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2955,7 +2955,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2999,7 +2999,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -3043,7 +3043,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3087,7 +3087,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -3131,7 +3131,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3175,7 +3175,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -3219,7 +3219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3263,7 +3263,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3307,7 +3307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B65" t="n